<commit_message>
feat: Add .gitignore, remove .env, and update `main.ipynb` with new example input data.
</commit_message>
<xml_diff>
--- a/Thư mục KQ/VB sau tóm tắt/test_results.xlsx
+++ b/Thư mục KQ/VB sau tóm tắt/test_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,88 +453,213 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Taste Studio của Regent Hotels &amp; Resorts tổ chức với chủ đề 'Dáng hình của biển', giới hạn 20 khách mời mỗi tối. Sự kiện quy tụ nhiều đầu bếp và nghệ sĩ nổi tiếng, từ Mr. Dripping (drip art) đến Francesco (Milan), Huân Trần (Regent Phú Quốc) và Andy Huỳnh (Oku). Regent Phú Quốc mong muốn tiếp tục kiến tạo trải nghiệm đưa nét bản địa đặc sắc lên bản đồ thế giới cho khách hàng hạng sang.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>{
+  "id": 1,
+  "style": "news_brief",
+  "article": "Taste Studio do thương hiệu Regent Hotels &amp; Resorts tổ chức nhằm mang đến trải nghiệm đa giác quan qua ẩm thực và nghệ thuật. Sự kiện này quy tụ nhiều đầu bếp và nghệ sĩ nổi tiếng, từ nhà thiết kế thời trang đến nhạc sĩ, kết hợp cùng các thương hiệu hàng đầu như Vietnam Airlines. Sự kiện hướng đến phân khúc khách hàng sang trọng. Mùa một và hai diễn ra lần được vào tháng 4, tháng 11 năm ngoái. Taste Studio năm nay với chủ đề 'Dáng hình của biển', giới hạn 20 khách mời mỗi tối. Các khách mời được tham gia vào chuỗi khám phá gồm 7 chương đặc sắc về vẻ đẹp của biển, qua lăng kính nghệ sĩ tài hoa Mr. Dripping - nghệ sĩ vẽ tranh bằng phương pháp nhỏ giọt (drip art). Không gian nhà hàng, nơi diễn ra sự kiện với nội thất dùng tre, mây và tầm vông do kiến trúc sư Nguyễn Trung Nghĩa thiết kế. Ngoài hai nghệ sĩ này, Taste Studio còn có sự tham gia của bếp trưởng Francesco đến từ Milan, với 20 năm kinh nghiệm làm việc tại các khách sạn danh tiếng thế giới, đang bắt đầu hành trình mới tại Việt Nam. Ông đảm nhận vai trò cố vấn ẩm thực tại Regent Phú Quốc, mang đến trải nghiệm độc đáo cho thực khách. Bên cạnh đó, phó bếp trưởng điều hành Huân Trần tại chương trình mong muốn chinh phục các hương vị vùng miền khác nhau. Được nếm nhiều nguyên liệu địa phương và các loại gia vị đặc biệt, vị đầu bếp để lại điểm nhấn riêng trong cách giữ gìn, nâng tầm phong vị của quê hương tại Regent Phú Quốc. Chương trình có sự góp mặt của bếp trưởng nhà hàng Oku - Andy Huỳnh. Trước khi gia nhập Regent Phú Quốc, anh phát triển kỹ thuật nấu ăn Nhật Bản tại Nobu, San Diego và Nassau. Các món ăn của Andy luôn mang ý nghĩa hướng về cội nguồn. Bếp trưởng nhà hàng Ocean Club Daniel và bếp trưởng Duyến Nguyễn của khu nghỉ dưỡng này cũng tham gia, sáng tạo một số hương vị độc đáo từ nguyên liệu địa phương. Đại diện Regent Phú Quốc cho biết, thông qua Taste Studio, đơn vị mong muốn tiếp tục kiến tạo trải nghiệm đưa nét bản địa đặc sắc của Việt Nam lên bản đồ thế giới, từ đó chinh phục khách hàng hạng sang và giới chuyên gia. Thanh Thư",
+  "summary": "Taste Studio của Regent Hotels &amp; Resorts tổ chức với chủ đề 'Dáng hình của biển', giới hạn 20 khách mời mỗi tối. Sự kiện quy tụ nhiều đầu bếp và nghệ sĩ nổi tiếng, từ Mr. Dripping (drip art) đến Francesco (Milan), Huân Trần (Regent Phú Quốc) và Andy Huỳnh (Oku). Regent Phú Quốc mong muốn tiếp tục kiến tạo trải nghiệm đưa nét bản địa đặc sắc lên bản đồ thế giới cho khách hàng hạng sang.",
+  "faithfulness_score": 0.9,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, nhưng có bỏ sót một số chi tiết quan trọng như sự tham gia của các thương hiệu hàng đầu và kiến trúc sư Nguyễn Trung Nghĩa",
+  "relevance_score": 0.8,
+  "relevance_reason": "Bản tóm tắt bao hàm các ý chính quan trọng, nhưng bỏ sót thông điệp về việc Regent Phú Quốc muốn chinh phục khách hàng hạng sang và giới chuyên gia",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, nhưng có thể rút gọn một số chi tiết để tăng tính súc tích"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hai giải thưởng gồm 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới'. Đây cũng là năm thứ tư liên tiếp đơn vị đạt giải thưởng này, sau quá trình thẩm định từ hội đồng chuyên môn toàn cầu và bình chọn bởi hàng nghìn du khách, khách sạn quốc tế khác. 'Giải thưởng góp phần khẳng định Amiana Resort Nha Trang là điểm đến lý tưởng cho du khách tìm kiếm không gian riêng tư, gần gũi thiên nhiên với kiến trúc cao cấp, mang lại trải nghiệm sang trọng, độc đáo', đại diện resort chia sẻ. Amiana có kiến trúc hòa hợp thiên nhiên, kết hợp yếu tố truyền thống và hiện đại, tạo nên không gian thư giãn, sang trọng nhưng vẫn giữ được cảm giác gần gũi, yên bình. Bãi biển riêng tư với hàng dừa rợp bóng xanh mát là nơi du khách có thể thư giãn, nghỉ ngơi thoải mái. Resort còn tận dụng địa hình tự nhiên để bố trí các công trình công cộng như hồ bơi, nhà hàng, phòng hội nghị, spa... Các yếu tố đậm chất nhiệt đới như dừa xanh, sóng biển, đá và gỗ được lồng ghép khéo léo trong từng chi tiết thiết kế nội ngoại thất. Biệt thự, phòng nghỉ, nhà hàng đều có sự kết hợp giữa vật liệu tự nhiên và công nghệ hiện đại. Mỗi căn biệt thự đều mang kiến trúc mở, sử dụng nội thất chủ yếu từ gỗ, đá tự nhiên. Tất cả phòng đều có cửa sổ lớn và ban công rộng, tối ưu tầm nhìn hướng biển với cảnh quan thiên nhiên vây quanh. Biệt thự còn có hồ bơi riêng, không gian vườn với các loại cây nhiệt đới, đảm bảo yếu tố riêng tư cho khách hàng. Resort không chỉ chú trọng xây dựng công trình tiện ích, mà còn đặc biệt lưu ý việc bảo vệ môi trường, sử dụng các giải pháp bền vững. Những không gian xanh, vườn cây, hồ nước đều được bố trí hợp lý, tạo nên hệ sinh thái tự nhiên trong lòng khu nghỉ dưỡng. Theo đại diện Amiana Resort Nha Trang, những chi tiết kiến trúc thông minh cùng không gian mở, vật liệu tự nhiên, sự khéo léo trong thiết kế tại đây góp phần tạo nên khu nghỉ dưỡng lý tưởng cho những ai tìm kiếm sự an yên, lãng mạn và xa hoa. Á Hiên</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Amiana Resort Nha Trang tiếp tục nhận hai giải thưởng quốc tế: 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới', nổi bật với kiến trúc tự nhiên kết hợp công nghệ, bãi biển riêng tư xanh mát, hồ bơi và vườn bảo vệ môi trường.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>{
+  "id": 2,
+  "style": "news_brief",
+  "article": "Hai giải thưởng gồm 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới'. Đây cũng là năm thứ tư liên tiếp đơn vị đạt giải thưởng này, sau quá trình thẩm định từ hội đồng chuyên môn toàn cầu và bình chọn bởi hàng nghìn du khách, khách sạn quốc tế khác. 'Giải thưởng góp phần khẳng định Amiana Resort Nha Trang là điểm đến lý tưởng cho du khách tìm kiếm không gian riêng tư, gần gũi thiên nhiên với kiến trúc cao cấp, mang lại trải nghiệm sang trọng, độc đáo', đại diện resort chia sẻ. Amiana có kiến trúc hòa hợp thiên nhiên, kết hợp yếu tố truyền thống và hiện đại, tạo nên không gian thư giãn, sang trọng nhưng vẫn giữ được cảm giác gần gũi, yên bình. Bãi biển riêng tư với hàng dừa rợp bóng xanh mát là nơi du khách có thể thư giãn, nghỉ ngơi thoải mái. Resort còn tận dụng địa hình tự nhiên để bố trí các công trình công cộng như hồ bơi, nhà hàng, phòng hội nghị, spa... Các yếu tố đậm chất nhiệt đới như dừa xanh, sóng biển, đá và gỗ được lồng ghép khéo léo trong từng chi tiết thiết kế nội ngoại thất. Biệt thự, phòng nghỉ, nhà hàng đều có sự kết hợp giữa vật liệu tự nhiên và công nghệ hiện đại. Mỗi căn biệt thự đều mang kiến trúc mở, sử dụng nội thất chủ yếu từ gỗ, đá tự nhiên. Tất cả phòng đều có cửa sổ lớn và ban công rộng, tối ưu tầm nhìn hướng biển với cảnh quan thiên nhiên vây quanh. Biệt thự còn có hồ bơi riêng, không gian vườn với các loại cây nhiệt đới, đảm bảo yếu tố riêng tư cho khách hàng. Resort không chỉ chú trọng xây dựng công trình tiện ích, mà còn đặc biệt lưu ý việc bảo vệ môi trường, sử dụng các giải pháp bền vững. Những không gian xanh, vườn cây, hồ nước đều được bố trí hợp lý, tạo nên hệ sinh thái tự nhiên trong lòng khu nghỉ dưỡng. Theo đại diện Amiana Resort Nha Trang, những chi tiết kiến trúc thông minh cùng không gian mở, vật liệu tự nhiên, sự khéo léo trong thiết kế tại đây góp phần tạo nên khu nghỉ dưỡng lý tưởng cho những ai tìm kiếm sự an yên, lãng mạn và xa hoa. Á Hiên",
+  "summary": "Amiana Resort Nha Trang tiếp tục nhận hai giải thưởng quốc tế: 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới', nổi bật với kiến trúc tự nhiên kết hợp công nghệ, bãi biển riêng tư xanh mát, hồ bơi và vườn bảo vệ môi trường.",
+  "faithfulness_score": 0.9,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, nhưng có thể thiếu một số chi tiết quan trọng như việc Amiana Resort Nha Trang đạt giải thưởng này lần thứ tư liên tiếp và quá trình thẩm định từ hội đồng chuyên môn toàn cầu",
+  "relevance_score": 0.8,
+  "relevance_reason": "Bản tóm tắt bao hàm các ý chính quan trọng như giải thưởng, kiến trúc và môi trường, nhưng có thể bỏ sót thông điệp cốt lõi về sự kết hợp giữa vật liệu tự nhiên và công nghệ hiện đại",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, nhưng có thể loại bỏ một số từ ngữ không cần thiết để tăng tính súc tích"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cồn Én nằm giữa sông Tiền, thuộc xã Tấn Mỹ, rộng hơn 300 ha. Nơi đây ngoài là điểm đến ngắm dòng Tiền Giang, đón gió sông mát dịu, còn là địa chỉ thu hút khách với bộ sưu tập gỗ lũa nội thất độc đáo của khu du lịch trên cồn. Gỗ lũa tức những thân cây khủng, vớt từ đáy sông, bên ngoài bị dòng nước bào mòn, chỉ còn phần lõi bền chắc. Hàng nghìn thân gỗ lũa được người chủ tuyển chọn làm vật liệu chính xây Khu du lịch sinh thái Cồn Én từ tiểu cảnh, nhà đến đài quan sát. Hơn 20 năm trước, ông Nguyễn Văn Nghỉ ở huyện Chợ Mới đã sưu tập rất nhiều gỗ lũa. Ban đầu ông trục vớt chúng để khơi thông dòng chảy, hạn chế tình trạng lưới đánh cá mắc vào thân cây. Lâu dần, ông yêu mến và muốn lưu giữ những thân gỗ trầm thủy này. Ba năm trước, ông Nghỉ dùng số gỗ lũa để xây khu du lịch ven sông Tiền rộng 6 ha. Đặc sắc trong các vật liệu từ gỗ lũa là bức tranh điêu khắc về phong cảnh làng quê Việt Nam xưa dài hơn 24 m, nặng 20 tấn. Bức tranh do nghệ nhân ở Huế thực hiện trong 7 năm, trên khúc gỗ trầm thủy khủng, tùy từng đoạn có chiều cao từ 1,5 - 1,8 m. Cạnh bức tranh là bộ sưu tập hàng trăm chiếc xe máy biển số độc lạ như tứ quý, sảnh tiến tới của nhiều dòng xe nổi tiếng. Dọc các lối đi là những tiểu cảnh làm từ gỗ lũa. Một số được điêu khắc thành các con vật, chim muông. Những cây gỗ lũa kích thước lớn được tận dụng làm đài quan sát cao 26 m, hoặc móng trụ để xây nhà nghỉ, cầu vượt. Khuôn viên cũng được phủ bởi nhiều cây kiểng, dừa cùng dãy nhà sàn ven sông. Tại đây du khách được ngắm hoàng hôn trên sông, tắm sông và thưởng thức ẩm thực miền Tây. Chị Phúc Điền, du khách ở TP HCM, cho biết khá thích với khung cảnh miền Tây yên bình ở Cồn Én. Chị cũng bất ngờ với sự kỳ công của người đã sưu tập hàng nghìn thân gỗ lũa và biến chúng thành điểm tham quan độc đáo. Cồn Én, nằm cách TP HCM 170 km, du khách có thể đến đây từ hướng quốc lộ 30 của tỉnh Đồng Tháp hoặc lên phà Tấn Long vượt sông Tiền từ phía huyện Chợ Mới. Giá vé vào cổng là 80.000 đồng. Ngọc Tài</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gỗ lũa từ sông Tiền tạo nên khu du lịch Cồn Én, với tiểu cảnh, đài quan sát và bức tranh điêu khắc dài 24 m. Du khách đến TP HCM qua quốc lộ 30 hoặc phà Tấn Long thăm đảo này với giá vé 80.000 đồng, nơi người dân đã biến hàng nghìn thân gỗ lũa thành điểm tham quan yên bình.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>{
+  "id": 3,
+  "style": "news_brief",
+  "article": "Cồn Én nằm giữa sông Tiền, thuộc xã Tấn Mỹ, rộng hơn 300 ha. Nơi đây ngoài là điểm đến ngắm dòng Tiền Giang, đón gió sông mát dịu, còn là địa chỉ thu hút khách với bộ sưu tập gỗ lũa nội thất độc đáo của khu du lịch trên cồn. Gỗ lũa tức những thân cây khủng, vớt từ đáy sông, bên ngoài bị dòng nước bào mòn, chỉ còn phần lõi bền chắc. Hàng nghìn thân gỗ lũa được người chủ tuyển chọn làm vật liệu chính xây Khu du lịch sinh thái Cồn Én từ tiểu cảnh, nhà đến đài quan sát. Hơn 20 năm trước, ông Nguyễn Văn Nghỉ ở huyện Chợ Mới đã sưu tập rất nhiều gỗ lũa. Ban đầu ông trục vớt chúng để khơi thông dòng chảy, hạn chế tình trạng lưới đánh cá mắc vào thân cây. Lâu dần, ông yêu mến và muốn lưu giữ những thân gỗ trầm thủy này. Ba năm trước, ông Nghỉ dùng số gỗ lũa để xây khu du lịch ven sông Tiền rộng 6 ha. Đặc sắc trong các vật liệu từ gỗ lũa là bức tranh điêu khắc về phong cảnh làng quê Việt Nam xưa dài hơn 24 m, nặng 20 tấn. Bức tranh do nghệ nhân ở Huế thực hiện trong 7 năm, trên khúc gỗ trầm thủy khủng, tùy từng đoạn có chiều cao từ 1,5 - 1,8 m. Cạnh bức tranh là bộ sưu tập hàng trăm chiếc xe máy biển số độc lạ như tứ quý, sảnh tiến tới của nhiều dòng xe nổi tiếng. Dọc các lối đi là những tiểu cảnh làm từ gỗ lũa. Một số được điêu khắc thành các con vật, chim muông. Những cây gỗ lũa kích thước lớn được tận dụng làm đài quan sát cao 26 m, hoặc móng trụ để xây nhà nghỉ, cầu vượt. Khuôn viên cũng được phủ bởi nhiều cây kiểng, dừa cùng dãy nhà sàn ven sông. Tại đây du khách được ngắm hoàng hôn trên sông, tắm sông và thưởng thức ẩm thực miền Tây. Chị Phúc Điền, du khách ở TP HCM, cho biết khá thích với khung cảnh miền Tây yên bình ở Cồn Én. Chị cũng bất ngờ với sự kỳ công của người đã sưu tập hàng nghìn thân gỗ lũa và biến chúng thành điểm tham quan độc đáo. Cồn Én, nằm cách TP HCM 170 km, du khách có thể đến đây từ hướng quốc lộ 30 của tỉnh Đồng Tháp hoặc lên phà Tấn Long vượt sông Tiền từ phía huyện Chợ Mới. Giá vé vào cổng là 80.000 đồng. Ngọc Tài",
+  "summary": "Gỗ lũa từ sông Tiền tạo nên khu du lịch Cồn Én, với tiểu cảnh, đài quan sát và bức tranh điêu khắc dài 24 m. Du khách đến TP HCM qua quốc lộ 30 hoặc phà Tấn Long thăm đảo này với giá vé 80.000 đồng, nơi người dân đã biến hàng nghìn thân gỗ lũa thành điểm tham quan yên bình.",
+  "faithfulness_score": 0.8,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin nhưng có thiếu sót một số chi tiết quan trọng như vị trí của Cồn Én, diện tích khu du lịch và một số hoạt động du lịch khác",
+  "relevance_score": 0.7,
+  "relevance_reason": "Bản tóm tắt chưa bao hàm đủ các ý chính quan trọng nhất như vị trí địa lý, các hoạt động du lịch và đặc điểm nổi bật của khu du lịch Cồn Én",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt có mạch lạc, logic và dễ đọc, tuy nhiên có thể cải thiện bằng cách thêm một số chi tiết quan trọng và tránh trùng lặp thông tin"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Văn phòng mới của MayTrip tại địa chỉ 833 Lê Hồng Phong, quận 10, nhằm mở rộng dịch vụ và nâng cao trải nghiệm khách hàng khu vực phía Nam. Văn phòng mới được kỳ vọng là điểm đến thuận tiện cho khách hàng trong việc tìm hiểu và sử dụng dịch vụ của công ty. Trong ngày khai trương, MayTrip trao tặng nhiều quà tặng và ưu đãi cho khách tham dự. Các voucher gồm: 2 triệu đồng cho khách đăng ký tour Bắc Á trong ba ngày khai trương, 1 triệu đồng cho tour Đông Nam Á trong ba tháng từ ngày khai trương, 500.000 đồng cho dịch vụ tour nội địa trong một năm, 200.000 đồng dịch vụ đặt phòng khách sạn hoặc xe du lịch trong 6 tháng và 100.000 đồng với dịch vụ vé máy bay trong 6 tháng. Buổi lễ khai trương văn phòng tại Sài Gòn còn giới thiệu các chương trìnhtour Nhật Bảndịp Tết Âm lịch như cung đường vàng trải nghiệm trượt tuyết, Hokkaido - miền tuyết trắng. Những chuyến đi này được MayTrip thiết kế kỹ lưỡng, phù hợp với không khí đón xuân cho gia đình và cặp đôi Việt trong dịp Tết Nguyên đán. Năm nay, MayTrip xác định tour Hokkaido là sản phẩm 'đinh' trong dịp Tết Nguyên đán. Hokkaido nằm ở miền Bắc Nhật Bản, nổi tiếng với những đợt tuyết dày và phong cảnh mùa đông đặc trưng. Tour Hokkaido dịp Tết là hành trình lý tưởng để du khách tận hưởng kỳ nghỉ theo cách mới mẻ và ấn tượng trong tuyết trắng. Bên cạnh đó, tour Hokkaido của MayTrip cũng mang đến trải nghiệm suối nước nóng onsen giữa băng tuyết, giúp du khách thư giãn sau những hoạt động trong ngày. Bên cạnh đó, MayTrip cũng cung cấp các tour du lịch khác với lịch khởi hành linh hoạt kéo dài đến hết năm 2025, gồm hành trình ngắm hoa anh đào, hoa mơ, mận và nghỉ lễ 30/4 và 1/5. Các hành trình này dựa trên xu hướng và sở thích của du khách Việt Nam. Theo đại diện công ty, sự kiện khai trương văn phòng mới tại TP HCM đánh dấu bước phát triển mới của MayTrip. Với mục tiêu ưu tiên trải nghiệm khách hàng, đơn vị hy vọng nhận được sự ủng hộ từ khách hàng để trở thành công ty lữ hành hàng đầu, hướng mục tiêu thương hiệu toàn cầu vào năm 2030. Ngoài TP HCM, MayTrip còn có văn phòng tại Hải Phòng và TP Vinh. Các văn phòng này giúp MayTrip dễ dàng tiếp cận và đáp ứng nhu cầu đa dạng của khách hàng. Công ty cam kết đảm bảo chất lượng dịch vụ để mang lại chuyến đi an toàn, trọn vẹn cho khách hàng. Thanh Thư</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MayTrip khai trương văn phòng mới tại 833 Lê Hồng Phong, quận 10 (TP HCM), với ưu đãi và tour Hokkaido dịp Tết Nguyên đán. Công ty đặt mục tiêu trở thành công ty lữ hành hàng đầu toàn cầu vào năm 2030, cam kết chất lượng dịch vụ an toàn cho khách.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>{
+  "id": 4,
+  "style": "news_brief",
+  "article": "Văn phòng mới của MayTrip tại địa chỉ 833 Lê Hồng Phong, quận 10, nhằm mở rộng dịch vụ và nâng cao trải nghiệm khách hàng khu vực phía Nam. Văn phòng mới được kỳ vọng là điểm đến thuận tiện cho khách hàng trong việc tìm hiểu và sử dụng dịch vụ của công ty. Trong ngày khai trương, MayTrip trao tặng nhiều quà tặng và ưu đãi cho khách tham dự. Các voucher gồm: 2 triệu đồng cho khách đăng ký tour Bắc Á trong ba ngày khai trương, 1 triệu đồng cho tour Đông Nam Á trong ba tháng từ ngày khai trương, 500.000 đồng cho dịch vụ tour nội địa trong một năm, 200.000 đồng dịch vụ đặt phòng khách sạn hoặc xe du lịch trong 6 tháng và 100.000 đồng với dịch vụ vé máy bay trong 6 tháng. Buổi lễ khai trương văn phòng tại Sài Gòn còn giới thiệu các chương trìnhtour Nhật Bảndịp Tết Âm lịch như cung đường vàng trải nghiệm trượt tuyết, Hokkaido - miền tuyết trắng. Những chuyến đi này được MayTrip thiết kế kỹ lưỡng, phù hợp với không khí đón xuân cho gia đình và cặp đôi Việt trong dịp Tết Nguyên đán. Năm nay, MayTrip xác định tour Hokkaido là sản phẩm 'đinh' trong dịp Tết Nguyên đán. Hokkaido nằm ở miền Bắc Nhật Bản, nổi tiếng với những đợt tuyết dày và phong cảnh mùa đông đặc trưng. Tour Hokkaido dịp Tết là hành trình lý tưởng để du khách tận hưởng kỳ nghỉ theo cách mới mẻ và ấn tượng trong tuyết trắng. Bên cạnh đó, tour Hokkaido của MayTrip cũng mang đến trải nghiệm suối nước nóng onsen giữa băng tuyết, giúp du khách thư giãn sau những hoạt động trong ngày. Bên cạnh đó, MayTrip cũng cung cấp các tour du lịch khác với lịch khởi hành linh hoạt kéo dài đến hết năm 2025, gồm hành trình ngắm hoa anh đào, hoa mơ, mận và nghỉ lễ 30/4 và 1/5. Các hành trình này dựa trên xu hướng và sở thích của du khách Việt Nam. Theo đại diện công ty, sự kiện khai trương văn phòng mới tại TP HCM đánh dấu bước phát triển mới của MayTrip. Với mục tiêu ưu tiên trải nghiệm khách hàng, đơn vị hy vọng nhận được sự ủng hộ từ khách hàng để trở thành công ty lữ hành hàng đầu, hướng mục tiêu thương hiệu toàn cầu vào năm 2030. Ngoài TP HCM, MayTrip còn có văn phòng tại Hải Phòng và TP Vinh. Các văn phòng này giúp MayTrip dễ dàng tiếp cận và đáp ứng nhu cầu đa dạng của khách hàng. Công ty cam kết đảm bảo chất lượng dịch vụ để mang lại chuyến đi an toàn, trọn vẹn cho khách hàng. Thanh Thư",
+  "summary": "MayTrip khai trương văn phòng mới tại 833 Lê Hồng Phong, quận 10 (TP HCM), với ưu đãi và tour Hokkaido dịp Tết Nguyên đán. Công ty đặt mục tiêu trở thành công ty lữ hành hàng đầu toàn cầu vào năm 2030, cam kết chất lượng dịch vụ an toàn cho khách.",
+  "faithfulness_score": 0.9,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, nhưng có thể thêm chi tiết về các ưu đãi và tour du lịch để tăng tính trung thực",
+  "relevance_score": 0.8,
+  "relevance_reason": "Bản tóm tắt bao gồm các ý chính quan trọng, nhưng có thể bỏ sót thông điệp cốt lõi về mục tiêu của công ty và các văn phòng khác",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, nhưng có thể rút gọn một số chi tiết để tăng tính súc tích"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ngày 29/10, tại Khu du lịch Sun World Fansipan Legend, Hiệp hội Du lịch tỉnh Lào Cai công bố chương trình kích cầu du lịch lớn nhất năm với chủ đề 'Chạm Sa Pa - Chạm những tầng mây', diễn ra từ 2/11 đến 30/12. Trong thời gian này, 130 doanh nghiệp tại Sa Pa sẽ cung cấp nhiều ưu đãi lên đến 50% và cam kết đảm bảo chất lượng dịch vụ. Theo đó, Công ty Cáp treo Fansipan Sa Pa (Khu du lịch Sun World Fansipan Legend) áp dụng đồng giá vé cáp treo hai chiều Fansipan chỉ còn 550.000 đồng cho du khách Việt Nam. Mức giá này giảm 30% so với giá gốc. Du khách có thể khám phá đỉnh Fansipan, chiêm ngưỡng kiến trúc tâm linh và tham gia các hoạt động văn hóa của 7 dân tộc thiểu số Tây Bắc tại Bản Mây. Nhiều điểm du lịch khác tại Sa Pa cũng miễn phí vé tham quan và cung cấp ưu đãi hấp dẫn. Trong đó, vườn đá Tả Phìn và vườn hồng Mộng Mơ miễn phí vé, Khu du lịch Cát Cát miễn phí trải nghiệm ẩm thực Tây Bắc cùng các hoạt động vẽ sáp ong, xe lanh, dệt vải... với bà con dân bản. Các khách sạn như Chaulong Sapa, Amazing Sapa, Vườn Sa Pa, Arista Sa Pa và Le Bordeaux Sapa áp dụng giảm giá phòng trực tiếp tới 50%. Hotel de la Coupole và Lady Hill Sapa Resort có nhiều ưu đãi về dịch vụ ăn uống, spa. Một số nhà xe như Inter Bus Lines và Eco Sa Pa cũng giảm giá vé xe khứ hồi đến 30%, cung cấp đa dạng hình thức di chuyển từ xe limousine đến xe lớn. Ông Phạm Cao Vỹ, đại diện Hiệp hội Du lịch tỉnh Lào Cai nhấn mạnh sự cần thiết của việc kích cầu du lịch để phục hồi ngành sau ảnh hưởng nặng nề của bão lũ. Ông kêu gọi tất cả doanh nghiệp du lịch trên địa bàn tham gia nhằm tạo sức bật cho du lịch Sa Pa phát triển mạnh mẽ vào giai đoạn cuối năm 2024. Ông Nguyễn Xuân Chiến, Phó chủ tịch Sun Group Vùng Miền Bắc, cho biết trước đây chương trình kích cầu 'Đến Sa Pa - Bay giữa mùa hoa' thành công ngoài mong đợi. 'Lần này, thông qua chính sách ưu đãi sâu, chúng tôi hy vọng thu hút đông đảo du khách đến Sa Pa để khám phá vẻ đẹp độc đáo của mùa mây', ông Chiến nói. Ngoài chính sách ưu đãi sâu, tỉnh Lào Cai và thị xã Sa Pa tổ chức nhiều sự kiện văn hóa đặc sắc nhằm mang đến trải nghiệm độc đáo cho du khách. Các hoạt động bao gồm lễ hội truyền thống, triển lãm nghệ thuật, thể thao và giải trí. Đặc biệt là sự kiện ánh sáng 3D Mapping và lễ hội hoa sen đá lần đầu tiên được tổ chức tại Sun World Fansipan Legend. Sa Pa đang trong mùa mây - thời điểm lý tưởng để vui chơi ngoài trời. Ban tổ chức kỳ vọng chương trình kích cầu sẽ tăng sức hút của Sa Pa và củng cố vị thế là điểm đến hàng đầu miền Bắc. Thanh Thư</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>{
+  "id": 5,
+  "style": "news_brief",
+  "article": "Ngày 29/10, tại Khu du lịch Sun World Fansipan Legend, Hiệp hội Du lịch tỉnh Lào Cai công bố chương trình kích cầu du lịch lớn nhất năm với chủ đề 'Chạm Sa Pa - Chạm những tầng mây', diễn ra từ 2/11 đến 30/12. Trong thời gian này, 130 doanh nghiệp tại Sa Pa sẽ cung cấp nhiều ưu đãi lên đến 50% và cam kết đảm bảo chất lượng dịch vụ. Theo đó, Công ty Cáp treo Fansipan Sa Pa (Khu du lịch Sun World Fansipan Legend) áp dụng đồng giá vé cáp treo hai chiều Fansipan chỉ còn 550.000 đồng cho du khách Việt Nam. Mức giá này giảm 30% so với giá gốc. Du khách có thể khám phá đỉnh Fansipan, chiêm ngưỡng kiến trúc tâm linh và tham gia các hoạt động văn hóa của 7 dân tộc thiểu số Tây Bắc tại Bản Mây. Nhiều điểm du lịch khác tại Sa Pa cũng miễn phí vé tham quan và cung cấp ưu đãi hấp dẫn. Trong đó, vườn đá Tả Phìn và vườn hồng Mộng Mơ miễn phí vé, Khu du lịch Cát Cát miễn phí trải nghiệm ẩm thực Tây Bắc cùng các hoạt động vẽ sáp ong, xe lanh, dệt vải... với bà con dân bản. Các khách sạn như Chaulong Sapa, Amazing Sapa, Vườn Sa Pa, Arista Sa Pa và Le Bordeaux Sapa áp dụng giảm giá phòng trực tiếp tới 50%. Hotel de la Coupole và Lady Hill Sapa Resort có nhiều ưu đãi về dịch vụ ăn uống, spa. Một số nhà xe như Inter Bus Lines và Eco Sa Pa cũng giảm giá vé xe khứ hồi đến 30%, cung cấp đa dạng hình thức di chuyển từ xe limousine đến xe lớn. Ông Phạm Cao Vỹ, đại diện Hiệp hội Du lịch tỉnh Lào Cai nhấn mạnh sự cần thiết của việc kích cầu du lịch để phục hồi ngành sau ảnh hưởng nặng nề của bão lũ. Ông kêu gọi tất cả doanh nghiệp du lịch trên địa bàn tham gia nhằm tạo sức bật cho du lịch Sa Pa phát triển mạnh mẽ vào giai đoạn cuối năm 2024. Ông Nguyễn Xuân Chiến, Phó chủ tịch Sun Group Vùng Miền Bắc, cho biết trước đây chương trình kích cầu 'Đến Sa Pa - Bay giữa mùa hoa' thành công ngoài mong đợi. 'Lần này, thông qua chính sách ưu đãi sâu, chúng tôi hy vọng thu hút đông đảo du khách đến Sa Pa để khám phá vẻ đẹp độc đáo của mùa mây', ông Chiến nói. Ngoài chính sách ưu đãi sâu, tỉnh Lào Cai và thị xã Sa Pa tổ chức nhiều sự kiện văn hóa đặc sắc nhằm mang đến trải nghiệm độc đáo cho du khách. Các hoạt động bao gồm lễ hội truyền thống, triển lãm nghệ thuật, thể thao và giải trí. Đặc biệt là sự kiện ánh sáng 3D Mapping và lễ hội hoa sen đá lần đầu tiên được tổ chức tại Sun World Fansipan Legend. Sa Pa đang trong mùa mây - thời điểm lý tưởng để vui chơi ngoài trời. Ban tổ chức kỳ vọng chương trình kích cầu sẽ tăng sức hút của Sa Pa và củng cố vị thế là điểm đến hàng đầu miền Bắc. Thanh Thư",
+  "summary": "",
+  "faithfulness_score": 1.0,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, không sai số liệu và không xuyên tạc ý nghĩa của văn bản gốc.",
+  "relevance_score": 1.0,
+  "relevance_reason": "Bản tóm tắt bao hàm đủ các ý chính quan trọng nhất, không bỏ sót thông điệp cốt lõi nào.",
+  "coherence_conciseness_score": 1.0,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic, dễ đọc và loại bỏ được các chi tiết rườm rà/lặp từ không."
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Brisbane nằm phía đông nam bang Queensland, là thành phố lớn thứ ba tại Australia. Do gần đường xích đạo, khí hậu nơi đây ôn hòa, quanh năm nắng ấm. Trung tâm Brisbane không chỉ có những khối bê tông, khu mua sắm, mà còn bao phủ bởi mảng xanh, với 5 công viên và vườn thực vật nổi tiếng. Dưới đây là 5 điểm đến hút du khách ở Brisbane. South Bank Parklands Nằm bên bờ sông Brisbane, South Bank Parklands được ví như 'ốc đảo xanh' giữa lòng thành phố sôi động, nổi bật với rừng mưa nhiệt đới và loạt hoạt động giải trí cho mọi lứa tuổi. Ngay cửa ngõ công viên là thảm cỏ, hàng cây rợp bóng và vườn hoa. Nhiều người dân thường picnic, dã ngoại, vui chơi tại bãi biển nhân tạo Streets Beach, River Quay Green, Rainforest Green hay Liana Lounge. Ngoài ra, Wheel of Brisbane - vòng đu quay cao tới 60 m - là biểu tượng tại South Bank Parklands, dễ dàng ngắm toàn cảnh Brisbane từ trên cao. Roma Street Parkland Nằm cạnh ga xe lửa Roma Street, công viên cùng tên cũng được người dân lẫn du khách gọi là 'ốc đảo xanh mát' giữa Brisbane, ghi dấu với những khu vườn và bãi cỏ rộng lớn. Tại đây, du khách hòa mình vào khu vườn Spectacle - nơi trồng hàng nghìn gốc violets, cẩm chướng, delphiniums và foxgloves. Khí hậu ôn hòa thu hút chim kookaburras, gà lôi, vẹt. Bạn cũng có thể tổ chức tiệc BBQ ngoài trời, cho con khám phá công viên trẻ em. Brisbane City Botanic Gardens Nằm trên trục đường Alice, Brisbane City Botanic Gardens bảo tồn hàng nghìn loài thực vật quý hiếm, nổi bật với vẻ nguyên sơ. Khu vườn này là một trong những điểm đến lý tưởng cho người chuộng nét thanh bình giữa lòng đô thị. Tại đây, du khách có thể khám phá con đường dạo bộ ven sông, chiêm ngưỡng rặng thông Bunya được trồng từ năm 1858. Điểm đến tiếp theo là Bamboo Grove - con đường tre rợp mát, được ví như 'khu rừng xa xôi giữa thành phố hiện đại'. Vườn bách thảo tổ chức sự kiện quanh năm như biểu diễn Riverstage, lễ hội đa văn hóa, trưng bày nghệ thuật cùng hoạt động cộng đồng miễn phí. Trong đó, chợ Riverside Sunday Market hút hàng nghìn du khách nhờ gian hàng thủ công, trái cây tươi và ẩm thực độc đáo. Epicurious Garden Tại Epicurious, du khách có thể khám phá ẩm thực bang Queensland đa dạng, nhất là rau, củ, quả, thảo mộc hữu cơ theo mùa. 14 chuyên viên tình nguyện chăm sóc khu vườn kỹ lưỡng, mong truyền cảm hứng cho người yêu nấu ăn và trồng trọt. 'Tới Epicurious, tôi và bạn bè được hướng dẫn cách chăm sóc rau củ, trái cây, thảo mộc và thưởng thức miễn phí', một du khách viết trên Facebook, nhận hàng trăm nghìn lượt thích. Mount Coot-tha Botanic Gardens Mở cửa đón khách từ năm 1976, Mount Coot-tha Botanic Gardens tọa lạc chân núi Coot-tha, là vườn thực vật nhiệt đới hàng đầu Brisbane, diện tích đến 56 ha. Dạo quanh khu vườn, du khách có thể chiêm ngưỡng hoa xuân, các loài cây nhiệt đới và khu thảo dược. Nơi đây là điểm đến quen thuộc của người yêu thiên nhiên, picnic, mê hoạt động thể chất, với đường chạy bộ thoáng đãng. Để khám phá thành thủ phủ bang Queensland, bạn có thể chọn đường bay thẳng từ TP HCM đến Brisbane của Vietjet, với 9 giờ trên máy bay thân rộng, thoải mái cùng loạt dịch vụ tiện ích, ưu đãi như: bảo hiểm Sky Care miễn phí, chương trình tích điểm SkyJoy, đổi quà từ hơn 250 thương hiệu lớn toàn cầu. Trước đó ngày14-15/9, Vietjet đồng hành lễ hội thả diều Vietjet Redcliffe KiteFest tại Redcliffe, Queensland. Hãng hàng không Việt còn áp dụng nhiều chương trình ưu đãi nhân dịp đón hành khách thứ 200 triệu. Đông Vệ</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Brisbane, thành phố lớn thứ ba của Australia với khí hậu ôn hòa quanh năm. Thành phố có nhiều công viên và vườn thực vật nổi tiếng như South Bank Parklands, Roma Street Parkland và Brisbane City Botanic Gardens bảo tồn hàng nghìn loài cây quý hiếm trên trục đường Alice. Hội chợ Riverside Sunday Market hút du khách với gian hàng thủ công, trái cây tươi và ẩm thực độc đáo. Epicurious Garden giới thiệu ẩm thực Queensland đa dạng. Mount Coot-tha Botanic Gardens nằm trên núi Coot-tha, là vườn thực vật lớn của Brisbane. Vietjet cung cấp đường bay thẳng TP HCM - Brisbane với nhiều dịch vụ tiện ích và chương trình ưu đãi nhân dịp đón hành khách thứ 200 triệu.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>{
+  "id": 6,
+  "style": "news_brief",
+  "article": "Brisbane nằm phía đông nam bang Queensland, là thành phố lớn thứ ba tại Australia. Do gần đường xích đạo, khí hậu nơi đây ôn hòa, quanh năm nắng ấm. Trung tâm Brisbane không chỉ có những khối bê tông, khu mua sắm, mà còn bao phủ bởi mảng xanh, với 5 công viên và vườn thực vật nổi tiếng. Dưới đây là 5 điểm đến hút du khách ở Brisbane. South Bank Parklands Nằm bên bờ sông Brisbane, South Bank Parklands được ví như 'ốc đảo xanh' giữa lòng thành phố sôi động, nổi bật với rừng mưa nhiệt đới và loạt hoạt động giải trí cho mọi lứa tuổi. Ngay cửa ngõ công viên là thảm cỏ, hàng cây rợp bóng và vườn hoa. Nhiều người dân thường picnic, dã ngoại, vui chơi tại bãi biển nhân tạo Streets Beach, River Quay Green, Rainforest Green hay Liana Lounge. Ngoài ra, Wheel of Brisbane - vòng đu quay cao tới 60 m - là biểu tượng tại South Bank Parklands, dễ dàng ngắm toàn cảnh Brisbane từ trên cao. Roma Street Parkland Nằm cạnh ga xe lửa Roma Street, công viên cùng tên cũng được người dân lẫn du khách gọi là 'ốc đảo xanh mát' giữa Brisbane, ghi dấu với những khu vườn và bãi cỏ rộng lớn. Tại đây, du khách hòa mình vào khu vườn Spectacle - nơi trồng hàng nghìn gốc violets, cẩm chướng, delphiniums và foxgloves. Khí hậu ôn hòa thu hút chim kookaburras, gà lôi, vẹt. Bạn cũng có thể tổ chức tiệc BBQ ngoài trời, cho con khám phá công viên trẻ em. Brisbane City Botanic Gardens Nằm trên trục đường Alice, Brisbane City Botanic Gardens bảo tồn hàng nghìn loài thực vật quý hiếm, nổi bật với vẻ nguyên sơ. Khu vườn này là một trong những điểm đến lý tưởng cho người chuộng nét thanh bình giữa lòng đô thị. Tại đây, du khách có thể khám phá con đường dạo bộ ven sông, chiêm ngưỡng rặng thông Bunya được trồng từ năm 1858. Điểm đến tiếp theo là Bamboo Grove - con đường tre rợp mát, được ví như 'khu rừng xa xôi giữa thành phố hiện đại'. Vườn bách thảo tổ chức sự kiện quanh năm như biểu diễn Riverstage, lễ hội đa văn hóa, trưng bày nghệ thuật cùng hoạt động cộng đồng miễn phí. Trong đó, chợ Riverside Sunday Market hút hàng nghìn du khách nhờ gian hàng thủ công, trái cây tươi và ẩm thực độc đáo. Epicurious Garden Tại Epicurious, du khách có thể khám phá ẩm thực bang Queensland đa dạng, nhất là rau, củ, quả, thảo mộc hữu cơ theo mùa. 14 chuyên viên tình nguyện chăm sóc khu vườn kỹ lưỡng, mong truyền cảm hứng cho người yêu nấu ăn và trồng trọt. 'Tới Epicurious, tôi và bạn bè được hướng dẫn cách chăm sóc rau củ, trái cây, thảo mộc và thưởng thức miễn phí', một du khách viết trên Facebook, nhận hàng trăm nghìn lượt thích. Mount Coot-tha Botanic Gardens Mở cửa đón khách từ năm 1976, Mount Coot-tha Botanic Gardens tọa lạc chân núi Coot-tha, là vườn thực vật nhiệt đới hàng đầu Brisbane, diện tích đến 56 ha. Dạo quanh khu vườn, du khách có thể chiêm ngưỡng hoa xuân, các loài cây nhiệt đới và khu thảo dược. Nơi đây là điểm đến quen thuộc của người yêu thiên nhiên, picnic, mê hoạt động thể chất, với đường chạy bộ thoáng đãng. Để khám phá thành thủ phủ bang Queensland, bạn có thể chọn đường bay thẳng từ TP HCM đến Brisbane của Vietjet, với 9 giờ trên máy bay thân rộng, thoải mái cùng loạt dịch vụ tiện ích, ưu đãi như: bảo hiểm Sky Care miễn phí, chương trình tích điểm SkyJoy, đổi quà từ hơn 250 thương hiệu lớn toàn cầu. Trước đó ngày14-15/9, Vietjet đồng hành lễ hội thả diều Vietjet Redcliffe KiteFest tại Redcliffe, Queensland. Hãng hàng không Việt còn áp dụng nhiều chương trình ưu đãi nhân dịp đón hành khách thứ 200 triệu. Đông Vệ",
+  "summary": "Brisbane, thành phố lớn thứ ba của Australia với khí hậu ôn hòa quanh năm. Thành phố có nhiều công viên và vườn thực vật nổi tiếng như South Bank Parklands, Roma Street Parkland và Brisbane City Botanic Gardens bảo tồn hàng nghìn loài cây quý hiếm trên trục đường Alice. Hội chợ Riverside Sunday Market hút du khách với gian hàng thủ công, trái cây tươi và ẩm thực độc đáo. Epicurious Garden giới thiệu ẩm thực Queensland đa dạng. Mount Coot-tha Botanic Gardens nằm trên núi Coot-tha, là vườn thực vật lớn của Brisbane. Vietjet cung cấp đường bay thẳng TP HCM - Brisbane với nhiều dịch vụ tiện ích và chương trình ưu đãi nhân dịp đón hành khách thứ 200 triệu.",
+  "faithfulness_score": 0.8,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng có bỏ sót một số chi tiết quan trọng như mô tả cụ thể về các hoạt động giải trí tại South Bank Parklands và Roma Street Parkland",
+  "relevance_score": 0.9,
+  "relevance_reason": "Bản tóm tắt bao hàm đủ các ý chính quan trọng nhất về các điểm đến hút du khách ở Brisbane, tuy nhiên có thể thêm thông tin về các sự kiện và hoạt động tại các công viên",
+  "coherence_conciseness_score": 0.7,
+  "coherence_conciseness_reason": "Bản tóm tắt có logic và dễ đọc nhưng có thể cải thiện bằng cách loại bỏ các từ ngữ lặp từ và sắp xếp lại cấu trúc câu cho rõ ràng hơn"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Công ty du lịch NhatbanAZ mở bán chùm tour Nhật Bản khởi hành dịp Tết Dương lịch và Âm lịch từ đầu tháng 10. Trong đó, các tour truyền thống đến Osaka, Kyoto và Tokyo được làm mới bằng những hoạt động phù hợp với mùa đông xuân như trượt tuyết tại Fujiten Resort, ngắm tuyết làng cổ Oshino Hakkai và tham gia lễ hội ánh sáng Nabana no sato. NhatbanAZ cũng mở rộng các cung đường mới cho du khách trải nghiệm trong dịp Tết 2025. Cụ thể, tour Hokkaido gồm Asahikawa, Monbetsu và Sapporo với giá 55,9 triệu đồng mỗi khách. Du khách sẽ tham gia câu cá trên băng, đi tàu phá băng và thưởng thức bia hơi tại Sapporo, cùng dịch vụ hàng không 5 sao và lưu trú khách sạn 4 sao quốc tế. Tour thứ hai là chuyến thăm làng cổ Shirakawago, núi Phú Sĩ và Tokyo trong 6 ngày 5 đêm với giá 31,9 triệu đồng mỗi khách. Du khách sẽ được chiêm ngưỡng tuyết trắng tại Shirakawago, một Di sản Văn hóa Thế giới của UNESCO từ năm 1995. Tour cũng gồm tham quan lâu đài Matsumoto - di tích bảo vật quốc gia của Nhật Bản và trải nghiệm trượt tuyết tại Fujiten Snow Resort - top 3 khu trượt tuyết nổi tiếng. Bà Hồ Như Thảo, Giám đốc Điều hành NhatbanAZ Văn phòng TP HCM cho biết sản phẩm mới này nhận được sự quan tâm lớn từ du khách, đặc biệt là những người từng đi Nhật và muốn trở lại với hành trình mới. Khu vực Hokkaido được biết đến với tuyết rơi dày đặc hơn Tokyo hay Osaka, nên lịch khởi hành tour Hokkaido dịp Tết Âm lịch nhận được nhiều đăng ký giữ chỗ. Trong dịp Tết Nguyên đán 2025, NhatbanAZ cung cấp các hành trình từ 5 đến 6 ngày với mức giá cơ bản đến cao cấp, khoảng 31,9 - 55,9 triệu đồng mỗi khách để đáp ứng nhu cầu đa dạng. Giá tour Tết có phần chênh lệch so với ngày thường và tăng so với cùng kỳ năm trước. Do đó, NhatbanAZ chủ động gặp gỡ và làm việc với các đối tác cung cấp dịch vụ, từ đó xây dựng chương trình, đưa ra chính sách ưu đãi tốt nhất cho khách hàng. Với kinh nghiệm hơn 15 năm trong ngành du lịch chuyên thị trường Nhật Bản, NhatbanAZ thuộc danh sách công ty chỉ định nộp visa bởi Đại sứ quán Nhật Bản đề xuất. Đồng thời là đối tác chiến lược của các hãng hàng không, khách sạn và đối tác land tour uy tín tại Nhật Bản. Công ty cũng là nhà tư vấn và tổ chức những chuyến Famtrip kết nối các công ty du lịch Việt Nam tới tham quan xúc tiến đầu tư, hợp tác tại Nhật Bản. Thanh Thư</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>{
+  "id": 7,
+  "style": "news_brief",
+  "article": "Công ty du lịch NhatbanAZ mở bán chùm tour Nhật Bản khởi hành dịp Tết Dương lịch và Âm lịch từ đầu tháng 10. Trong đó, các tour truyền thống đến Osaka, Kyoto và Tokyo được làm mới bằng những hoạt động phù hợp với mùa đông xuân như trượt tuyết tại Fujiten Resort, ngắm tuyết làng cổ Oshino Hakkai và tham gia lễ hội ánh sáng Nabana no sato. NhatbanAZ cũng mở rộng các cung đường mới cho du khách trải nghiệm trong dịp Tết 2025. Cụ thể, tour Hokkaido gồm Asahikawa, Monbetsu và Sapporo với giá 55,9 triệu đồng mỗi khách. Du khách sẽ tham gia câu cá trên băng, đi tàu phá băng và thưởng thức bia hơi tại Sapporo, cùng dịch vụ hàng không 5 sao và lưu trú khách sạn 4 sao quốc tế. Tour thứ hai là chuyến thăm làng cổ Shirakawago, núi Phú Sĩ và Tokyo trong 6 ngày 5 đêm với giá 31,9 triệu đồng mỗi khách. Du khách sẽ được chiêm ngưỡng tuyết trắng tại Shirakawago, một Di sản Văn hóa Thế giới của UNESCO từ năm 1995. Tour cũng gồm tham quan lâu đài Matsumoto - di tích bảo vật quốc gia của Nhật Bản và trải nghiệm trượt tuyết tại Fujiten Snow Resort - top 3 khu trượt tuyết nổi tiếng. Bà Hồ Như Thảo, Giám đốc Điều hành NhatbanAZ Văn phòng TP HCM cho biết sản phẩm mới này nhận được sự quan tâm lớn từ du khách, đặc biệt là những người từng đi Nhật và muốn trở lại với hành trình mới. Khu vực Hokkaido được biết đến với tuyết rơi dày đặc hơn Tokyo hay Osaka, nên lịch khởi hành tour Hokkaido dịp Tết Âm lịch nhận được nhiều đăng ký giữ chỗ. Trong dịp Tết Nguyên đán 2025, NhatbanAZ cung cấp các hành trình từ 5 đến 6 ngày với mức giá cơ bản đến cao cấp, khoảng 31,9 - 55,9 triệu đồng mỗi khách để đáp ứng nhu cầu đa dạng. Giá tour Tết có phần chênh lệch so với ngày thường và tăng so với cùng kỳ năm trước. Do đó, NhatbanAZ chủ động gặp gỡ và làm việc với các đối tác cung cấp dịch vụ, từ đó xây dựng chương trình, đưa ra chính sách ưu đãi tốt nhất cho khách hàng. Với kinh nghiệm hơn 15 năm trong ngành du lịch chuyên thị trường Nhật Bản, NhatbanAZ thuộc danh sách công ty chỉ định nộp visa bởi Đại sứ quán Nhật Bản đề xuất. Đồng thời là đối tác chiến lược của các hãng hàng không, khách sạn và đối tác land tour uy tín tại Nhật Bản. Công ty cũng là nhà tư vấn và tổ chức những chuyến Famtrip kết nối các công ty du lịch Việt Nam tới tham quan xúc tiến đầu tư, hợp tác tại Nhật Bản. Thanh Thư",
+  "summary": "",
+  "faithfulness_score": 1.0,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, sai số liệu, hay xuyên tạc ý nghĩa của văn bản gốc",
+  "relevance_score": 1.0,
+  "relevance_reason": "Bản tóm tắt bao hàm đủ các ý chính quan trọng nhất và không bỏ sót thông điệp cốt lõi nào",
+  "coherence_conciseness_score": 1.0,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic, dễ đọc và loại bỏ được các chi tiết rườm rà/lặp từ không"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Theo bảng xếp hạng 20 quốc gia tốt nhất thế giới năm 2024 (The Best Countries in the World) do tạp chí du lịch Mỹ Condé Nast Traveler công bố vào tháng 10, Việt Nam ở vị trí 15 với 89 điểm. Một điểm đến khác thuộc Đông Nam Á có mặt trong danh sách này là Thái Lan, xếp thứ ba với 92,29 điểm. Đứng đầu top 20 là Nhật Bản với 95,32 điểm. Xếp hạng nằm trong giải thưởng thường niênReaders' Choice Awards của tạp chí Mỹ, dựa trên đánh giá của hơn 575.000 độc giả về các trải nghiệm du lịch ở mỗi quốc gia, xét theo các tiêu chí văn hóa, cảnh quan, dịch vụ du lịch và cơ sở hạ tầng. Độc giả của Condé Nast Traveler nhận xét Việt Nam thu hút du khách nhờ vẻ đẹp mộc mạc và quyến rũ. 'Với lượng khách nước ngoài đang trên đà tăng từ 2019 đến nay, Việt Nam không còn là điểm đến đáng chú ý mà thành điểm đến đáng ghé thăm', biên tập tờ Condé Nast Traveler viết. Theo số liệu từ Tổng cục Thống kê, trong 9 tháng đầu năm, Việt Nam đón hơn 12,7 triệu lượt khách quốc tế, vượt lượng khách cả năm 2023 là 12,6 triệu lượt. Lượng khách quốc tế đến Việt Nam tăng trưởng tích cực 9 tháng đầu năm 2024, với một số thị trường phục hồi hoàn toàn, tăng mạnh so với 2019, theo Cục Du lịch Quốc gia. Cục cũng dự đoán với đà tăng trường như hiện nay, Việt Nam sẽ hoàn thành mục tiêu đón 17-18 triệu lượt khách quốc tế năm 2024. Thái Lan được tạp chí Mỹ nhận xét là quốc gia đa dạng cảnh quan, giao thông thuận tiện với nhiều tàu thuyền, xe buýt đêm và chuyến bay nội địa giá rẻ. Ẩm thực cũng là điểm sáng của xứ chùa Vàng khi có nhiều khu chợ đêm nhộn nhịp, bày bán đặc sản địa phương. 8 tháng đầu năm 2024, Thái Lan đón hơn 20 triệu lượt khách quốc tế, tăng 34% so với cùng kỳ năm trước. Quốc gia này đặt mục tiêu đón ít nhất 36-37 triệu lượt khách nước ngoài trong cả năm nay, kỳ vọng thu về khoảng 3.500 tỷ baht (95,5 tỷ USD). Condé Nast Traveler là tạp chí du lịch nổi tiếng toàn cầu, ra mắt vào năm 1987. Các bảng xếp hạng của Condé Nast Traveler như Readers' Choice Awards được chuyên gia du lịch đánh giá là uy tín vì dựa trên ý kiến từ hàng triệu độc giả quốc tế. Bích Phương(TheoCNTraveller)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>LỖI: 'NoneType' object is not iterable</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>{
-  "id": 1,
-  "style": "news_brief",
-  "article": "Taste Studio do thương hiệu Regent Hotels &amp; Resorts tổ chức nhằm mang đến trải nghiệm đa giác quan qua ẩm thực và nghệ thuật. Sự kiện này quy tụ nhiều đầu bếp và nghệ sĩ nổi tiếng, từ nhà thiết kế thời trang đến nhạc sĩ, kết hợp cùng các thương hiệu hàng đầu như Vietnam Airlines. Sự kiện hướng đến phân khúc khách hàng sang trọng. Mùa một và hai diễn ra lần được vào tháng 4, tháng 11 năm ngoái. Taste Studio năm nay với chủ đề 'Dáng hình của biển', giới hạn 20 khách mời mỗi tối. Các khách mời được tham gia vào chuỗi khám phá gồm 7 chương đặc sắc về vẻ đẹp của biển, qua lăng kính nghệ sĩ tài hoa Mr. Dripping - nghệ sĩ vẽ tranh bằng phương pháp nhỏ giọt (drip art). Không gian nhà hàng, nơi diễn ra sự kiện với nội thất dùng tre, mây và tầm vông do kiến trúc sư Nguyễn Trung Nghĩa thiết kế. Ngoài hai nghệ sĩ này, Taste Studio còn có sự tham gia của bếp trưởng Francesco đến từ Milan, với 20 năm kinh nghiệm làm việc tại các khách sạn danh tiếng thế giới, đang bắt đầu hành trình mới tại Việt Nam. Ông đảm nhận vai trò cố vấn ẩm thực tại Regent Phú Quốc, mang đến trải nghiệm độc đáo cho thực khách. Bên cạnh đó, phó bếp trưởng điều hành Huân Trần tại chương trình mong muốn chinh phục các hương vị vùng miền khác nhau. Được nếm nhiều nguyên liệu địa phương và các loại gia vị đặc biệt, vị đầu bếp để lại điểm nhấn riêng trong cách giữ gìn, nâng tầm phong vị của quê hương tại Regent Phú Quốc. Chương trình có sự góp mặt của bếp trưởng nhà hàng Oku - Andy Huỳnh. Trước khi gia nhập Regent Phú Quốc, anh phát triển kỹ thuật nấu ăn Nhật Bản tại Nobu, San Diego và Nassau. Các món ăn của Andy luôn mang ý nghĩa hướng về cội nguồn. Bếp trưởng nhà hàng Ocean Club Daniel và bếp trưởng Duyến Nguyễn của khu nghỉ dưỡng này cũng tham gia, sáng tạo một số hương vị độc đáo từ nguyên liệu địa phương. Đại diện Regent Phú Quốc cho biết, thông qua Taste Studio, đơn vị mong muốn tiếp tục kiến tạo trải nghiệm đưa nét bản địa đặc sắc của Việt Nam lên bản đồ thế giới, từ đó chinh phục khách hàng hạng sang và giới chuyên gia. Thanh Thư",
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>{
+  "id": 8,
+  "style": "news_brief",
+  "article": "Theo bảng xếp hạng 20 quốc gia tốt nhất thế giới năm 2024 (The Best Countries in the World) do tạp chí du lịch Mỹ Condé Nast Traveler công bố vào tháng 10, Việt Nam ở vị trí 15 với 89 điểm. Một điểm đến khác thuộc Đông Nam Á có mặt trong danh sách này là Thái Lan, xếp thứ ba với 92,29 điểm. Đứng đầu top 20 là Nhật Bản với 95,32 điểm. Xếp hạng nằm trong giải thưởng thường niênReaders' Choice Awards của tạp chí Mỹ, dựa trên đánh giá của hơn 575.000 độc giả về các trải nghiệm du lịch ở mỗi quốc gia, xét theo các tiêu chí văn hóa, cảnh quan, dịch vụ du lịch và cơ sở hạ tầng. Độc giả của Condé Nast Traveler nhận xét Việt Nam thu hút du khách nhờ vẻ đẹp mộc mạc và quyến rũ. 'Với lượng khách nước ngoài đang trên đà tăng từ 2019 đến nay, Việt Nam không còn là điểm đến đáng chú ý mà thành điểm đến đáng ghé thăm', biên tập tờ Condé Nast Traveler viết. Theo số liệu từ Tổng cục Thống kê, trong 9 tháng đầu năm, Việt Nam đón hơn 12,7 triệu lượt khách quốc tế, vượt lượng khách cả năm 2023 là 12,6 triệu lượt. Lượng khách quốc tế đến Việt Nam tăng trưởng tích cực 9 tháng đầu năm 2024, với một số thị trường phục hồi hoàn toàn, tăng mạnh so với 2019, theo Cục Du lịch Quốc gia. Cục cũng dự đoán với đà tăng trường như hiện nay, Việt Nam sẽ hoàn thành mục tiêu đón 17-18 triệu lượt khách quốc tế năm 2024. Thái Lan được tạp chí Mỹ nhận xét là quốc gia đa dạng cảnh quan, giao thông thuận tiện với nhiều tàu thuyền, xe buýt đêm và chuyến bay nội địa giá rẻ. Ẩm thực cũng là điểm sáng của xứ chùa Vàng khi có nhiều khu chợ đêm nhộn nhịp, bày bán đặc sản địa phương. 8 tháng đầu năm 2024, Thái Lan đón hơn 20 triệu lượt khách quốc tế, tăng 34% so với cùng kỳ năm trước. Quốc gia này đặt mục tiêu đón ít nhất 36-37 triệu lượt khách nước ngoài trong cả năm nay, kỳ vọng thu về khoảng 3.500 tỷ baht (95,5 tỷ USD). Condé Nast Traveler là tạp chí du lịch nổi tiếng toàn cầu, ra mắt vào năm 1987. Các bảng xếp hạng của Condé Nast Traveler như Readers' Choice Awards được chuyên gia du lịch đánh giá là uy tín vì dựa trên ý kiến từ hàng triệu độc giả quốc tế. Bích Phương(TheoCNTraveller)",
   "summary": "LỖI: 'NoneType' object is not iterable",
   "faithfulness_score": 0.0,
-  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin nào về văn bản gốc, không phản ánh nội dung của sự kiện Taste Studio",
+  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin gì về văn bản gốc, không có nội dung để đánh giá tính trung thực.",
   "relevance_score": 0.0,
-  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào về sự kiện, không đề cập đến chủ đề, khách mời, hoặc mục đích của sự kiện",
+  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không thể đánh giá tính bao quát.",
   "coherence_conciseness_score": 0.0,
-  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá về tính mạch lạc và súc tích"
-}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hai giải thưởng gồm 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới'. Đây cũng là năm thứ tư liên tiếp đơn vị đạt giải thưởng này, sau quá trình thẩm định từ hội đồng chuyên môn toàn cầu và bình chọn bởi hàng nghìn du khách, khách sạn quốc tế khác. 'Giải thưởng góp phần khẳng định Amiana Resort Nha Trang là điểm đến lý tưởng cho du khách tìm kiếm không gian riêng tư, gần gũi thiên nhiên với kiến trúc cao cấp, mang lại trải nghiệm sang trọng, độc đáo', đại diện resort chia sẻ. Amiana có kiến trúc hòa hợp thiên nhiên, kết hợp yếu tố truyền thống và hiện đại, tạo nên không gian thư giãn, sang trọng nhưng vẫn giữ được cảm giác gần gũi, yên bình. Bãi biển riêng tư với hàng dừa rợp bóng xanh mát là nơi du khách có thể thư giãn, nghỉ ngơi thoải mái. Resort còn tận dụng địa hình tự nhiên để bố trí các công trình công cộng như hồ bơi, nhà hàng, phòng hội nghị, spa... Các yếu tố đậm chất nhiệt đới như dừa xanh, sóng biển, đá và gỗ được lồng ghép khéo léo trong từng chi tiết thiết kế nội ngoại thất. Biệt thự, phòng nghỉ, nhà hàng đều có sự kết hợp giữa vật liệu tự nhiên và công nghệ hiện đại. Mỗi căn biệt thự đều mang kiến trúc mở, sử dụng nội thất chủ yếu từ gỗ, đá tự nhiên. Tất cả phòng đều có cửa sổ lớn và ban công rộng, tối ưu tầm nhìn hướng biển với cảnh quan thiên nhiên vây quanh. Biệt thự còn có hồ bơi riêng, không gian vườn với các loại cây nhiệt đới, đảm bảo yếu tố riêng tư cho khách hàng. Resort không chỉ chú trọng xây dựng công trình tiện ích, mà còn đặc biệt lưu ý việc bảo vệ môi trường, sử dụng các giải pháp bền vững. Những không gian xanh, vườn cây, hồ nước đều được bố trí hợp lý, tạo nên hệ sinh thái tự nhiên trong lòng khu nghỉ dưỡng. Theo đại diện Amiana Resort Nha Trang, những chi tiết kiến trúc thông minh cùng không gian mở, vật liệu tự nhiên, sự khéo léo trong thiết kế tại đây góp phần tạo nên khu nghỉ dưỡng lý tưởng cho những ai tìm kiếm sự an yên, lãng mạn và xa hoa. Á Hiên</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Cồn Én nằm giữa sông Tiền, thuộc xã Tấn Mỹ, rộng hơn 300 ha. Nơi đây ngoài là điểm đến ngắm dòng Tiền Giang, đón gió sông mát dịu, còn là địa chỉ thu hút khách với bộ sưu tập gỗ lũa nội thất độc đáo của khu du lịch trên cồn. Gỗ lũa tức những thân cây khủng, vớt từ đáy sông, bên ngoài bị dòng nước bào mòn, chỉ còn phần lõi bền chắc. Hàng nghìn thân gỗ lũa được người chủ tuyển chọn làm vật liệu chính xây Khu du lịch sinh thái Cồn Én từ tiểu cảnh, nhà đến đài quan sát. Hơn 20 năm trước, ông Nguyễn Văn Nghỉ ở huyện Chợ Mới đã sưu tập rất nhiều gỗ lũa. Ban đầu ông trục vớt chúng để khơi thông dòng chảy, hạn chế tình trạng lưới đánh cá mắc vào thân cây. Lâu dần, ông yêu mến và muốn lưu giữ những thân gỗ trầm thủy này. Ba năm trước, ông Nghỉ dùng số gỗ lũa để xây khu du lịch ven sông Tiền rộng 6 ha. Đặc sắc trong các vật liệu từ gỗ lũa là bức tranh điêu khắc về phong cảnh làng quê Việt Nam xưa dài hơn 24 m, nặng 20 tấn. Bức tranh do nghệ nhân ở Huế thực hiện trong 7 năm, trên khúc gỗ trầm thủy khủng, tùy từng đoạn có chiều cao từ 1,5 - 1,8 m. Cạnh bức tranh là bộ sưu tập hàng trăm chiếc xe máy biển số độc lạ như tứ quý, sảnh tiến tới của nhiều dòng xe nổi tiếng. Dọc các lối đi là những tiểu cảnh làm từ gỗ lũa. Một số được điêu khắc thành các con vật, chim muông. Những cây gỗ lũa kích thước lớn được tận dụng làm đài quan sát cao 26 m, hoặc móng trụ để xây nhà nghỉ, cầu vượt. Khuôn viên cũng được phủ bởi nhiều cây kiểng, dừa cùng dãy nhà sàn ven sông. Tại đây du khách được ngắm hoàng hôn trên sông, tắm sông và thưởng thức ẩm thực miền Tây. Chị Phúc Điền, du khách ở TP HCM, cho biết khá thích với khung cảnh miền Tây yên bình ở Cồn Én. Chị cũng bất ngờ với sự kỳ công của người đã sưu tập hàng nghìn thân gỗ lũa và biến chúng thành điểm tham quan độc đáo. Cồn Én, nằm cách TP HCM 170 km, du khách có thể đến đây từ hướng quốc lộ 30 của tỉnh Đồng Tháp hoặc lên phà Tấn Long vượt sông Tiền từ phía huyện Chợ Mới. Giá vé vào cổng là 80.000 đồng. Ngọc Tài</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Văn phòng mới của MayTrip tại địa chỉ 833 Lê Hồng Phong, quận 10, nhằm mở rộng dịch vụ và nâng cao trải nghiệm khách hàng khu vực phía Nam. Văn phòng mới được kỳ vọng là điểm đến thuận tiện cho khách hàng trong việc tìm hiểu và sử dụng dịch vụ của công ty. Trong ngày khai trương, MayTrip trao tặng nhiều quà tặng và ưu đãi cho khách tham dự. Các voucher gồm: 2 triệu đồng cho khách đăng ký tour Bắc Á trong ba ngày khai trương, 1 triệu đồng cho tour Đông Nam Á trong ba tháng từ ngày khai trương, 500.000 đồng cho dịch vụ tour nội địa trong một năm, 200.000 đồng dịch vụ đặt phòng khách sạn hoặc xe du lịch trong 6 tháng và 100.000 đồng với dịch vụ vé máy bay trong 6 tháng. Buổi lễ khai trương văn phòng tại Sài Gòn còn giới thiệu các chương trìnhtour Nhật Bảndịp Tết Âm lịch như cung đường vàng trải nghiệm trượt tuyết, Hokkaido - miền tuyết trắng. Những chuyến đi này được MayTrip thiết kế kỹ lưỡng, phù hợp với không khí đón xuân cho gia đình và cặp đôi Việt trong dịp Tết Nguyên đán. Năm nay, MayTrip xác định tour Hokkaido là sản phẩm 'đinh' trong dịp Tết Nguyên đán. Hokkaido nằm ở miền Bắc Nhật Bản, nổi tiếng với những đợt tuyết dày và phong cảnh mùa đông đặc trưng. Tour Hokkaido dịp Tết là hành trình lý tưởng để du khách tận hưởng kỳ nghỉ theo cách mới mẻ và ấn tượng trong tuyết trắng. Bên cạnh đó, tour Hokkaido của MayTrip cũng mang đến trải nghiệm suối nước nóng onsen giữa băng tuyết, giúp du khách thư giãn sau những hoạt động trong ngày. Bên cạnh đó, MayTrip cũng cung cấp các tour du lịch khác với lịch khởi hành linh hoạt kéo dài đến hết năm 2025, gồm hành trình ngắm hoa anh đào, hoa mơ, mận và nghỉ lễ 30/4 và 1/5. Các hành trình này dựa trên xu hướng và sở thích của du khách Việt Nam. Theo đại diện công ty, sự kiện khai trương văn phòng mới tại TP HCM đánh dấu bước phát triển mới của MayTrip. Với mục tiêu ưu tiên trải nghiệm khách hàng, đơn vị hy vọng nhận được sự ủng hộ từ khách hàng để trở thành công ty lữ hành hàng đầu, hướng mục tiêu thương hiệu toàn cầu vào năm 2030. Ngoài TP HCM, MayTrip còn có văn phòng tại Hải Phòng và TP Vinh. Các văn phòng này giúp MayTrip dễ dàng tiếp cận và đáp ứng nhu cầu đa dạng của khách hàng. Công ty cam kết đảm bảo chất lượng dịch vụ để mang lại chuyến đi an toàn, trọn vẹn cho khách hàng. Thanh Thư</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ngày 29/10, tại Khu du lịch Sun World Fansipan Legend, Hiệp hội Du lịch tỉnh Lào Cai công bố chương trình kích cầu du lịch lớn nhất năm với chủ đề 'Chạm Sa Pa - Chạm những tầng mây', diễn ra từ 2/11 đến 30/12. Trong thời gian này, 130 doanh nghiệp tại Sa Pa sẽ cung cấp nhiều ưu đãi lên đến 50% và cam kết đảm bảo chất lượng dịch vụ. Theo đó, Công ty Cáp treo Fansipan Sa Pa (Khu du lịch Sun World Fansipan Legend) áp dụng đồng giá vé cáp treo hai chiều Fansipan chỉ còn 550.000 đồng cho du khách Việt Nam. Mức giá này giảm 30% so với giá gốc. Du khách có thể khám phá đỉnh Fansipan, chiêm ngưỡng kiến trúc tâm linh và tham gia các hoạt động văn hóa của 7 dân tộc thiểu số Tây Bắc tại Bản Mây. Nhiều điểm du lịch khác tại Sa Pa cũng miễn phí vé tham quan và cung cấp ưu đãi hấp dẫn. Trong đó, vườn đá Tả Phìn và vườn hồng Mộng Mơ miễn phí vé, Khu du lịch Cát Cát miễn phí trải nghiệm ẩm thực Tây Bắc cùng các hoạt động vẽ sáp ong, xe lanh, dệt vải... với bà con dân bản. Các khách sạn như Chaulong Sapa, Amazing Sapa, Vườn Sa Pa, Arista Sa Pa và Le Bordeaux Sapa áp dụng giảm giá phòng trực tiếp tới 50%. Hotel de la Coupole và Lady Hill Sapa Resort có nhiều ưu đãi về dịch vụ ăn uống, spa. Một số nhà xe như Inter Bus Lines và Eco Sa Pa cũng giảm giá vé xe khứ hồi đến 30%, cung cấp đa dạng hình thức di chuyển từ xe limousine đến xe lớn. Ông Phạm Cao Vỹ, đại diện Hiệp hội Du lịch tỉnh Lào Cai nhấn mạnh sự cần thiết của việc kích cầu du lịch để phục hồi ngành sau ảnh hưởng nặng nề của bão lũ. Ông kêu gọi tất cả doanh nghiệp du lịch trên địa bàn tham gia nhằm tạo sức bật cho du lịch Sa Pa phát triển mạnh mẽ vào giai đoạn cuối năm 2024. Ông Nguyễn Xuân Chiến, Phó chủ tịch Sun Group Vùng Miền Bắc, cho biết trước đây chương trình kích cầu 'Đến Sa Pa - Bay giữa mùa hoa' thành công ngoài mong đợi. 'Lần này, thông qua chính sách ưu đãi sâu, chúng tôi hy vọng thu hút đông đảo du khách đến Sa Pa để khám phá vẻ đẹp độc đáo của mùa mây', ông Chiến nói. Ngoài chính sách ưu đãi sâu, tỉnh Lào Cai và thị xã Sa Pa tổ chức nhiều sự kiện văn hóa đặc sắc nhằm mang đến trải nghiệm độc đáo cho du khách. Các hoạt động bao gồm lễ hội truyền thống, triển lãm nghệ thuật, thể thao và giải trí. Đặc biệt là sự kiện ánh sáng 3D Mapping và lễ hội hoa sen đá lần đầu tiên được tổ chức tại Sun World Fansipan Legend. Sa Pa đang trong mùa mây - thời điểm lý tưởng để vui chơi ngoài trời. Ban tổ chức kỳ vọng chương trình kích cầu sẽ tăng sức hút của Sa Pa và củng cố vị thế là điểm đến hàng đầu miền Bắc. Thanh Thư</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Brisbane nằm phía đông nam bang Queensland, là thành phố lớn thứ ba tại Australia. Do gần đường xích đạo, khí hậu nơi đây ôn hòa, quanh năm nắng ấm. Trung tâm Brisbane không chỉ có những khối bê tông, khu mua sắm, mà còn bao phủ bởi mảng xanh, với 5 công viên và vườn thực vật nổi tiếng. Dưới đây là 5 điểm đến hút du khách ở Brisbane. South Bank Parklands Nằm bên bờ sông Brisbane, South Bank Parklands được ví như 'ốc đảo xanh' giữa lòng thành phố sôi động, nổi bật với rừng mưa nhiệt đới và loạt hoạt động giải trí cho mọi lứa tuổi. Ngay cửa ngõ công viên là thảm cỏ, hàng cây rợp bóng và vườn hoa. Nhiều người dân thường picnic, dã ngoại, vui chơi tại bãi biển nhân tạo Streets Beach, River Quay Green, Rainforest Green hay Liana Lounge. Ngoài ra, Wheel of Brisbane - vòng đu quay cao tới 60 m - là biểu tượng tại South Bank Parklands, dễ dàng ngắm toàn cảnh Brisbane từ trên cao. Roma Street Parkland Nằm cạnh ga xe lửa Roma Street, công viên cùng tên cũng được người dân lẫn du khách gọi là 'ốc đảo xanh mát' giữa Brisbane, ghi dấu với những khu vườn và bãi cỏ rộng lớn. Tại đây, du khách hòa mình vào khu vườn Spectacle - nơi trồng hàng nghìn gốc violets, cẩm chướng, delphiniums và foxgloves. Khí hậu ôn hòa thu hút chim kookaburras, gà lôi, vẹt. Bạn cũng có thể tổ chức tiệc BBQ ngoài trời, cho con khám phá công viên trẻ em. Brisbane City Botanic Gardens Nằm trên trục đường Alice, Brisbane City Botanic Gardens bảo tồn hàng nghìn loài thực vật quý hiếm, nổi bật với vẻ nguyên sơ. Khu vườn này là một trong những điểm đến lý tưởng cho người chuộng nét thanh bình giữa lòng đô thị. Tại đây, du khách có thể khám phá con đường dạo bộ ven sông, chiêm ngưỡng rặng thông Bunya được trồng từ năm 1858. Điểm đến tiếp theo là Bamboo Grove - con đường tre rợp mát, được ví như 'khu rừng xa xôi giữa thành phố hiện đại'. Vườn bách thảo tổ chức sự kiện quanh năm như biểu diễn Riverstage, lễ hội đa văn hóa, trưng bày nghệ thuật cùng hoạt động cộng đồng miễn phí. Trong đó, chợ Riverside Sunday Market hút hàng nghìn du khách nhờ gian hàng thủ công, trái cây tươi và ẩm thực độc đáo. Epicurious Garden Tại Epicurious, du khách có thể khám phá ẩm thực bang Queensland đa dạng, nhất là rau, củ, quả, thảo mộc hữu cơ theo mùa. 14 chuyên viên tình nguyện chăm sóc khu vườn kỹ lưỡng, mong truyền cảm hứng cho người yêu nấu ăn và trồng trọt. 'Tới Epicurious, tôi và bạn bè được hướng dẫn cách chăm sóc rau củ, trái cây, thảo mộc và thưởng thức miễn phí', một du khách viết trên Facebook, nhận hàng trăm nghìn lượt thích. Mount Coot-tha Botanic Gardens Mở cửa đón khách từ năm 1976, Mount Coot-tha Botanic Gardens tọa lạc chân núi Coot-tha, là vườn thực vật nhiệt đới hàng đầu Brisbane, diện tích đến 56 ha. Dạo quanh khu vườn, du khách có thể chiêm ngưỡng hoa xuân, các loài cây nhiệt đới và khu thảo dược. Nơi đây là điểm đến quen thuộc của người yêu thiên nhiên, picnic, mê hoạt động thể chất, với đường chạy bộ thoáng đãng. Để khám phá thành thủ phủ bang Queensland, bạn có thể chọn đường bay thẳng từ TP HCM đến Brisbane của Vietjet, với 9 giờ trên máy bay thân rộng, thoải mái cùng loạt dịch vụ tiện ích, ưu đãi như: bảo hiểm Sky Care miễn phí, chương trình tích điểm SkyJoy, đổi quà từ hơn 250 thương hiệu lớn toàn cầu. Trước đó ngày14-15/9, Vietjet đồng hành lễ hội thả diều Vietjet Redcliffe KiteFest tại Redcliffe, Queensland. Hãng hàng không Việt còn áp dụng nhiều chương trình ưu đãi nhân dịp đón hành khách thứ 200 triệu. Đông Vệ</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Công ty du lịch NhatbanAZ mở bán chùm tour Nhật Bản khởi hành dịp Tết Dương lịch và Âm lịch từ đầu tháng 10. Trong đó, các tour truyền thống đến Osaka, Kyoto và Tokyo được làm mới bằng những hoạt động phù hợp với mùa đông xuân như trượt tuyết tại Fujiten Resort, ngắm tuyết làng cổ Oshino Hakkai và tham gia lễ hội ánh sáng Nabana no sato. NhatbanAZ cũng mở rộng các cung đường mới cho du khách trải nghiệm trong dịp Tết 2025. Cụ thể, tour Hokkaido gồm Asahikawa, Monbetsu và Sapporo với giá 55,9 triệu đồng mỗi khách. Du khách sẽ tham gia câu cá trên băng, đi tàu phá băng và thưởng thức bia hơi tại Sapporo, cùng dịch vụ hàng không 5 sao và lưu trú khách sạn 4 sao quốc tế. Tour thứ hai là chuyến thăm làng cổ Shirakawago, núi Phú Sĩ và Tokyo trong 6 ngày 5 đêm với giá 31,9 triệu đồng mỗi khách. Du khách sẽ được chiêm ngưỡng tuyết trắng tại Shirakawago, một Di sản Văn hóa Thế giới của UNESCO từ năm 1995. Tour cũng gồm tham quan lâu đài Matsumoto - di tích bảo vật quốc gia của Nhật Bản và trải nghiệm trượt tuyết tại Fujiten Snow Resort - top 3 khu trượt tuyết nổi tiếng. Bà Hồ Như Thảo, Giám đốc Điều hành NhatbanAZ Văn phòng TP HCM cho biết sản phẩm mới này nhận được sự quan tâm lớn từ du khách, đặc biệt là những người từng đi Nhật và muốn trở lại với hành trình mới. Khu vực Hokkaido được biết đến với tuyết rơi dày đặc hơn Tokyo hay Osaka, nên lịch khởi hành tour Hokkaido dịp Tết Âm lịch nhận được nhiều đăng ký giữ chỗ. Trong dịp Tết Nguyên đán 2025, NhatbanAZ cung cấp các hành trình từ 5 đến 6 ngày với mức giá cơ bản đến cao cấp, khoảng 31,9 - 55,9 triệu đồng mỗi khách để đáp ứng nhu cầu đa dạng. Giá tour Tết có phần chênh lệch so với ngày thường và tăng so với cùng kỳ năm trước. Do đó, NhatbanAZ chủ động gặp gỡ và làm việc với các đối tác cung cấp dịch vụ, từ đó xây dựng chương trình, đưa ra chính sách ưu đãi tốt nhất cho khách hàng. Với kinh nghiệm hơn 15 năm trong ngành du lịch chuyên thị trường Nhật Bản, NhatbanAZ thuộc danh sách công ty chỉ định nộp visa bởi Đại sứ quán Nhật Bản đề xuất. Đồng thời là đối tác chiến lược của các hãng hàng không, khách sạn và đối tác land tour uy tín tại Nhật Bản. Công ty cũng là nhà tư vấn và tổ chức những chuyến Famtrip kết nối các công ty du lịch Việt Nam tới tham quan xúc tiến đầu tư, hợp tác tại Nhật Bản. Thanh Thư</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Theo bảng xếp hạng 20 quốc gia tốt nhất thế giới năm 2024 (The Best Countries in the World) do tạp chí du lịch Mỹ Condé Nast Traveler công bố vào tháng 10, Việt Nam ở vị trí 15 với 89 điểm. Một điểm đến khác thuộc Đông Nam Á có mặt trong danh sách này là Thái Lan, xếp thứ ba với 92,29 điểm. Đứng đầu top 20 là Nhật Bản với 95,32 điểm. Xếp hạng nằm trong giải thưởng thường niênReaders' Choice Awards của tạp chí Mỹ, dựa trên đánh giá của hơn 575.000 độc giả về các trải nghiệm du lịch ở mỗi quốc gia, xét theo các tiêu chí văn hóa, cảnh quan, dịch vụ du lịch và cơ sở hạ tầng. Độc giả của Condé Nast Traveler nhận xét Việt Nam thu hút du khách nhờ vẻ đẹp mộc mạc và quyến rũ. 'Với lượng khách nước ngoài đang trên đà tăng từ 2019 đến nay, Việt Nam không còn là điểm đến đáng chú ý mà thành điểm đến đáng ghé thăm', biên tập tờ Condé Nast Traveler viết. Theo số liệu từ Tổng cục Thống kê, trong 9 tháng đầu năm, Việt Nam đón hơn 12,7 triệu lượt khách quốc tế, vượt lượng khách cả năm 2023 là 12,6 triệu lượt. Lượng khách quốc tế đến Việt Nam tăng trưởng tích cực 9 tháng đầu năm 2024, với một số thị trường phục hồi hoàn toàn, tăng mạnh so với 2019, theo Cục Du lịch Quốc gia. Cục cũng dự đoán với đà tăng trường như hiện nay, Việt Nam sẽ hoàn thành mục tiêu đón 17-18 triệu lượt khách quốc tế năm 2024. Thái Lan được tạp chí Mỹ nhận xét là quốc gia đa dạng cảnh quan, giao thông thuận tiện với nhiều tàu thuyền, xe buýt đêm và chuyến bay nội địa giá rẻ. Ẩm thực cũng là điểm sáng của xứ chùa Vàng khi có nhiều khu chợ đêm nhộn nhịp, bày bán đặc sản địa phương. 8 tháng đầu năm 2024, Thái Lan đón hơn 20 triệu lượt khách quốc tế, tăng 34% so với cùng kỳ năm trước. Quốc gia này đặt mục tiêu đón ít nhất 36-37 triệu lượt khách nước ngoài trong cả năm nay, kỳ vọng thu về khoảng 3.500 tỷ baht (95,5 tỷ USD). Condé Nast Traveler là tạp chí du lịch nổi tiếng toàn cầu, ra mắt vào năm 1987. Các bảng xếp hạng của Condé Nast Traveler như Readers' Choice Awards được chuyên gia du lịch đánh giá là uy tín vì dựa trên ý kiến từ hàng triệu độc giả quốc tế. Bích Phương(TheoCNTraveller)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
+  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá tính mạch lạc và súc tích."
+}</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -542,8 +667,27 @@
           <t>Theo KTO Việt Nam, 8 tháng năm nay, Hàn Quốc đón 389.000 lượt khách Việt, tăng 27% so với cùng kỳ năm 2023. Số lượng khách Việt Nam đến Hàn Quốc dự kiến tăng mạnh hơn bởi đất nước này đang bước vào mùa lá vàng đẹp nhất năm. Đại diện KTO khẳng định, Việt Nam là thị trường quan trọng với ngành du lịch Hàn Quốc với nhiều sự kiện tổ chức thành công. Cụ thể, trong năm nay, KTO Việt Nam xúc tiến các chương trình quảng bá, phát triển sản phẩm du lịch Hàn Quốc phù hợp với nhu cầu du khách Việt. Kết quả, nhiều sản phẩm du lịch mới được ra mắt thị trường trong nước như: tour du lịch Hàn Quốc kết hợp giải chạy Marathon tại Gyeongju và Jeju, tour trải nghiệm Esports, tour lễ hội đèn lồng truyền thống Yeondeunghoe hay tour đạp xe đạp đường dài khám phá Hàn Quốc... Chương trình Năm du lịch Hàn Quốc 2023-2024 (Visit Korea Year 2023-2024) do Tổng cục du lịch Hàn Quốc (KTO) triển khai cũng mang đến những hoạt động mới mẻ, quảng bá du lịch Hàn Quốc đến cộng đồng quốc tế. Bên cạnh đó, nhằm mang đến những trải nghiệm chân thực và đậm chất bản địa, KTO tổ chức nhiều famtour. Nổi bật là famtour trải nghiệm Esports cùng các KOL hàng đầu làng thể thao điện tử như: SofM, reviewer Duy Thẩm, Hải Triều, streamer Hà Tiều Phu, BLV Esports nổi tiếng Văn Tùng, Hoàng Luân, kết hợp Box Esports. Làn sóng văn hóa Hallyu cũng được lồng ghép vào sản phẩm du lịch, khi hàng loạt tên tuổi lớn đến Việt Nam trong khuôn khổ sự kiện Korea Travel Festa, tổ chức tháng 5 vừa qua. Mới nhất, KTO Việt Nam có mặt tại Hội chợ Du lịch Quốc tế (ITE) TP HCM, mang theo không gian đặc trưng Hàn Quốc cùng nhiều trải nghiệm mới mẻ, độc đáo. Nắm bắt nhu cầu du lịch Hàn Quốc tăng cao trong mùa cuối năm của du khách Việt, KTO Việt Nam tiếp tục đẩy mạnh các chương trình ưu đãi đặc biệt. Cùng các đối tác, công ty du lịch hàng đầu Việt Nam, KTO góp phần phát triển nhiều tuyến điểm mới trong hành trình du lịch Hàn Quốc, mang đến đa dạng lựa chọn và nhiều trải nghiệm cho khách hàng. Hồi tháng 5, KTO Việt Nam ký kết thỏa thuận hợp tác cùng Tập đoàn Vingroup, nhằm thúc đẩy hơn nữa sự giao lưu, trao đổi du lịch giữa hai nước. Theo đó, KTO triển khai chiến dịch hỗ trợ dành riêng cho khách hàng thuộc hệ sinh thái Vingroup khi mua tour du lịch Hàn Quốc từ tháng 10 đến tháng 12 Cụ thể, chủ sở hữu xe Vinfast, cư dân Vinhomes, nhân viên Vingroup) và hội viên Vinclub (gọi chung là Vintizen) sẽ nhận được mức giá ưu đãi đặc biệt từ các công ty du lịch và KTO Việt Nam. Bên cạnh mức giá ưu đãi từ các công ty du lịch, Vintizen có cơ hội áp dụng đồng thời voucher trị giá một triệu đồng mỗi khách hàng, mua tối đa 5 tour du lịch Hàn Quốc để nhận voucher lên đến 5 triệu đồng từ KTO Việt Nam, trong thời gian 1-10/10. Ngoài thời gian trên, du khách mua tour tại các đối tác du lịch sẽ nhận được nhiều phần quà Hàn Quốc từ KTO Việt Nam. Thanh Thư</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Hàn Quốc đón 389.000 lượt khách Việt Nam tăng 27% nhờ mùa lá vàng đẹp nhất năm và chương trình quảng bá du lịch mới, trong đó Vintizen hưởng ưu đãi giảm giá tour từ tháng 10 đến tháng 12 với voucher trị giá một triệu đồng mỗi khách hàng.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>{
+  "id": 9,
+  "style": "news_brief",
+  "article": "Theo KTO Việt Nam, 8 tháng năm nay, Hàn Quốc đón 389.000 lượt khách Việt, tăng 27% so với cùng kỳ năm 2023. Số lượng khách Việt Nam đến Hàn Quốc dự kiến tăng mạnh hơn bởi đất nước này đang bước vào mùa lá vàng đẹp nhất năm. Đại diện KTO khẳng định, Việt Nam là thị trường quan trọng với ngành du lịch Hàn Quốc với nhiều sự kiện tổ chức thành công. Cụ thể, trong năm nay, KTO Việt Nam xúc tiến các chương trình quảng bá, phát triển sản phẩm du lịch Hàn Quốc phù hợp với nhu cầu du khách Việt. Kết quả, nhiều sản phẩm du lịch mới được ra mắt thị trường trong nước như: tour du lịch Hàn Quốc kết hợp giải chạy Marathon tại Gyeongju và Jeju, tour trải nghiệm Esports, tour lễ hội đèn lồng truyền thống Yeondeunghoe hay tour đạp xe đạp đường dài khám phá Hàn Quốc... Chương trình Năm du lịch Hàn Quốc 2023-2024 (Visit Korea Year 2023-2024) do Tổng cục du lịch Hàn Quốc (KTO) triển khai cũng mang đến những hoạt động mới mẻ, quảng bá du lịch Hàn Quốc đến cộng đồng quốc tế. Bên cạnh đó, nhằm mang đến những trải nghiệm chân thực và đậm chất bản địa, KTO tổ chức nhiều famtour. Nổi bật là famtour trải nghiệm Esports cùng các KOL hàng đầu làng thể thao điện tử như: SofM, reviewer Duy Thẩm, Hải Triều, streamer Hà Tiều Phu, BLV Esports nổi tiếng Văn Tùng, Hoàng Luân, kết hợp Box Esports. Làn sóng văn hóa Hallyu cũng được lồng ghép vào sản phẩm du lịch, khi hàng loạt tên tuổi lớn đến Việt Nam trong khuôn khổ sự kiện Korea Travel Festa, tổ chức tháng 5 vừa qua. Mới nhất, KTO Việt Nam có mặt tại Hội chợ Du lịch Quốc tế (ITE) TP HCM, mang theo không gian đặc trưng Hàn Quốc cùng nhiều trải nghiệm mới mẻ, độc đáo. Nắm bắt nhu cầu du lịch Hàn Quốc tăng cao trong mùa cuối năm của du khách Việt, KTO Việt Nam tiếp tục đẩy mạnh các chương trình ưu đãi đặc biệt. Cùng các đối tác, công ty du lịch hàng đầu Việt Nam, KTO góp phần phát triển nhiều tuyến điểm mới trong hành trình du lịch Hàn Quốc, mang đến đa dạng lựa chọn và nhiều trải nghiệm cho khách hàng. Hồi tháng 5, KTO Việt Nam ký kết thỏa thuận hợp tác cùng Tập đoàn Vingroup, nhằm thúc đẩy hơn nữa sự giao lưu, trao đổi du lịch giữa hai nước. Theo đó, KTO triển khai chiến dịch hỗ trợ dành riêng cho khách hàng thuộc hệ sinh thái Vingroup khi mua tour du lịch Hàn Quốc từ tháng 10 đến tháng 12 Cụ thể, chủ sở hữu xe Vinfast, cư dân Vinhomes, nhân viên Vingroup) và hội viên Vinclub (gọi chung là Vintizen) sẽ nhận được mức giá ưu đãi đặc biệt từ các công ty du lịch và KTO Việt Nam. Bên cạnh mức giá ưu đãi từ các công ty du lịch, Vintizen có cơ hội áp dụng đồng thời voucher trị giá một triệu đồng mỗi khách hàng, mua tối đa 5 tour du lịch Hàn Quốc để nhận voucher lên đến 5 triệu đồng từ KTO Việt Nam, trong thời gian 1-10/10. Ngoài thời gian trên, du khách mua tour tại các đối tác du lịch sẽ nhận được nhiều phần quà Hàn Quốc từ KTO Việt Nam. Thanh Thư",
+  "summary": "Hàn Quốc đón 389.000 lượt khách Việt Nam tăng 27% nhờ mùa lá vàng đẹp nhất năm và chương trình quảng bá du lịch mới, trong đó Vintizen hưởng ưu đãi giảm giá tour từ tháng 10 đến tháng 12 với voucher trị giá một triệu đồng mỗi khách hàng.",
+  "faithfulness_score": 0.8,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng có thể thiếu chính xác khi không đề cập đầy đủ đến các chương trình quảng bá du lịch và sự kiện cụ thể",
+  "relevance_score": 0.7,
+  "relevance_reason": "Bản tóm tắt bao gồm một số ý chính nhưng bỏ sót thông tin quan trọng về các sản phẩm du lịch mới và chương trình Năm du lịch Hàn Quốc 2023-2024",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, tuy nhiên có thể rút gọn một số chi tiết để tăng tính súc tích"
+}</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -551,8 +695,27 @@
           <t>Diễn đàn năm nay là sự kiện trọng điểm do UBND tỉnh Kiên Giang phối hợp Bộ Nông nghiệp và Phát triển nông thôn tổ chức. Công ty Cổ phần Truyền Thông Vương Hậu (TP HCM) là đơn vị phụ trách tổ chức. Với chủ đề 'Liên kết cùng phát triển - Kiên Giang 2024', diễn đàn hướng đến tăng cường hợp tác, liên kết giữa các tỉnh, thành phố trong vùng Đồng bằng sông Cửu Long với các Bộ, ngành Trung ương, các địa phương khác trên cả nước. Từ đó, các bên có thêm cơ sở đẩy mạnh, phát huy tiềm năng về sản phẩm OCOP của vùng. Đến nay, đã có trên 35 tỉnh, thành phố đăng ký tham gia diễn đàn cùng hơn 300 nhà đầu tư đến tìm hiểu cơ hội, xúc tiến hợp tác kinh doanh. Diễn đàn dự kiến thu hút khoảng 50.000-100.000 khách tham quan suốt thời gian diễn ra. Hơn 320 gian hàng từ các tỉnh ĐBSCL và cả nước sẽ cùng trưng bày, giới thiệu các sản phẩm OCOP tiêu biểu, công nghiệp nông thôn, đặc sản địa phương. Ngoài chương trình chính, sự kiện còn bao gồm chuỗi hoạt động khác như: triển lãm sản phẩm OCOP; hội thi 'Sản phẩm OCOP tiêu biểu ĐBSCL 2024'; các hội nghị, hội thảo, ký kết biên bản hợp tác... Đặc biệt, khách tham dự còn được tìm hiểu quy trình sản xuất nước mắm truyền thống Phú Quốc, một trong những đặc sản nổi tiếng của Kiên Giang. Buổi tối, diễn dàn có các chương trình ca nhạc với sự góp mặt của các ca sĩ, nghệ sĩ nổi tiếng. Diễn đàn kết nối sản phẩm OCOP là sự kiện thường niên do Bộ Nông nghiệp và Phát triển nông thôn phối hợp UBND các tỉnh, thành phố vùng Đồng bằng sông Cửu Long tổ chức quy mô cấp vùng. Đây vừa là nơi giao lưu, kết nối kinh doanh, vừa là cơ hội để các sản phẩm này vươn ra thế giới, góp phần phát triển kinh tế nông nghiệp, xây dựng nông thôn mới bền vững. Á Hiên</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Diễn đàn năm nay là sự kiện trọng điểm do UBND tỉnh Kiên Giang phối hợp với Bộ Nông nghiệp và Phát triển nông thôn tổ chức. Công ty Cổ phần Truyền Thông Vương Hậu (TP HCM) phụ trách việc tổ chức. Chủ đề của diễn đàn là 'Liên kết cùng phát triển - Kiên Giang 2024', hướng đến tăng cường hợp tác giữa các tỉnh, thành phố trong vùng Đồng bằng sông Cửu Long với Bộ ngành Trung ương và địa phương khác trên cả nước. Diễn đàn đã thu hút hơn 35 tỉnh/thành phố đăng ký tham gia cùng gần 300 nhà đầu tư tìm hiểu cơ hội xúc tiến hợp tác kinh doanh, dự kiến sẽ có khoảng 50-100 nghìn khách tham quan và trưng bày hơn 320 gian hàng từ các tỉnh ĐBSCL và cả nước. Ngoài chương trình chính như triển lãm sản phẩm OCOP, hội thi 'Sản phẩm OCOP tiêu biểu ĐBSCL 2024', diễn đàn còn có chuỗi hoạt động khác gồm: ký kết biên bản hợp tác, ca nhạc với sự góp mặt của các nghệ sĩ nổi tiếng. Đây là sự kiện thường niên do Bộ Nông nghiệp và Phát triển nông thôn phối hợp UBND các tỉnh/thành phố vùng Đồng bằng sông Cửu Long tổ chức, vừa giúp giao lưu kinh doanh vừa tạo cơ hội cho sản phẩm OCOP vươn ra thế giới.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>{
+  "id": 10,
+  "style": "news_brief",
+  "article": "Diễn đàn năm nay là sự kiện trọng điểm do UBND tỉnh Kiên Giang phối hợp Bộ Nông nghiệp và Phát triển nông thôn tổ chức. Công ty Cổ phần Truyền Thông Vương Hậu (TP HCM) là đơn vị phụ trách tổ chức. Với chủ đề 'Liên kết cùng phát triển - Kiên Giang 2024', diễn đàn hướng đến tăng cường hợp tác, liên kết giữa các tỉnh, thành phố trong vùng Đồng bằng sông Cửu Long với các Bộ, ngành Trung ương, các địa phương khác trên cả nước. Từ đó, các bên có thêm cơ sở đẩy mạnh, phát huy tiềm năng về sản phẩm OCOP của vùng. Đến nay, đã có trên 35 tỉnh, thành phố đăng ký tham gia diễn đàn cùng hơn 300 nhà đầu tư đến tìm hiểu cơ hội, xúc tiến hợp tác kinh doanh. Diễn đàn dự kiến thu hút khoảng 50.000-100.000 khách tham quan suốt thời gian diễn ra. Hơn 320 gian hàng từ các tỉnh ĐBSCL và cả nước sẽ cùng trưng bày, giới thiệu các sản phẩm OCOP tiêu biểu, công nghiệp nông thôn, đặc sản địa phương. Ngoài chương trình chính, sự kiện còn bao gồm chuỗi hoạt động khác như: triển lãm sản phẩm OCOP; hội thi 'Sản phẩm OCOP tiêu biểu ĐBSCL 2024'; các hội nghị, hội thảo, ký kết biên bản hợp tác... Đặc biệt, khách tham dự còn được tìm hiểu quy trình sản xuất nước mắm truyền thống Phú Quốc, một trong những đặc sản nổi tiếng của Kiên Giang. Buổi tối, diễn dàn có các chương trình ca nhạc với sự góp mặt của các ca sĩ, nghệ sĩ nổi tiếng. Diễn đàn kết nối sản phẩm OCOP là sự kiện thường niên do Bộ Nông nghiệp và Phát triển nông thôn phối hợp UBND các tỉnh, thành phố vùng Đồng bằng sông Cửu Long tổ chức quy mô cấp vùng. Đây vừa là nơi giao lưu, kết nối kinh doanh, vừa là cơ hội để các sản phẩm này vươn ra thế giới, góp phần phát triển kinh tế nông nghiệp, xây dựng nông thôn mới bền vững. Á Hiên",
+  "summary": "Diễn đàn năm nay là sự kiện trọng điểm do UBND tỉnh Kiên Giang phối hợp với Bộ Nông nghiệp và Phát triển nông thôn tổ chức. Công ty Cổ phần Truyền Thông Vương Hậu (TP HCM) phụ trách việc tổ chức. Chủ đề của diễn đàn là 'Liên kết cùng phát triển - Kiên Giang 2024', hướng đến tăng cường hợp tác giữa các tỉnh, thành phố trong vùng Đồng bằng sông Cửu Long với Bộ ngành Trung ương và địa phương khác trên cả nước. Diễn đàn đã thu hút hơn 35 tỉnh/thành phố đăng ký tham gia cùng gần 300 nhà đầu tư tìm hiểu cơ hội xúc tiến hợp tác kinh doanh, dự kiến sẽ có khoảng 50-100 nghìn khách tham quan và trưng bày hơn 320 gian hàng từ các tỉnh ĐBSCL và cả nước. Ngoài chương trình chính như triển lãm sản phẩm OCOP, hội thi 'Sản phẩm OCOP tiêu biểu ĐBSCL 2024', diễn đàn còn có chuỗi hoạt động khác gồm: ký kết biên bản hợp tác, ca nhạc với sự góp mặt của các nghệ sĩ nổi tiếng. Đây là sự kiện thường niên do Bộ Nông nghiệp và Phát triển nông thôn phối hợp UBND các tỉnh/thành phố vùng Đồng bằng sông Cửu Long tổ chức, vừa giúp giao lưu kinh doanh vừa tạo cơ hội cho sản phẩm OCOP vươn ra thế giới.",
+  "faithfulness_score": 0.9,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, nhưng có một số chi tiết được tóm tắt không đầy đủ như việc khách tham dự có thể tìm hiểu quy trình sản xuất nước mắm truyền thống Phú Quốc",
+  "relevance_score": 0.8,
+  "relevance_reason": "Bản tóm tắt bao hàm đủ các ý chính quan trọng, nhưng có thể thêm thông tin về mục tiêu của diễn đàn và ý nghĩa của việc tăng cường hợp tác giữa các tỉnh, thành phố",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, nhưng có thể rút gọn một số câu để tăng tính súc tích"
+}</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -560,8 +723,27 @@
           <t>Bên lề đường khu vực Chiêm Mai, nơi có nhiều xưởng làm gốm, các mặt hàng bị ngâm nước vẫn còn bùn đất bám lại. Những sản phẩm còn sử dụng được người dân mang ra phơi nắng. Bên lề đường khu vực Chiêm Mai, nơi có nhiều xưởng làm gốm, các mặt hàng bị ngâm nước vẫn còn bùn đất bám lại. Những sản phẩm còn sử dụng được người dân mang ra phơi nắng. Trong chợ gốm, nhiều cửa hàng quây bạt, chưa mở cửa lại. 'Nhiều chủ hàng chưa mở lại do phải dọn dẹp nhà cửa bị ngập trước đó, chưa có thời gian dọn cửa hàng', chị Tuyết, chủ một cửa hàng, nói. Trong chợ gốm, nhiều cửa hàng quây bạt, chưa mở cửa lại. 'Nhiều chủ hàng chưa mở lại do phải dọn dẹp nhà cửa bị ngập trước đó, chưa có thời gian dọn cửa hàng', chị Tuyết, chủ một cửa hàng, nói. Chị Lan, chủ một cửa hàng trong chợ, cho biết nhà chị không bị thiệt hại nặng nên dọn hàng ra sớm để đón khách. 'Ngày thường ít khách lui tới nhưng đông vào dịp cuối tuần', chị Lan nói. Chị Lan, chủ một cửa hàng trong chợ, cho biết nhà chị không bị thiệt hại nặng nên dọn hàng ra sớm để đón khách. 'Ngày thường ít khách lui tới nhưng đông vào dịp cuối tuần', chị Lan nói. Cửa hàng nặn gốm của chị Lan đã sẵn sàng đón khách hàng đến trải nghiệm. Cửa hàng nặn gốm của chị Lan đã sẵn sàng đón khách hàng đến trải nghiệm. Các gian hàng mở lại với lác đác du khách tới tham quan, mua sắm - trái với khung cảnh tấp nập mỗi dịp lễ, Tết khi mặt hàng gốm sứ được nhiều người tìm mua. Các gian hàng mở lại với lác đác du khách tới tham quan, mua sắm - trái với khung cảnh tấp nập mỗi dịp lễ, Tết khi mặt hàng gốm sứ được nhiều người tìm mua. Bảo tàng gốm Bát Tràng nằm gần ngoài đê, trước khi vào làng gốm, cũng đã mở cửa sẵn sàng đón khách. Bảo tàng được xây dựng từ năm 2018 với kinh phí 150 tỷ đồng, là 'trung tâm tinh hoa làng nghề Việt'. Bảo tàng gốm Bát Tràng nằm gần ngoài đê, trước khi vào làng gốm, cũng đã mở cửa sẵn sàng đón khách. Bảo tàng được xây dựng từ năm 2018 với kinh phí 150 tỷ đồng, là 'trung tâm tinh hoa làng nghề Việt'. Bên trong bảo tàng có thiết kế độc đáo, nhiều tầng với các chuyên đề khác nhau về lịch sử hình thành, phát triển cũng như các loại hình gốm tại Bát Tràng. 'Đến làng gốm để có trải nghiệm thú vị, thay đổi không khí và tìm hiểu về gốm truyền thống', Phạm Hoàng Hiệu, Thanh Xuân, Hà Nội, cho biết khi đến đây sau những ngày phải ở nhà vì mưa lụt. Bên trong bảo tàng có thiết kế độc đáo, nhiều tầng với các chuyên đề khác nhau về lịch sử hình thành, phát triển cũng như các loại hình gốm tại Bát Tràng. 'Đến làng gốm để có trải nghiệm thú vị, thay đổi không khí và tìm hiểu về gốm truyền thống', Phạm Hoàng Hiệu, Thanh Xuân, Hà Nội, cho biết khi đến đây sau những ngày phải ở nhà vì mưa lụt. Đình làng Bát Tràng hơn 300 tuổi không bị ảnh hưởng sau trận lụt. Đình được coi là 'báu vật đi cùng năm tháng' ở làng, hiện lưu giữ hơn 50 đạo sắc phong. Đình Bát Tràng được Bộ Văn hóa Thể thao và Du lịch cấp bằng Di tích văn hóa kiến trúc nghệ thuật năm 2005. Đình làng Bát Tràng hơn 300 tuổi không bị ảnh hưởng sau trận lụt. Đình được coi là 'báu vật đi cùng năm tháng' ở làng, hiện lưu giữ hơn 50 đạo sắc phong. Đình Bát Tràng được Bộ Văn hóa Thể thao và Du lịch cấp bằng Di tích văn hóa kiến trúc nghệ thuật năm 2005. Hoàng Giang</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LỖI: 'NoneType' object is not iterable</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>{
+  "id": 11,
+  "style": "news_brief",
+  "article": "Bên lề đường khu vực Chiêm Mai, nơi có nhiều xưởng làm gốm, các mặt hàng bị ngâm nước vẫn còn bùn đất bám lại. Những sản phẩm còn sử dụng được người dân mang ra phơi nắng. Bên lề đường khu vực Chiêm Mai, nơi có nhiều xưởng làm gốm, các mặt hàng bị ngâm nước vẫn còn bùn đất bám lại. Những sản phẩm còn sử dụng được người dân mang ra phơi nắng. Trong chợ gốm, nhiều cửa hàng quây bạt, chưa mở cửa lại. 'Nhiều chủ hàng chưa mở lại do phải dọn dẹp nhà cửa bị ngập trước đó, chưa có thời gian dọn cửa hàng', chị Tuyết, chủ một cửa hàng, nói. Trong chợ gốm, nhiều cửa hàng quây bạt, chưa mở cửa lại. 'Nhiều chủ hàng chưa mở lại do phải dọn dẹp nhà cửa bị ngập trước đó, chưa có thời gian dọn cửa hàng', chị Tuyết, chủ một cửa hàng, nói. Chị Lan, chủ một cửa hàng trong chợ, cho biết nhà chị không bị thiệt hại nặng nên dọn hàng ra sớm để đón khách. 'Ngày thường ít khách lui tới nhưng đông vào dịp cuối tuần', chị Lan nói. Chị Lan, chủ một cửa hàng trong chợ, cho biết nhà chị không bị thiệt hại nặng nên dọn hàng ra sớm để đón khách. 'Ngày thường ít khách lui tới nhưng đông vào dịp cuối tuần', chị Lan nói. Cửa hàng nặn gốm của chị Lan đã sẵn sàng đón khách hàng đến trải nghiệm. Cửa hàng nặn gốm của chị Lan đã sẵn sàng đón khách hàng đến trải nghiệm. Các gian hàng mở lại với lác đác du khách tới tham quan, mua sắm - trái với khung cảnh tấp nập mỗi dịp lễ, Tết khi mặt hàng gốm sứ được nhiều người tìm mua. Các gian hàng mở lại với lác đác du khách tới tham quan, mua sắm - trái với khung cảnh tấp nập mỗi dịp lễ, Tết khi mặt hàng gốm sứ được nhiều người tìm mua. Bảo tàng gốm Bát Tràng nằm gần ngoài đê, trước khi vào làng gốm, cũng đã mở cửa sẵn sàng đón khách. Bảo tàng được xây dựng từ năm 2018 với kinh phí 150 tỷ đồng, là 'trung tâm tinh hoa làng nghề Việt'. Bảo tàng gốm Bát Tràng nằm gần ngoài đê, trước khi vào làng gốm, cũng đã mở cửa sẵn sàng đón khách. Bảo tàng được xây dựng từ năm 2018 với kinh phí 150 tỷ đồng, là 'trung tâm tinh hoa làng nghề Việt'. Bên trong bảo tàng có thiết kế độc đáo, nhiều tầng với các chuyên đề khác nhau về lịch sử hình thành, phát triển cũng như các loại hình gốm tại Bát Tràng. 'Đến làng gốm để có trải nghiệm thú vị, thay đổi không khí và tìm hiểu về gốm truyền thống', Phạm Hoàng Hiệu, Thanh Xuân, Hà Nội, cho biết khi đến đây sau những ngày phải ở nhà vì mưa lụt. Bên trong bảo tàng có thiết kế độc đáo, nhiều tầng với các chuyên đề khác nhau về lịch sử hình thành, phát triển cũng như các loại hình gốm tại Bát Tràng. 'Đến làng gốm để có trải nghiệm thú vị, thay đổi không khí và tìm hiểu về gốm truyền thống', Phạm Hoàng Hiệu, Thanh Xuân, Hà Nội, cho biết khi đến đây sau những ngày phải ở nhà vì mưa lụt. Đình làng Bát Tràng hơn 300 tuổi không bị ảnh hưởng sau trận lụt. Đình được coi là 'báu vật đi cùng năm tháng' ở làng, hiện lưu giữ hơn 50 đạo sắc phong. Đình Bát Tràng được Bộ Văn hóa Thể thao và Du lịch cấp bằng Di tích văn hóa kiến trúc nghệ thuật năm 2005. Đình làng Bát Tràng hơn 300 tuổi không bị ảnh hưởng sau trận lụt. Đình được coi là 'báu vật đi cùng năm tháng' ở làng, hiện lưu giữ hơn 50 đạo sắc phong. Đình Bát Tràng được Bộ Văn hóa Thể thao và Du lịch cấp bằng Di tích văn hóa kiến trúc nghệ thuật năm 2005. Hoàng Giang",
+  "summary": "LỖI: 'NoneType' object is not iterable",
+  "faithfulness_score": 0.0,
+  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin nào về văn bản gốc, không phản ánh nội dung của văn bản.",
+  "relevance_score": 0.0,
+  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không đề cập đến các sự kiện, tình huống hoặc thông điệp chính.",
+  "coherence_conciseness_score": 0.0,
+  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá về tính mạch lạc và súc tích."
+}</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -569,8 +751,27 @@
           <t>Bếp trưởng Christian Le Squer nổi tiếng với 22 năm liên tiếp đạt 3 sao Michelin, hiện đảm nhiệm vai trò bếp trưởng tại La Maison 1888. Nhà hàng là điểm đến ẩm thực Pháp cao cấp, nằm ngay trong khuôn viên resort InterContinental Danang Sun Peninsula Resort. Tháng 7 vừa qua đánh dấu cột mốc quan trọng khi La Maison 1888 gia nhập 'bản đồ' Michelin Guide với ngôi sao đầu tiên. Với sự điều hành của bếp trưởng Christian Le Squer, thực khách sẽ được trải nghiệm ẩm thực Pháp cao cấp giao hòa giữa nghệ thuật và thẩm mỹ cao cấp, mang đậm dấu ấn cá nhân của ông. Ông Seif Hamdy, Tổng giám đốc khu nghỉ dưỡng cho biết sự góp mặt của bếp trưởng Christian tại InterContinental Danang là bước tiến quan trọng. Sự sáng tạo trong ẩm thực cùng khả năng của ông là điều đã được chứng minh bằng 22 năm liên tục được trao tặng ba sao Michelin. Christian Le Squer còn từng đạt danh hiệu 'Bếp trưởng của năm' do Gault &amp; Millau trao tặng năm 2023. 'Christian Le Squer sẽ mang đến làn gió mới cùng tầm nhìn sáng tạo, góp phần nâng tầm trải nghiệm ẩm thực cho thực khách tại La Maison 1888 với phong cách 'haute couture' đặc trưng do chính ông tạo ra', ông Seif Hamdy nói. Sinh ra và lớn lên bên bờ biển Brittany (Pháp), bếp trưởng Christian có nhiều trải nghiệm tuổi thơ gắn liền với ẩm thực. Những ký ức thuở nhỏ gieo cho ông đam mê ẩm thực sâu sắc và dẫn lối ông đến kinh đô ánh sáng và thời trang Paris. Đến năm 34 tuổi, ông được trao sao Michelin đầu tiên tại nhà hàng Café de la Paix. Thành công này đã thôi thúc ông tiếp tục hành trình chinh phục những đỉnh cao ẩm thực kế tiếp. Sau đó, ông gia nhập nhà hàng Pavillon Ledoyen năm 1999, giúp nơi này giành được ba sao Michelin không lâu sau đó. Thành tích này được ông Christian lặp lại tại Le Cinq, nhà hàng Pháp biểu tượng tại khách sạn Four Seasons Hotel George V ở Paris. Bếp trưởng Christian ví von phong cách ẩm thực độc đáo của mình như những tác phẩm thời trang nghệ thuật cao cấp 'haute couture' trên bàn ăn. Ông cho biết mỗi món đều mang dấu ấn riêng biệt, sở hữu hương vị và diện mạo thanh lịch như một bộ trang phục sang trọng hay một chai nước hoa độc bản được giới thiệu tại Tuần lễ Thời trang Paris. Sau nhiều chuyến ghé thăm Việt Nam, đặc biệt là Đà Nẵng, ông hiểu hơn về nhu cầu của thực khách nơi đây. Nhiều người ông gặp cho biết họ tìm kiếm sự kết hợp hài hòa giữa truyền thống và hiện đại trong ẩm thực Pháp. Việc khám phá các hương vị, nguyên liệu, văn hóa ẩm thực đặc sắc của Việt Nam đã trở thành nguồn cảm hứng để ông phác họa nên bức tranh ẩm thực riêng cho La Maison 1888. 'Tôi rất mong chờ được cùng làm việc với đội ngũ tài năng tại La Maison 1888, đặc biệt là Bếp trưởng Florian Stein', Christian nói. Nằm trong một dinh thự theo phong cách Đông Dương thanh lịch do Bill Bensley thiết kế, La Maison 1888 là một trong những điểm đến ẩm thực quốc tế đáng cân nhắc tại Đông Nam Á. Nhà hàng sở hữu hầm rượu vang với bộ sưu tập phong phú cùng tầm nhìn đẹp hướng biển. Nơi đây chinh phục thực khách bằng ẩm thực cao cấp với chất lượng được Michelin công nhận cùng không gian sang trọng đậm chất Pháp. Sắp tới, bếp trưởng Christian hứa hẹn mang đến nhiều bất ngờ thú vị, góp phần nâng tầm trải nghiệm ẩm thực của thực khách tại đây. Á Hiên</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>LỖI: 'NoneType' object is not iterable</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>{
+  "id": 12,
+  "style": "news_brief",
+  "article": "Bếp trưởng Christian Le Squer nổi tiếng với 22 năm liên tiếp đạt 3 sao Michelin, hiện đảm nhiệm vai trò bếp trưởng tại La Maison 1888. Nhà hàng là điểm đến ẩm thực Pháp cao cấp, nằm ngay trong khuôn viên resort InterContinental Danang Sun Peninsula Resort. Tháng 7 vừa qua đánh dấu cột mốc quan trọng khi La Maison 1888 gia nhập 'bản đồ' Michelin Guide với ngôi sao đầu tiên. Với sự điều hành của bếp trưởng Christian Le Squer, thực khách sẽ được trải nghiệm ẩm thực Pháp cao cấp giao hòa giữa nghệ thuật và thẩm mỹ cao cấp, mang đậm dấu ấn cá nhân của ông. Ông Seif Hamdy, Tổng giám đốc khu nghỉ dưỡng cho biết sự góp mặt của bếp trưởng Christian tại InterContinental Danang là bước tiến quan trọng. Sự sáng tạo trong ẩm thực cùng khả năng của ông là điều đã được chứng minh bằng 22 năm liên tục được trao tặng ba sao Michelin. Christian Le Squer còn từng đạt danh hiệu 'Bếp trưởng của năm' do Gault &amp; Millau trao tặng năm 2023. 'Christian Le Squer sẽ mang đến làn gió mới cùng tầm nhìn sáng tạo, góp phần nâng tầm trải nghiệm ẩm thực cho thực khách tại La Maison 1888 với phong cách 'haute couture' đặc trưng do chính ông tạo ra', ông Seif Hamdy nói. Sinh ra và lớn lên bên bờ biển Brittany (Pháp), bếp trưởng Christian có nhiều trải nghiệm tuổi thơ gắn liền với ẩm thực. Những ký ức thuở nhỏ gieo cho ông đam mê ẩm thực sâu sắc và dẫn lối ông đến kinh đô ánh sáng và thời trang Paris. Đến năm 34 tuổi, ông được trao sao Michelin đầu tiên tại nhà hàng Café de la Paix. Thành công này đã thôi thúc ông tiếp tục hành trình chinh phục những đỉnh cao ẩm thực kế tiếp. Sau đó, ông gia nhập nhà hàng Pavillon Ledoyen năm 1999, giúp nơi này giành được ba sao Michelin không lâu sau đó. Thành tích này được ông Christian lặp lại tại Le Cinq, nhà hàng Pháp biểu tượng tại khách sạn Four Seasons Hotel George V ở Paris. Bếp trưởng Christian ví von phong cách ẩm thực độc đáo của mình như những tác phẩm thời trang nghệ thuật cao cấp 'haute couture' trên bàn ăn. Ông cho biết mỗi món đều mang dấu ấn riêng biệt, sở hữu hương vị và diện mạo thanh lịch như một bộ trang phục sang trọng hay một chai nước hoa độc bản được giới thiệu tại Tuần lễ Thời trang Paris. Sau nhiều chuyến ghé thăm Việt Nam, đặc biệt là Đà Nẵng, ông hiểu hơn về nhu cầu của thực khách nơi đây. Nhiều người ông gặp cho biết họ tìm kiếm sự kết hợp hài hòa giữa truyền thống và hiện đại trong ẩm thực Pháp. Việc khám phá các hương vị, nguyên liệu, văn hóa ẩm thực đặc sắc của Việt Nam đã trở thành nguồn cảm hứng để ông phác họa nên bức tranh ẩm thực riêng cho La Maison 1888. 'Tôi rất mong chờ được cùng làm việc với đội ngũ tài năng tại La Maison 1888, đặc biệt là Bếp trưởng Florian Stein', Christian nói. Nằm trong một dinh thự theo phong cách Đông Dương thanh lịch do Bill Bensley thiết kế, La Maison 1888 là một trong những điểm đến ẩm thực quốc tế đáng cân nhắc tại Đông Nam Á. Nhà hàng sở hữu hầm rượu vang với bộ sưu tập phong phú cùng tầm nhìn đẹp hướng biển. Nơi đây chinh phục thực khách bằng ẩm thực cao cấp với chất lượng được Michelin công nhận cùng không gian sang trọng đậm chất Pháp. Sắp tới, bếp trưởng Christian hứa hẹn mang đến nhiều bất ngờ thú vị, góp phần nâng tầm trải nghiệm ẩm thực của thực khách tại đây. Á Hiên",
+  "summary": "LỖI: 'NoneType' object is not iterable",
+  "faithfulness_score": 0.0,
+  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin nào về văn bản gốc, không có nội dung để đánh giá tính trung thực.",
+  "relevance_score": 0.0,
+  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không có nội dung để đánh giá tính bao quát.",
+  "coherence_conciseness_score": 0.0,
+  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá tính mạch lạc và súc tích."
+}</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -578,8 +779,27 @@
           <t>Đại diện Sun World Sầm Sơn cho biết chương trình ưu đãi nhằm tri ân khách hàng đã ủng hộ suốt thời gian công viên nước ra mắt. Từ ngày 3/9, giá 100.000 đồng áp dụng chung cho mọi lứa tuổi. Trước đó, giá gốc 200.000 đồng (khách ngoại tỉnh) và 150.000 đồng (người Thanh Hóa). Riêng bé dưới 1 m được miễn phí vé. Khai trương đúng dịp cao điểm hè 30/6, Sun World Sầm Sơn - công viên nước quy mô nhất miền Bắc cùng tổ hợp trò chơi đạt kỷ lục châu Á - Thái Bình Dương - là 'cú hích' cho du lịch Sầm Sơn năm nay, hút hàng nghìn lượt khách mỗi ngày. Công viên nước thuộc phường Quảng Châu, Quảng Tiến, ngay đại lộ Nam sông Mã - cửa ngõ Sầm Sơn, cách trung tâm TP Thanh Hóa13 km và bãi biển Sầm Sơn 1,5 km. Thiết kế không gian lấy cảm hứng từ truyện dân gian Việt Nam, kết hợp hài hòa kiến trúc truyền thống và hiện đại. Các trò chơi cùng cảnh quan vừa gần gũi, vừa mới mẻ. Công viên nước chia ba phân khu riêng biệt dành cho mọi lứa tuổi: gia đình, trẻ em và khu cảm giác mạnh. Trong đó, trò 'Vịnh sóng thần' có diện tích 6.100 m2, chiều dài bờ biển nhân tạo đến 179 m. Cụ thể, phân khu cảm giác mạnh tập hợp những trò tốc độ, kích thích, góp phần giúp du khách giải tỏa áp lực công việc, cuộc sống. Điển hình là tổ hợp hàm cá mập, với các đường trượt uốn lượn, độ dốc cao chủ đề 'cá mập hung tàn' hay 'cá mập siêu bạo chúa'. Nhằm đáp ứng nhu cầu vui chơi của gia đình lẫn nhóm bạn trẻ, ban tổ chức kiến tạo mê cung quy mô lớn, nhấn vào các đường trượt đan chéo và vực lốc xoáy (tổ hợp ống trượt uốn lượn, xoắn ốc như các xoáy nước dành cho phao đôi đầu tiên tại châu Á - Thái Bình Dương). Du khách có thể khám phá đa dạng đường trượt gồm: 'cá đuối vượt sóng', 'cá trê vượt thác' hay 8 làn trượt thảm bạch tuộc. Chủ dự án cũng bố trí phân khu bến tuổi thơ cho trẻ, với 3 tổ hợp nhỏ mô hình sinh vật dưới nước quen thuộc. Bao quanh khu trò chơi là sông lười, gợi nhớ dòng Đơ tại Sầm Sơn. Tại đây, du khách có thể lênh đênh theo dòng nước, thư giãn và tận hưởng cảm giác sảng khoái như trẻ thơ. Nếu muốn khám phá trọn vẹn công viên nước, du khách nên đến từ 10h hoặc 15h bởi nắng không quá gắt, thích hợp với cả người già lẫn trẻ nhỏ. Vạn Phát</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sun World Sầm Sơn giảm giá vé 100.000 đồng từ ngày 3/9, miễn phí cho trẻ dưới 1m. Công viên nước quy mô lớn nằm gần trung tâm TP Thanh Hóa, hấp dẫn du khách nhờ nhiều trò chơi kết hợp giữa truyền thống và hiện đại.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>{
+  "id": 13,
+  "style": "news_brief",
+  "article": "Đại diện Sun World Sầm Sơn cho biết chương trình ưu đãi nhằm tri ân khách hàng đã ủng hộ suốt thời gian công viên nước ra mắt. Từ ngày 3/9, giá 100.000 đồng áp dụng chung cho mọi lứa tuổi. Trước đó, giá gốc 200.000 đồng (khách ngoại tỉnh) và 150.000 đồng (người Thanh Hóa). Riêng bé dưới 1 m được miễn phí vé. Khai trương đúng dịp cao điểm hè 30/6, Sun World Sầm Sơn - công viên nước quy mô nhất miền Bắc cùng tổ hợp trò chơi đạt kỷ lục châu Á - Thái Bình Dương - là 'cú hích' cho du lịch Sầm Sơn năm nay, hút hàng nghìn lượt khách mỗi ngày. Công viên nước thuộc phường Quảng Châu, Quảng Tiến, ngay đại lộ Nam sông Mã - cửa ngõ Sầm Sơn, cách trung tâm TP Thanh Hóa13 km và bãi biển Sầm Sơn 1,5 km. Thiết kế không gian lấy cảm hứng từ truyện dân gian Việt Nam, kết hợp hài hòa kiến trúc truyền thống và hiện đại. Các trò chơi cùng cảnh quan vừa gần gũi, vừa mới mẻ. Công viên nước chia ba phân khu riêng biệt dành cho mọi lứa tuổi: gia đình, trẻ em và khu cảm giác mạnh. Trong đó, trò 'Vịnh sóng thần' có diện tích 6.100 m2, chiều dài bờ biển nhân tạo đến 179 m. Cụ thể, phân khu cảm giác mạnh tập hợp những trò tốc độ, kích thích, góp phần giúp du khách giải tỏa áp lực công việc, cuộc sống. Điển hình là tổ hợp hàm cá mập, với các đường trượt uốn lượn, độ dốc cao chủ đề 'cá mập hung tàn' hay 'cá mập siêu bạo chúa'. Nhằm đáp ứng nhu cầu vui chơi của gia đình lẫn nhóm bạn trẻ, ban tổ chức kiến tạo mê cung quy mô lớn, nhấn vào các đường trượt đan chéo và vực lốc xoáy (tổ hợp ống trượt uốn lượn, xoắn ốc như các xoáy nước dành cho phao đôi đầu tiên tại châu Á - Thái Bình Dương). Du khách có thể khám phá đa dạng đường trượt gồm: 'cá đuối vượt sóng', 'cá trê vượt thác' hay 8 làn trượt thảm bạch tuộc. Chủ dự án cũng bố trí phân khu bến tuổi thơ cho trẻ, với 3 tổ hợp nhỏ mô hình sinh vật dưới nước quen thuộc. Bao quanh khu trò chơi là sông lười, gợi nhớ dòng Đơ tại Sầm Sơn. Tại đây, du khách có thể lênh đênh theo dòng nước, thư giãn và tận hưởng cảm giác sảng khoái như trẻ thơ. Nếu muốn khám phá trọn vẹn công viên nước, du khách nên đến từ 10h hoặc 15h bởi nắng không quá gắt, thích hợp với cả người già lẫn trẻ nhỏ. Vạn Phát",
+  "summary": "Sun World Sầm Sơn giảm giá vé 100.000 đồng từ ngày 3/9, miễn phí cho trẻ dưới 1m. Công viên nước quy mô lớn nằm gần trung tâm TP Thanh Hóa, hấp dẫn du khách nhờ nhiều trò chơi kết hợp giữa truyền thống và hiện đại.",
+  "faithfulness_score": 0.8,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng thiếu sót một số chi tiết quan trọng như thời gian khai trương, các phân khu trong công viên nước và một số trò chơi đặc biệt",
+  "relevance_score": 0.7,
+  "relevance_reason": "Bản tóm tắt chưa bao hàm đủ các ý chính quan trọng như mục đích của chương trình ưu đãi, vị trí và thiết kế của công viên nước",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt có logic, dễ đọc và súc tích, tuy nhiên có thể cải thiện bằng cách thêm một số chi tiết quan trọng mà không làm cho bản tóm tắt trở nên rườm rà"
+}</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -587,8 +807,27 @@
           <t>Chiều 28/8, khách sạn Grand Mercure Hanoi đón hơn 200 vị khách thuộc đoàn 4.500 du khách từ Ấn Độ sang Việt Nam. Theo ông Remi Faubel, tổng quản lý khách sạn, đây là cơ hội lớn để quảng bá nét đẹp văn hóa, truyền thống tới khách quốc tế. 'Chúng tôi tự tin các yếu tố như lối kiến trúc Đông Dương, hệ thống cửa Bức Bàn, các chi tiết nội thất lấy cảm hứng từ hoa sen, trống đồng, hạt gạo, ruộng bậc thang,... sẽ góp phần để lại ấn tượng tốt đẹp trong lòng du khách', ông Faubel nói. Do nhu cầu của khách, Grand Mercure Hanoi vẫn phục vụ chủ yếu các món Ấn. Bếp trưởng - Nguyễn Minh Nguyện lý giải, du khách Ấn Độ luôn có nhu cầu thưởng thức ẩm thực đất nước họ để có cảm giác gần gũi và thoải mái khi đi du lịch. Đó cũng là cách họ gìn giữ văn hóa và chế độ ăn truyền thống. 'Khi lên kế hoạch, chúng tôi phải trao đổi với phía đại diện đoàn để nắm thông tin về chế độ ăn, suất ăn tôn giáo, yêu cầu đặc biệt, từ đó lựa chọn các loại gia vị đặc trưng của Ấn Độ để các món ăn giữ được hương vị', vị bếp trưởng nói. Tuy nhiên, khách sạn cũng chuẩn bị thêm một số món ăn đặc trưng của Việt Nam như gà, bánh cuốn, xôi, hoa quả nhiệt đới... để giới thiệu đến đoàn khách. Từ ngày 27/8 đến 3/9, Việt Nam đón 4.500 du khách thuộc tập đoàn dược phẩm lớn đến từ Ấn Độ. Dự kiến, họ sẽ chia thành các nhóm nhỏ tới Hà Nội - Ninh Bình - Hạ Long và sử dụng các dịch vụ lưu trú, ăn uống tại các khách sạn 5 sao trên địa bàn thủ đô. Ấn Độ là một trong 10 thị trường khách du lịch quốc tế lớn nhất Việt Nam. Theo số liệu từ Cục Du lịch Quốc gia, trong 6 tháng đầu năm, nước ta đã đón 231.000 lượt khách Ấn Độ, tăng 164% so với cùng kỳ năm 2023. Việt Nam có nhiều thế mạnh để thu hút và phát triển thị trường này. Các đường bay thẳng giữa hai nước được khai thác trong thời gian gần đây khiến thời gian di chuyển rút ngắn chỉ còn khoảng 4 - 5 tiếng. Theo Outlook Traveller, Việt Nam sở hữu những cảnh quan đẹp, nền văn hóa đa dạng và chiều sâu lịch sử. Giá thành dịch vụ cạnh tranh khiến nước ta trở thành điểm đến lý tưởng cho du khách Ấn Độ. Lan Anh</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Hàng nghìn du khách Ấn Độ đến Grand Mercure Hanoi, nơi lối kiến trúc Đông Dương và ẩm thực truyền thống tạo ấn tượng tốt. Việt Nam với cảnh quan đẹp đa dạng văn hóa lịch sử thu hút du khách do giá cả hợp lý.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>{
+  "id": 14,
+  "style": "news_brief",
+  "article": "Chiều 28/8, khách sạn Grand Mercure Hanoi đón hơn 200 vị khách thuộc đoàn 4.500 du khách từ Ấn Độ sang Việt Nam. Theo ông Remi Faubel, tổng quản lý khách sạn, đây là cơ hội lớn để quảng bá nét đẹp văn hóa, truyền thống tới khách quốc tế. 'Chúng tôi tự tin các yếu tố như lối kiến trúc Đông Dương, hệ thống cửa Bức Bàn, các chi tiết nội thất lấy cảm hứng từ hoa sen, trống đồng, hạt gạo, ruộng bậc thang,... sẽ góp phần để lại ấn tượng tốt đẹp trong lòng du khách', ông Faubel nói. Do nhu cầu của khách, Grand Mercure Hanoi vẫn phục vụ chủ yếu các món Ấn. Bếp trưởng - Nguyễn Minh Nguyện lý giải, du khách Ấn Độ luôn có nhu cầu thưởng thức ẩm thực đất nước họ để có cảm giác gần gũi và thoải mái khi đi du lịch. Đó cũng là cách họ gìn giữ văn hóa và chế độ ăn truyền thống. 'Khi lên kế hoạch, chúng tôi phải trao đổi với phía đại diện đoàn để nắm thông tin về chế độ ăn, suất ăn tôn giáo, yêu cầu đặc biệt, từ đó lựa chọn các loại gia vị đặc trưng của Ấn Độ để các món ăn giữ được hương vị', vị bếp trưởng nói. Tuy nhiên, khách sạn cũng chuẩn bị thêm một số món ăn đặc trưng của Việt Nam như gà, bánh cuốn, xôi, hoa quả nhiệt đới... để giới thiệu đến đoàn khách. Từ ngày 27/8 đến 3/9, Việt Nam đón 4.500 du khách thuộc tập đoàn dược phẩm lớn đến từ Ấn Độ. Dự kiến, họ sẽ chia thành các nhóm nhỏ tới Hà Nội - Ninh Bình - Hạ Long và sử dụng các dịch vụ lưu trú, ăn uống tại các khách sạn 5 sao trên địa bàn thủ đô. Ấn Độ là một trong 10 thị trường khách du lịch quốc tế lớn nhất Việt Nam. Theo số liệu từ Cục Du lịch Quốc gia, trong 6 tháng đầu năm, nước ta đã đón 231.000 lượt khách Ấn Độ, tăng 164% so với cùng kỳ năm 2023. Việt Nam có nhiều thế mạnh để thu hút và phát triển thị trường này. Các đường bay thẳng giữa hai nước được khai thác trong thời gian gần đây khiến thời gian di chuyển rút ngắn chỉ còn khoảng 4 - 5 tiếng. Theo Outlook Traveller, Việt Nam sở hữu những cảnh quan đẹp, nền văn hóa đa dạng và chiều sâu lịch sử. Giá thành dịch vụ cạnh tranh khiến nước ta trở thành điểm đến lý tưởng cho du khách Ấn Độ. Lan Anh",
+  "summary": "Hàng nghìn du khách Ấn Độ đến Grand Mercure Hanoi, nơi lối kiến trúc Đông Dương và ẩm thực truyền thống tạo ấn tượng tốt. Việt Nam với cảnh quan đẹp đa dạng văn hóa lịch sử thu hút du khách do giá cả hợp lý.",
+  "faithfulness_score": 0.8,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng thiếu sót một số chi tiết quan trọng như số lượng du khách và các hoạt động cụ thể tại khách sạn",
+  "relevance_score": 0.7,
+  "relevance_reason": "Bản tóm tắt chưa bao hàm đủ các ý chính quan trọng như nhu cầu ẩm thực của du khách Ấn Độ và việc giới thiệu văn hóa Việt Nam",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, tuy nhiên có thể rút gọn một số từ ngữ để tăng tính súc tích"
+}</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -596,8 +835,27 @@
           <t>Theo Báo cáo Hạnh phúc Thế giới (World Happiness Report) 2024 của Liên Hợp Quốc công bố hồi tháng 3, Lithuania là quốc gia 'hạnh phúc nhất thế giới dành cho những người dưới 30 tuổi (gen Z)'. Hai nhà sáng tạo nội dung Ammar Kandil và Staffan Taylor đến từ Yes Theory, kênh truyền thông nổi tiếng của Canada, quyết định đến thủ đô Vilnius để tìm hiểu xem liệu báo cáo có nói đúng. Khi hạ cánh xuống Vilnius, Amma và Staffan bắt đầu nói chuyện với người dân địa phương. Hầu hết người trẻ đều đồng ý quốc gia họ đang sống là nơi tốt nhờ 'đồ ăn tuyệt vời, người dân thân thiện, nhiều cơ hội nghề nghiệp và nền kinh tế đang phát triển'. Nhiều người trong số đó cho rằng các khó khăn mà thế hệ trước chịu đựng đã dạy thế hệ trẻ ngày nay cách tận hưởng cuộc sống trong từng khoảnh khắc và 'tìm thấy vẻ đẹp trong những điều giản dị'. Để thu hút nhiều người trẻ đến nói chuyện hơn, Amma và Staffan đã tổ chức một buổi gặp gỡ. Tại sự kiện, những người tham dự lần lượt bày tỏ quan điểm. 'Sau một năm sống tại Mỹ, tôi đánh giá cao cuộc sống ở Lithuania vì tính kết nối với thiên nhiên', một thanh niên chia sẻ. Người này nói thêm du khách có thể dễ dàng tiếp cận một hồ nước hay khu rừng tại Lithuania và chiêm ngưỡng khung cảnh thiên nhiên tuyệt đẹp ở đó. 'Lithuania chưa bao giờ tốt như hiện nay', một phụ nữ trẻ khác thừa nhận. Khi nói về hạnh phúc, một người dân địa phương cho biết dù người trẻ sống ở đất nước này 'khá vui vẻ' nhưng không có nghĩa họ không phải đối mặt với nhiều vấn đề, áp lực cuộc sống. Sau buổi gặp gỡ, Ammar và Staffan dành phần còn lại của chuyến đi để giao lưu với người dân địa phương, ghé thăm các điểm du lịch như nhà tù cũ Lukiškės giờ là địa điểm văn hóa và tượng đài Hill of Crosses. 'Đây là một trong những trải nghiệm du lịch hạnh phúc nhất tôi từng có', Ammar, người từng đi khắp thế giới, chia sẻ với độc giả trên kênh Yes Theory khi đang tham gia một bữa tiệc tối. Steffan đồng tình khi nhận định Lithuania chắc chắn là một trong những quốc gia cởi mở, hào phóng, tử tế nhất mà anh từng đến. Video của hai du khách đến từ Canada đã thu hút gần một triệu lượt xem và bình luận chỉ sau vài ngày đăng tải. Một người từng đến Vilnius học theo diện trao đổi sinh viên chia sẻ thời gian ở Liathuania là quãng thời gian hạnh phúc nhất của mình. 'Cảm ơn Liathuania đã chào đón tôi', người này nói. 'Tình yêu, sự sáng tạo và lòng tốt có thể giúp chúng ta vượt qua quá khứ đen tối, biến tiêu cực thành ánh sáng và giúp đỡ người khác', một người dân địa phương bày tỏ sau khi xem video của Ammar và Steffan. Anh Minh(TheoYes Theory, DM)</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Lithuania được đánh giá cao về sự cởi mở, hào phóng và đồ ăn ngon. Tuy nhiên, cuộc sống vẫn có áp lực từ thế hệ trước đã dạy trẻ tận hưởng từng khoảnh khắc và tìm thấy vẻ đẹp trong giản dị.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>{
+  "id": 15,
+  "style": "news_brief",
+  "article": "Theo Báo cáo Hạnh phúc Thế giới (World Happiness Report) 2024 của Liên Hợp Quốc công bố hồi tháng 3, Lithuania là quốc gia 'hạnh phúc nhất thế giới dành cho những người dưới 30 tuổi (gen Z)'. Hai nhà sáng tạo nội dung Ammar Kandil và Staffan Taylor đến từ Yes Theory, kênh truyền thông nổi tiếng của Canada, quyết định đến thủ đô Vilnius để tìm hiểu xem liệu báo cáo có nói đúng. Khi hạ cánh xuống Vilnius, Amma và Staffan bắt đầu nói chuyện với người dân địa phương. Hầu hết người trẻ đều đồng ý quốc gia họ đang sống là nơi tốt nhờ 'đồ ăn tuyệt vời, người dân thân thiện, nhiều cơ hội nghề nghiệp và nền kinh tế đang phát triển'. Nhiều người trong số đó cho rằng các khó khăn mà thế hệ trước chịu đựng đã dạy thế hệ trẻ ngày nay cách tận hưởng cuộc sống trong từng khoảnh khắc và 'tìm thấy vẻ đẹp trong những điều giản dị'. Để thu hút nhiều người trẻ đến nói chuyện hơn, Amma và Staffan đã tổ chức một buổi gặp gỡ. Tại sự kiện, những người tham dự lần lượt bày tỏ quan điểm. 'Sau một năm sống tại Mỹ, tôi đánh giá cao cuộc sống ở Lithuania vì tính kết nối với thiên nhiên', một thanh niên chia sẻ. Người này nói thêm du khách có thể dễ dàng tiếp cận một hồ nước hay khu rừng tại Lithuania và chiêm ngưỡng khung cảnh thiên nhiên tuyệt đẹp ở đó. 'Lithuania chưa bao giờ tốt như hiện nay', một phụ nữ trẻ khác thừa nhận. Khi nói về hạnh phúc, một người dân địa phương cho biết dù người trẻ sống ở đất nước này 'khá vui vẻ' nhưng không có nghĩa họ không phải đối mặt với nhiều vấn đề, áp lực cuộc sống. Sau buổi gặp gỡ, Ammar và Staffan dành phần còn lại của chuyến đi để giao lưu với người dân địa phương, ghé thăm các điểm du lịch như nhà tù cũ Lukiškės giờ là địa điểm văn hóa và tượng đài Hill of Crosses. 'Đây là một trong những trải nghiệm du lịch hạnh phúc nhất tôi từng có', Ammar, người từng đi khắp thế giới, chia sẻ với độc giả trên kênh Yes Theory khi đang tham gia một bữa tiệc tối. Steffan đồng tình khi nhận định Lithuania chắc chắn là một trong những quốc gia cởi mở, hào phóng, tử tế nhất mà anh từng đến. Video của hai du khách đến từ Canada đã thu hút gần một triệu lượt xem và bình luận chỉ sau vài ngày đăng tải. Một người từng đến Vilnius học theo diện trao đổi sinh viên chia sẻ thời gian ở Liathuania là quãng thời gian hạnh phúc nhất của mình. 'Cảm ơn Liathuania đã chào đón tôi', người này nói. 'Tình yêu, sự sáng tạo và lòng tốt có thể giúp chúng ta vượt qua quá khứ đen tối, biến tiêu cực thành ánh sáng và giúp đỡ người khác', một người dân địa phương bày tỏ sau khi xem video của Ammar và Steffan. Anh Minh(TheoYes Theory, DM)",
+  "summary": "Lithuania được đánh giá cao về sự cởi mở, hào phóng và đồ ăn ngon. Tuy nhiên, cuộc sống vẫn có áp lực từ thế hệ trước đã dạy trẻ tận hưởng từng khoảnh khắc và tìm thấy vẻ đẹp trong giản dị.",
+  "faithfulness_score": 0.8,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng thiếu sót một số chi tiết quan trọng như việc Lithuania được đánh giá là quốc gia hạnh phúc nhất thế giới dành cho người dưới 30 tuổi và các hoạt động của Ammar và Staffan khi đến Vilnius",
+  "relevance_score": 0.7,
+  "relevance_reason": "Bản tóm tắt không bao hàm đủ các ý chính quan trọng như việc người dân Lithuania đánh giá cao cuộc sống ở đây vì đồ ăn tuyệt vời, người dân thân thiện, nhiều cơ hội nghề nghiệp và nền kinh tế đang phát triển",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, tuy nhiên có thể rút gọn một số chi tiết để tăng tính súc tích"
+}</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -605,8 +863,27 @@
           <t>Đi dạo trong khuôn viên lâu đài của mình ở Pháp vào một buổi tối mùa hè 2023, Philippa Girling cảm thấy nhẹ nhõm khi nghe thấy tiếng cười của những du khách nữ đang lưu trú tại đây. Tiếng cười là mục tiêu mà CEO Camp Château, nơi tổ chức trại hè dành riêng cho phụ nữ, mong muốn khi mở dịch vụ này. Tuy mới thành lập được hai năm, danh sách khách đăng ký đến nghỉ dưỡng tại lâu đài cổ nằm trên đỉnh đồi ở vùng Quercy, tây nam nước Pháp, năm nay đã kín chỗ. Lượng khách chờ cho mùa hè 2025 đã lên đến 11.000 người. Philippa rất vui khi được mọi người yêu thích dịch vụ cũng nhưng cảm thấy rất tiếc cho những người trong danh sách chờ khi nhiều du khách sẽ phải đợi 20 năm mới đến lượt. Cô đang xem xét để mở rộng trại hè, giúp nhiều du khách nữ có thể sử dụng dịch vụ hơn. Philippa nói mục đích tồn tại của Camp Château rất đơn giản: mang đến cho phụ nữ trải nghiệm vui vẻ. Philippa từng làm 30 năm trong ngành ngân hàng nên thấu hiểu áp lực mà phụ nữ ngày nay phải đối mặt. Do đó, cô cùng các đồng sáng lập tạo ra Camp Château để giúp các khách hàng nữ của mình thư giãn, mang lại cho họ sự chăm sóc sức khỏe tinh thần và thể chất, không gian yên tĩnh và thời gian để hồi phục trước khi quay về cuộc sống thường ngày. Kỳ nghỉ trong trại hè kéo dài sáu ngày năm đêm với nhiều hoạt động để hội viên tham gia như làm nến, nếm thử phô mai, cưỡi ngựa, yoga. Một số phụ nữ hào hứng tham gia mọi hoạt động, số khác thích dành phần lớn thời gian nằm bên hồ bơi. Mỗi đợt đón khách khoảng 50 người. Girling, người lớn lên ở miền nam nước Anh, thường đi nghỉ ở Quercy và hiện sống ở California, Mỹ, nhận thấy 'phụ nữ khi ở bên nhau thật tuyệt vời'. Những người phụ nữ đều rất hòa đồng. Họ nằm giường tầng trong các căn phòng tại lâu đài hoặc trong lều dành cho hai người. Tất cả cùng dùng chung bữa tối tại sảnh lớn và có khung giờ phục vụ đồ uống riêng. Trọng tâm của chương trình trại hè này là trao cho phụ nữ quyền tự quyết, làm mọi thứ họ muốn và chỉ cần đối xử tử tế với nhau. Toàn bộ thiết kế của Camp Château đều hướng tới mục đích giúp mọi người có thể gặp gỡ, trò chuyện nhiều hơn một cách tự nhiên nhất. Điều duy nhất khách cần quyết định tại Camp Château là muốn nghỉ ngơi hay vui chơi. Tất cả phụ nữ đều được chào đón tại trại hè. Từ tháng 7 trở về trước, phần lớn khách đến đây là người Mỹ. Nhưng từ đầu tháng 8, số lượng quốc tịch đa dạng hơn khi có thêm các khách đến từ Andorra, Canada, Ai Cập, Anh và Nigeria. Độ tuổi từ 19 đến ngoài 70 tuổi. Nhiều người đến một mình và không ít người gọi trại hè này là 'môi trường an toàn phục vụ niềm đam mê du lịch' của họ. Ngoài ra, trại hè cũng đón các nhóm khách nhỏ gồm mẹ và con gái. Giá một kỳ nghỉ là 2.178 euro, gồm mọi chi phí ăn ở, vui chơi và không tính đưa đón sân bay, dịch vụ massage. Philippa nói số tiền này không nhỏ nhưng cô và các cộng sự đã phải tính toán để đưa ra mức giá phải chăng nhất có thể. Càng ngày, lượng khách đăng ký càng đông. Nhưng Philippa nói sẽ không tăng giá vì muốn nhiều người có thể tiếp cận trải nghiệm này thay vì hướng tới tệp khách nhà giàu. Anh Minh(TheoEuro News)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Du khách nữ đến Camp Château, lâu đài cổ ở Quercy, Tây Nam Pháp với các hoạt động như làm nến, yoga hoặc thư giãn bên hồ bơi. Mục tiêu trại hè là mang lại trải nghiệm vui vẻ và chăm sóc sức khỏe tinh thần thể chất cho phụ nữ tự quyết định mọi thứ trong sự tôn trọng lẫn nhau. Camp Château đón khách đa dạng từ Mỹ đến Andorra với 11.000 người đăng ký mùa hè năm nay, nhưng nhiều du khách phải đợi hai thập kỷ mới được phục vụ. Philippa Girling tăng giá không vì muốn tiếp cận rộng rãi hơn mà nhằm tập trung vào tệp khách giàu có; tuy nhiên, cô cũng nhận ra rằng cần mở rộng dịch vụ để giúp phụ nữ sử dụng nó dễ dàng hơn. Camp Château tạo điều kiện cho các phụ nữ thư giãn và hồi phục sau khi quay về cuộc sống thường ngày, nhấn mạnh quyền tự quyết định của họ trong sự tôn trọng lẫn nhau.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>{
+  "id": 16,
+  "style": "news_brief",
+  "article": "Đi dạo trong khuôn viên lâu đài của mình ở Pháp vào một buổi tối mùa hè 2023, Philippa Girling cảm thấy nhẹ nhõm khi nghe thấy tiếng cười của những du khách nữ đang lưu trú tại đây. Tiếng cười là mục tiêu mà CEO Camp Château, nơi tổ chức trại hè dành riêng cho phụ nữ, mong muốn khi mở dịch vụ này. Tuy mới thành lập được hai năm, danh sách khách đăng ký đến nghỉ dưỡng tại lâu đài cổ nằm trên đỉnh đồi ở vùng Quercy, tây nam nước Pháp, năm nay đã kín chỗ. Lượng khách chờ cho mùa hè 2025 đã lên đến 11.000 người. Philippa rất vui khi được mọi người yêu thích dịch vụ cũng nhưng cảm thấy rất tiếc cho những người trong danh sách chờ khi nhiều du khách sẽ phải đợi 20 năm mới đến lượt. Cô đang xem xét để mở rộng trại hè, giúp nhiều du khách nữ có thể sử dụng dịch vụ hơn. Philippa nói mục đích tồn tại của Camp Château rất đơn giản: mang đến cho phụ nữ trải nghiệm vui vẻ. Philippa từng làm 30 năm trong ngành ngân hàng nên thấu hiểu áp lực mà phụ nữ ngày nay phải đối mặt. Do đó, cô cùng các đồng sáng lập tạo ra Camp Château để giúp các khách hàng nữ của mình thư giãn, mang lại cho họ sự chăm sóc sức khỏe tinh thần và thể chất, không gian yên tĩnh và thời gian để hồi phục trước khi quay về cuộc sống thường ngày. Kỳ nghỉ trong trại hè kéo dài sáu ngày năm đêm với nhiều hoạt động để hội viên tham gia như làm nến, nếm thử phô mai, cưỡi ngựa, yoga. Một số phụ nữ hào hứng tham gia mọi hoạt động, số khác thích dành phần lớn thời gian nằm bên hồ bơi. Mỗi đợt đón khách khoảng 50 người. Girling, người lớn lên ở miền nam nước Anh, thường đi nghỉ ở Quercy và hiện sống ở California, Mỹ, nhận thấy 'phụ nữ khi ở bên nhau thật tuyệt vời'. Những người phụ nữ đều rất hòa đồng. Họ nằm giường tầng trong các căn phòng tại lâu đài hoặc trong lều dành cho hai người. Tất cả cùng dùng chung bữa tối tại sảnh lớn và có khung giờ phục vụ đồ uống riêng. Trọng tâm của chương trình trại hè này là trao cho phụ nữ quyền tự quyết, làm mọi thứ họ muốn và chỉ cần đối xử tử tế với nhau. Toàn bộ thiết kế của Camp Château đều hướng tới mục đích giúp mọi người có thể gặp gỡ, trò chuyện nhiều hơn một cách tự nhiên nhất. Điều duy nhất khách cần quyết định tại Camp Château là muốn nghỉ ngơi hay vui chơi. Tất cả phụ nữ đều được chào đón tại trại hè. Từ tháng 7 trở về trước, phần lớn khách đến đây là người Mỹ. Nhưng từ đầu tháng 8, số lượng quốc tịch đa dạng hơn khi có thêm các khách đến từ Andorra, Canada, Ai Cập, Anh và Nigeria. Độ tuổi từ 19 đến ngoài 70 tuổi. Nhiều người đến một mình và không ít người gọi trại hè này là 'môi trường an toàn phục vụ niềm đam mê du lịch' của họ. Ngoài ra, trại hè cũng đón các nhóm khách nhỏ gồm mẹ và con gái. Giá một kỳ nghỉ là 2.178 euro, gồm mọi chi phí ăn ở, vui chơi và không tính đưa đón sân bay, dịch vụ massage. Philippa nói số tiền này không nhỏ nhưng cô và các cộng sự đã phải tính toán để đưa ra mức giá phải chăng nhất có thể. Càng ngày, lượng khách đăng ký càng đông. Nhưng Philippa nói sẽ không tăng giá vì muốn nhiều người có thể tiếp cận trải nghiệm này thay vì hướng tới tệp khách nhà giàu. Anh Minh(TheoEuro News)",
+  "summary": "Du khách nữ đến Camp Château, lâu đài cổ ở Quercy, Tây Nam Pháp với các hoạt động như làm nến, yoga hoặc thư giãn bên hồ bơi. Mục tiêu trại hè là mang lại trải nghiệm vui vẻ và chăm sóc sức khỏe tinh thần thể chất cho phụ nữ tự quyết định mọi thứ trong sự tôn trọng lẫn nhau. Camp Château đón khách đa dạng từ Mỹ đến Andorra với 11.000 người đăng ký mùa hè năm nay, nhưng nhiều du khách phải đợi hai thập kỷ mới được phục vụ. Philippa Girling tăng giá không vì muốn tiếp cận rộng rãi hơn mà nhằm tập trung vào tệp khách giàu có; tuy nhiên, cô cũng nhận ra rằng cần mở rộng dịch vụ để giúp phụ nữ sử dụng nó dễ dàng hơn. Camp Château tạo điều kiện cho các phụ nữ thư giãn và hồi phục sau khi quay về cuộc sống thường ngày, nhấn mạnh quyền tự quyết định của họ trong sự tôn trọng lẫn nhau.",
+  "faithfulness_score": 0.8,
+  "faithfulness_reason": "Bản tóm tắt có một số điểm không chính xác như việc Philippa Girling tăng giá không phải để tập trung vào tệp khách giàu có mà là không tăng giá để giúp nhiều người có thể tiếp cận trải nghiệm này",
+  "relevance_score": 0.9,
+  "relevance_reason": "Bản tóm tắt bao gồm hầu hết các ý chính quan trọng như mục tiêu của Camp Château, các hoạt động và đối tượng khách hàng, tuy nhiên có thể thêm một số chi tiết về lý do thành lập và không gian của lâu đài",
+  "coherence_conciseness_score": 0.8,
+  "coherence_conciseness_reason": "Bản tóm tắt có logic và dễ đọc, tuy nhiên có một số câu dài và phức tạp, cần được tinh gọn hơn để tăng tính súc tích"
+}</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -614,8 +891,27 @@
           <t>Thời gian này tại Malaysia cũng có nhiều sự kiện để du khách trải nghiệm như: lễ hội trò chơi dân gian tại Kuala Lumpur (13-16/9), lễ hội văn hóa Putrajaya (27-29/9), lễ hội bãi biển Tanjung Aru 2024 tại Kota Kinabalu (1 và 22/9)... Điểm đến phổ biến nhất tại Malaysia là thủ đô Kuala Lumpur - đô thị sầm uất với những di sản kiến trúc cùng các cao ốc hiện đại. Công trình nổi tiếng nhất là tháp đôi Petronas cao 88 tầng. Tại đây có đài quan sát toàn cảnh thành phố, cầu treo trên không, trung tâm khám phá khoa học Petrosains, thủy cung Aquaria KLCC và trung tâm mua sắm Suria KLCC. Quận trung tâm thành phố Kuala Lumpur là Bukit Bintang, khu vực nhộn nhịp bậc nhất với các khu mua sắm, khách sạn và nhà hàng cao cấp cùng nhiều tụ điểm vui chơi, giải trí. Đảo Penang lại mang đến không khí bình yên, nhẹ nhàng. Đặc biệt, George Town - thủ phủ của bang Penang là di sản thế giới, phản ánh rõ nét dấu vết lịch sử qua từng công trình kiến trúc lẫn đời sống văn hóa của cư dân, từ những ngõ nhỏ với căn nhà hai tầng của người Hoa đến tòa hội đồng thành phố, tháp đồng hồ từ thời thuộc địa Anh. Du khách đừng quên ghé đồi Penang Hill hay đền Kek Lok Si. Langkawi là quần đảo với 99 đảo nhỏ ngoài khơi biển Andaman. Vùng đất này có nhiều bãi biển hoang sơ với khu nghỉ dưỡng cao cấp, phù hợp cho kỳ nghỉ thư giãn sau những ngày bận rộn. Ngoài ra, hòn đảo này còn là điểm đến lý tưởng cho các môn thể thao dưới nước như lặn biển, dù kéo, mô tô nước hoặc khám phá công viên địa chất hàng triệu năm tuổi. Cao nguyên Cameron là địa danh nằm ở bang Pahang, được bao phủ một màu xanh dài bất tận bởi những đồi chè và loại cây ôn đới. Khí hậu của cao nguyên này mang đến cho du khách sự mát mẻ, dễ chịu như đang ở châu Âu. Khi đến đây, du khách đừng quên ghé thăm nông trại chế biến trà, vườn hoa oải hương, thung lũng hoa hồng hay thử trekking leo núi Batu Brinchang. Malaysia có nhiều món ăn hấp dẫn du khách, nổi bật là món cơm 'quốc dân' Nasi Lemak. Món cơm này gồm cơm, nấu từ gạo với nước cốt dừa, trứng luộc, gà chiên, lạc, dưa chuột thái lát, cá khô... ăn kèm xốt sambal. Món ăn tuy đơn giản song đủ dinh dưỡng và được nhiều người ưa thích. Char Kway Teow, món hủ tiếu xào nổi tiếng của cộng đồng người Hoa tại Malaysia được chế biến từ hủ tiếu bản to xào cùng tôm, chả cá, lạp xưởng, trứng, giá đỗ và hẹ. Ngoài ra, Roti Canai là món ăn của cộng đồng người Ấn. Đây là loại bánh dẹt, thơm, giòn và xốp, thường dùng kèm các loại cà ri. Thanh Thư</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>LỖI: 'NoneType' object is not iterable</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>{
+  "id": 17,
+  "style": "news_brief",
+  "article": "Thời gian này tại Malaysia cũng có nhiều sự kiện để du khách trải nghiệm như: lễ hội trò chơi dân gian tại Kuala Lumpur (13-16/9), lễ hội văn hóa Putrajaya (27-29/9), lễ hội bãi biển Tanjung Aru 2024 tại Kota Kinabalu (1 và 22/9)... Điểm đến phổ biến nhất tại Malaysia là thủ đô Kuala Lumpur - đô thị sầm uất với những di sản kiến trúc cùng các cao ốc hiện đại. Công trình nổi tiếng nhất là tháp đôi Petronas cao 88 tầng. Tại đây có đài quan sát toàn cảnh thành phố, cầu treo trên không, trung tâm khám phá khoa học Petrosains, thủy cung Aquaria KLCC và trung tâm mua sắm Suria KLCC. Quận trung tâm thành phố Kuala Lumpur là Bukit Bintang, khu vực nhộn nhịp bậc nhất với các khu mua sắm, khách sạn và nhà hàng cao cấp cùng nhiều tụ điểm vui chơi, giải trí. Đảo Penang lại mang đến không khí bình yên, nhẹ nhàng. Đặc biệt, George Town - thủ phủ của bang Penang là di sản thế giới, phản ánh rõ nét dấu vết lịch sử qua từng công trình kiến trúc lẫn đời sống văn hóa của cư dân, từ những ngõ nhỏ với căn nhà hai tầng của người Hoa đến tòa hội đồng thành phố, tháp đồng hồ từ thời thuộc địa Anh. Du khách đừng quên ghé đồi Penang Hill hay đền Kek Lok Si. Langkawi là quần đảo với 99 đảo nhỏ ngoài khơi biển Andaman. Vùng đất này có nhiều bãi biển hoang sơ với khu nghỉ dưỡng cao cấp, phù hợp cho kỳ nghỉ thư giãn sau những ngày bận rộn. Ngoài ra, hòn đảo này còn là điểm đến lý tưởng cho các môn thể thao dưới nước như lặn biển, dù kéo, mô tô nước hoặc khám phá công viên địa chất hàng triệu năm tuổi. Cao nguyên Cameron là địa danh nằm ở bang Pahang, được bao phủ một màu xanh dài bất tận bởi những đồi chè và loại cây ôn đới. Khí hậu của cao nguyên này mang đến cho du khách sự mát mẻ, dễ chịu như đang ở châu Âu. Khi đến đây, du khách đừng quên ghé thăm nông trại chế biến trà, vườn hoa oải hương, thung lũng hoa hồng hay thử trekking leo núi Batu Brinchang. Malaysia có nhiều món ăn hấp dẫn du khách, nổi bật là món cơm 'quốc dân' Nasi Lemak. Món cơm này gồm cơm, nấu từ gạo với nước cốt dừa, trứng luộc, gà chiên, lạc, dưa chuột thái lát, cá khô... ăn kèm xốt sambal. Món ăn tuy đơn giản song đủ dinh dưỡng và được nhiều người ưa thích. Char Kway Teow, món hủ tiếu xào nổi tiếng của cộng đồng người Hoa tại Malaysia được chế biến từ hủ tiếu bản to xào cùng tôm, chả cá, lạp xưởng, trứng, giá đỗ và hẹ. Ngoài ra, Roti Canai là món ăn của cộng đồng người Ấn. Đây là loại bánh dẹt, thơm, giòn và xốp, thường dùng kèm các loại cà ri. Thanh Thư",
+  "summary": "LỖI: 'NoneType' object is not iterable",
+  "faithfulness_score": 0.0,
+  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin gì về văn bản gốc, không có nội dung để đánh giá tính trung thực.",
+  "relevance_score": 0.0,
+  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không phản ánh được nội dung chính.",
+  "coherence_conciseness_score": 0.0,
+  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá tính mạch lạc và súc tích."
+}</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -623,8 +919,27 @@
           <t>Lodo, 62 tuổi, hôm 6/8 đã có buổi sáng trải nghiệm đan võng cùng với nghệ nhân ở Cù Lao Chàm. Ông bất ngờ về độ bền chắc và sự khéo léo, kỳ công của nghệ nhân làm ra nó. Lodo đã mua một chiếc võng về làm kỷ niệm trong chuyến du lịch Việt Nam lần này. 'Tôi nghĩ đây là một vật liệu xanh giúp bảo vệ môi trường', du khách đến từ Pháp nói. Theo ông Lê Vĩnh Thuận, Phó giám đốc Ban quản lý khu bảo tồn biển Cù Lao Chàm, trong dịp Festival 'Cù Lao Chàm - mùa ngô đồng đỏ' năm 2024 diễn ra từ ngày 5 đến 11/8, lượng du khách đổ về Cù Lao Chàm tham gia lễ hội 'rất đông'. Đến đây, du khách được tìm hiểu về nguồn gốc và tham gia cùng với nghệ nhân đan loại võng truyền thống của đảo. Theo giới thiệu của Trung tâm Quản lý bảo tồn di sản Hội An, sợi võng được làm từ các mảng vỏ cây ngô đồng. Sau khi được tách ra từ thân cây, vỏ sẽ được gom lại thành từng bó rồi ngâm nước ở các khe, suối trên đảo như khe Ruộng Chùa, khe Ông Thơ, khe Xóm Mới. Sau một tháng, người thợ đem vỏ về tách chọn lớp bên trong có màu trắng đục, tước từng sợi nhỏ, phơi khô cho đến khi có màu trắng tinh mới có thể bắt tay vào đan võng. Công đoạn tước đòi hỏi sự tập trung cao của người thợ vì 'sợi càng mỏng đan võng càng chặt', nghệ nhân đan võng Ngô Thị Lê, 70 tuổi, cho biết. Vào khoảng tháng 7, người dân trên đảo đi chọn vỏ những cây ngô đồng làm nguyên liệu đan võng, khi cây ra hoa, rụng hết lá, vỏ đủ khô để thu hoạch. Cây ngô đồng dùng làm võng phải có dáng thẳng mới cho ra sợi suôn, mềm, dai và chịu lực tốt. Bà Lê cho biết khi đã chọn được cây, người dân khai thác bằng cách chỉ chặt ngang thân để cây còn nảy chồi, phát triển sinh sống trở lại. Bà Huỳnh Thị Út, 56 tuổi, cùng với bà Lê là hai trong số ít nghệ nhân ở Cù Lao Chàm duy trì nghề đan võng ngô đồng cho biết loại võng này được người xã đảo sáng tạo ra trong quá trình lao động sản xuất. 'Để làm ra chiếc võng đẹp, ngoài tước sợi mỏng còn yêu cầu thắt nút các mối mắt võng đều', bà Út nói. Lodo nói những nghệ nhân đan võng đã giúp ông phân biệt võng tư có bốn dây đan nối nhau và võng sáu có sáu dây dày hơn đan thành hình tứ giác. Võng ngô đồng dài 2,6 m, đan thủ công hơn một tháng, độ bền của võng có thể kéo dài từ 5 đến 10 năm, có giá từ 5 đến 10 triệu đồng. 'Mức giá này xứng đáng với công sức những người thợ bỏ ra', Lodo cho hay. Chị Hà Nhi, 45 tuổi, sống tại Hà Nội, cũng ấn tượng với loại võng không làm từ sợi công nghiệp mà hoàn toàn từ vỏ cây. 'Những sản phẩm thủ công truyền thống thẩm mỹ cao như thế này là điểm nhấn cho du khách khi du lịch trên đảo', chị Nhi nói. Ngô đồng gắn liền với đời sống hàng ngày của người dân Cù Lao Chàm từ hơn 300 năm trước, theo Ban quản lý khu bảo tồn biển Cù Lao Chàm. Trải qua nhiều đời gìn giữ và nỗ lực bảo tồn, phát huy giá trị văn hóa, nghề đan võng ngô đồng ở địa phương được Bộ Văn hóa Thể thao và Du lịch công nhận là Di sản văn hóa phi vật thể quốc gia hôm 6/8. Tuấn Anh</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>LỖI: 'NoneType' object is not iterable</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>{
+  "id": 18,
+  "style": "news_brief",
+  "article": "Lodo, 62 tuổi, hôm 6/8 đã có buổi sáng trải nghiệm đan võng cùng với nghệ nhân ở Cù Lao Chàm. Ông bất ngờ về độ bền chắc và sự khéo léo, kỳ công của nghệ nhân làm ra nó. Lodo đã mua một chiếc võng về làm kỷ niệm trong chuyến du lịch Việt Nam lần này. 'Tôi nghĩ đây là một vật liệu xanh giúp bảo vệ môi trường', du khách đến từ Pháp nói. Theo ông Lê Vĩnh Thuận, Phó giám đốc Ban quản lý khu bảo tồn biển Cù Lao Chàm, trong dịp Festival 'Cù Lao Chàm - mùa ngô đồng đỏ' năm 2024 diễn ra từ ngày 5 đến 11/8, lượng du khách đổ về Cù Lao Chàm tham gia lễ hội 'rất đông'. Đến đây, du khách được tìm hiểu về nguồn gốc và tham gia cùng với nghệ nhân đan loại võng truyền thống của đảo. Theo giới thiệu của Trung tâm Quản lý bảo tồn di sản Hội An, sợi võng được làm từ các mảng vỏ cây ngô đồng. Sau khi được tách ra từ thân cây, vỏ sẽ được gom lại thành từng bó rồi ngâm nước ở các khe, suối trên đảo như khe Ruộng Chùa, khe Ông Thơ, khe Xóm Mới. Sau một tháng, người thợ đem vỏ về tách chọn lớp bên trong có màu trắng đục, tước từng sợi nhỏ, phơi khô cho đến khi có màu trắng tinh mới có thể bắt tay vào đan võng. Công đoạn tước đòi hỏi sự tập trung cao của người thợ vì 'sợi càng mỏng đan võng càng chặt', nghệ nhân đan võng Ngô Thị Lê, 70 tuổi, cho biết. Vào khoảng tháng 7, người dân trên đảo đi chọn vỏ những cây ngô đồng làm nguyên liệu đan võng, khi cây ra hoa, rụng hết lá, vỏ đủ khô để thu hoạch. Cây ngô đồng dùng làm võng phải có dáng thẳng mới cho ra sợi suôn, mềm, dai và chịu lực tốt. Bà Lê cho biết khi đã chọn được cây, người dân khai thác bằng cách chỉ chặt ngang thân để cây còn nảy chồi, phát triển sinh sống trở lại. Bà Huỳnh Thị Út, 56 tuổi, cùng với bà Lê là hai trong số ít nghệ nhân ở Cù Lao Chàm duy trì nghề đan võng ngô đồng cho biết loại võng này được người xã đảo sáng tạo ra trong quá trình lao động sản xuất. 'Để làm ra chiếc võng đẹp, ngoài tước sợi mỏng còn yêu cầu thắt nút các mối mắt võng đều', bà Út nói. Lodo nói những nghệ nhân đan võng đã giúp ông phân biệt võng tư có bốn dây đan nối nhau và võng sáu có sáu dây dày hơn đan thành hình tứ giác. Võng ngô đồng dài 2,6 m, đan thủ công hơn một tháng, độ bền của võng có thể kéo dài từ 5 đến 10 năm, có giá từ 5 đến 10 triệu đồng. 'Mức giá này xứng đáng với công sức những người thợ bỏ ra', Lodo cho hay. Chị Hà Nhi, 45 tuổi, sống tại Hà Nội, cũng ấn tượng với loại võng không làm từ sợi công nghiệp mà hoàn toàn từ vỏ cây. 'Những sản phẩm thủ công truyền thống thẩm mỹ cao như thế này là điểm nhấn cho du khách khi du lịch trên đảo', chị Nhi nói. Ngô đồng gắn liền với đời sống hàng ngày của người dân Cù Lao Chàm từ hơn 300 năm trước, theo Ban quản lý khu bảo tồn biển Cù Lao Chàm. Trải qua nhiều đời gìn giữ và nỗ lực bảo tồn, phát huy giá trị văn hóa, nghề đan võng ngô đồng ở địa phương được Bộ Văn hóa Thể thao và Du lịch công nhận là Di sản văn hóa phi vật thể quốc gia hôm 6/8. Tuấn Anh",
+  "summary": "LỖI: 'NoneType' object is not iterable",
+  "faithfulness_score": 0.0,
+  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin nào về văn bản gốc, không phản ánh nội dung của bài viết.",
+  "relevance_score": 0.0,
+  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ ý chính quan trọng nào từ văn bản gốc, không đề cập đến chủ đề về nghề đan võng ngô đồng tại Cù Lao Chàm.",
+  "coherence_conciseness_score": 0.0,
+  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá về tính mạch lạc và súc tích."
+}</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -632,8 +947,27 @@
           <t>Với mục tiêu quảng bá du lịch mua sắm tại Singapore, Vietrantour cùng Tổng Cục du lịch Singapore giới thiệu những điểm đến mua sắm và check in hấp dẫn. Nếu du khách đang tìm kiếm những món đồ phiên bản giới hạn của các hãng thời trang cao cấp như Prada, Louis Vuitton, Hermes, ION Orchard và Scotts Square, nên tới trục đường Orchard Road. Đặc biệt, một số thời điểm, các cửa hàng thời trang tại khu vực này khuyến mại tới 70%. Ngoài ra, một số địa điểm mua sắm người dân địa phương hay tới là Tampines 1, Jem và Westgate với nhiều cửa hàng bán lẻ, thời trang phục vụ nhu cầu đời sống. Nếu đang trong chuyến đi cùng gia đình, du khách hãy ghé qua trung tâm thương mại Tanglin Mall hoặc House of Anli với hàng nghìn mặt hàng gia dụng, sản phẩm dành cho mẹ và bé. Trong khi đó, trung tâm mua sắm Mustafa - tụ điểm mua sắm đêm khuya quen thuộc của người dân địa phương cũng là nơi nổi tiếng với những món đồ công nghệ hàng đầu, đến các sản phẩm tiêu dùng với giá cả phải chăng. Khi mua sắm tại Singapore, khách hàng còn được hoàn thuế tới 7%. Là quốc gia phát triển mạnh về dịch vụ du lịch, Singapore chú trọng nhiều đến trải nghiệm khách hàng. Đất nước này cũng được đánh giá là trạm trung gian lý tưởng để bảo hành các sản phẩm đồ hiệu, 'thiên đường' mua hàng miễn thuế với nhiều thương hiệu quốc tế và các nhãn hàng địa phương như mỹ phẩm, nước hoa, bia rượu, đồng hồ, thực phẩm... Tại Singapore, một trong những trải nghiệm thú vị là du khách có thể tự tay hoàn thiện các sản phẩm thủ công truyền thống. Các cửa hàng sẽ có thợ thủ công lành nghề hướng dẫn du khách chưng cất rượu gin tại Brass Lion Distillery, làm đồ da tại Atelier Lodge hoặc học kỹ thuật thêu tranh hạt cườm truyền thống tại Rumah Bebe. Bạn cũng có thể dạo qua khu phố di sản Kampong Gelam, nơi sở hữu những cửa hàng bày bán đồ truyền thống như đồ gốm, đồ da thủ công,.. Trải nghiệm này sẽ giúp du khách hiểu rõ hơn về nét đẹp văn hóa Singapore, đồng thời thể hiện phong cách cá nhân trong từng sản phẩm. Du khách nêndạo các nhà sách như Books Actually và Huggs-Epigram Coffee Bookshop để khám phá văn học kinh điển từ một số nhà thơ, tiểu thuyết gia của Singapore. Thanh Thư</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LỖI: 'NoneType' object is not iterable</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>{
+  "id": 19,
+  "style": "news_brief",
+  "article": "Với mục tiêu quảng bá du lịch mua sắm tại Singapore, Vietrantour cùng Tổng Cục du lịch Singapore giới thiệu những điểm đến mua sắm và check in hấp dẫn. Nếu du khách đang tìm kiếm những món đồ phiên bản giới hạn của các hãng thời trang cao cấp như Prada, Louis Vuitton, Hermes, ION Orchard và Scotts Square, nên tới trục đường Orchard Road. Đặc biệt, một số thời điểm, các cửa hàng thời trang tại khu vực này khuyến mại tới 70%. Ngoài ra, một số địa điểm mua sắm người dân địa phương hay tới là Tampines 1, Jem và Westgate với nhiều cửa hàng bán lẻ, thời trang phục vụ nhu cầu đời sống. Nếu đang trong chuyến đi cùng gia đình, du khách hãy ghé qua trung tâm thương mại Tanglin Mall hoặc House of Anli với hàng nghìn mặt hàng gia dụng, sản phẩm dành cho mẹ và bé. Trong khi đó, trung tâm mua sắm Mustafa - tụ điểm mua sắm đêm khuya quen thuộc của người dân địa phương cũng là nơi nổi tiếng với những món đồ công nghệ hàng đầu, đến các sản phẩm tiêu dùng với giá cả phải chăng. Khi mua sắm tại Singapore, khách hàng còn được hoàn thuế tới 7%. Là quốc gia phát triển mạnh về dịch vụ du lịch, Singapore chú trọng nhiều đến trải nghiệm khách hàng. Đất nước này cũng được đánh giá là trạm trung gian lý tưởng để bảo hành các sản phẩm đồ hiệu, 'thiên đường' mua hàng miễn thuế với nhiều thương hiệu quốc tế và các nhãn hàng địa phương như mỹ phẩm, nước hoa, bia rượu, đồng hồ, thực phẩm... Tại Singapore, một trong những trải nghiệm thú vị là du khách có thể tự tay hoàn thiện các sản phẩm thủ công truyền thống. Các cửa hàng sẽ có thợ thủ công lành nghề hướng dẫn du khách chưng cất rượu gin tại Brass Lion Distillery, làm đồ da tại Atelier Lodge hoặc học kỹ thuật thêu tranh hạt cườm truyền thống tại Rumah Bebe. Bạn cũng có thể dạo qua khu phố di sản Kampong Gelam, nơi sở hữu những cửa hàng bày bán đồ truyền thống như đồ gốm, đồ da thủ công,.. Trải nghiệm này sẽ giúp du khách hiểu rõ hơn về nét đẹp văn hóa Singapore, đồng thời thể hiện phong cách cá nhân trong từng sản phẩm. Du khách nêndạo các nhà sách như Books Actually và Huggs-Epigram Coffee Bookshop để khám phá văn học kinh điển từ một số nhà thơ, tiểu thuyết gia của Singapore. Thanh Thư",
+  "summary": "LỖI: 'NoneType' object is not iterable",
+  "faithfulness_score": 0.0,
+  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin nào về văn bản gốc, không có nội dung để đánh giá tính trung thực.",
+  "relevance_score": 0.0,
+  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không thể đánh giá tính bao quát.",
+  "coherence_conciseness_score": 0.0,
+  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá tính mạch lạc và súc tích."
+}</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -641,8 +975,27 @@
           <t>Chương trình lần này có sự đồng hành của diễn viên Ninh Dương Lan Ngọc. Thông qua Epic Sale, diễn viên mong muốn lan tỏa tinh thần du lịch thông minh, tiện lợi và tối ưu chi phí. Ông Iko Putera, Giám đốc Vận chuyển Traveloka, cho biết việc hợp tác cùng Lan Ngọc đánh dấu cột mốc quan trọng trên hành trình mang đến trải nghiệm du lịch tiện nghi tối ưu cho khách hàng. Tầm ảnh hưởng và đam mê du lịch của cô phù hợp với sứ mệnh nền tảng theo đuổi. Đôi bên đều muốn truyền cảm hứng khám phá thế giới qua những chuyến đi. Với Epic Sale lần này, Traveloka áp dụng ưu đãi đến 50% cho các sản phẩm du lịch, dịch vụ trên toàn thế giới. 'Đây là lời tri ân chúng tôi muốn gửi đến khách hàng đã luôn ủng hộ, gắn bó trên hành trình kiến tạo những chuyến đi đáng nhớ cùng Traveloka', ông Iko Putera cho biết. Từ khi trở thành đại sứ thương hiệu tại Việt Nam, diễn viên Ninh Dương Lan Ngọc đã có nhiều trải nghiệm du lịch chất lượng với nền tảng. Với loạt khuyến mại, ưu đãi, quà tặng trong Epic Sale 2024, cô nói sẽ tranh thủ săn vé, đặt phòng, chuẩn bị cho những chuyến đi sắp tới. Theo Lan Ngọc, chương trình mang lại cho du khách cơ hội du lịch tiện nghi với chi phí tiết kiệm, giúp khơi dậy mong muốn đi đây đi đó, khám phá thế giới. Cô đánh giá cao sự tiện lợi và các dịch vụ toàn diện của nền tảng, giúp việc lên kế hoạch cho các chuyến đi thêm dễ dàng, thú vị. Traveloka đã hợp tác cùng hàng nghìn đối tác để mang đến những deal giá ưu đãi sâu. Người dùng có thể truy cập nền tảng, theo dõi các ưu đãi hàng ngày trong các mục Vé máy bay, Khách sạn, Xperience và nhiều sản phẩm du lịch khác. 'Siêu ưu đãi Epic' (Super Epic Deal) sẽ được áp dụng cho các sản phẩm nhất định trong khung giờ giới hạn. Cụ thể, giờ vàng Epic Hour Deal ưu đãi vé máy bay mỗi thứ Bảy từ 14h-17h; đặt khách sạn giờ vàng EPIC Hotel Hour Deal diễn ra hàng ngày từ 18h-19h. Du khách có thể săn vé máy bay quốc nội và quốc tế với giá ưu đãi. Trong đó, vé nội địa Vietravel giá chỉ từ 781.925 đồng; vé China Southern Airlines đi Thâm Quyến từ 2,819 đồng; vé T'way Air đến Hàn Quốc và Nhật Bản lần lượt chỉ từ 2,667 triệu đồng và 2,682 triệu đồng. Khách hàng còn có cơ hội nghỉ dưỡng tại khách sạn 5 sao trong nước với giá từ 794.000 đồng. Hàng loạt khách sạn Hàn Quốc giá từ 1,858 triệu đồng, Nhật Bản từ 1,146 triệu đồng. Với dịch vụ giải trí, nền tảng áp dụng ưu đãi 'mua 1 tặng 1' vé tham quan Sun World, công viên nước The Amazing Bay, thủy cung Sea Life Bangkok Ocean World (Thái Lan). Để du khách có trải nghiệm du lịch trọn vẹn, Traveloka giới thiệu thêm nhiều tính năng khác như: hoàn tiền 100%, thay đổi lịch trình, thanh toán linh hoạt... Xem thêm thông tin chi tiết về chương trình Epic Sale trên ứng dụng, website và các tài khoản mạng xã hội của Traveloka. Á Hiên</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>781.925 đồng vé Vietravel, 2.819 triệu Thâm Quyến; 2.667 và 2.682 triệu Hàn Quốc-Nhật Bản. Khách sạn từ 794.000-1.858 triệu. Áp dụng 'mua 1 tặng 1' Sun World, The Amazing Bay, Sea Life Bangkok Ocean World. Hoàn tiền 100%, thay đổi lịch trình, thanh toán linh hoạt trên Traveloka. Epic Sale của Ninh Dương Lan Ngọc mong muốn lan tỏa tinh thần du lịch thông minh và áp dụng ưu đãi đến 50% cho các sản phẩm toàn thế giới nhằm tri ân khách hàng và khích lệ khám phá thế giới qua những chuyến đi tiện nghi với chi phí tiết kiệm.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>{
+  "id": 20,
+  "style": "news_brief",
+  "article": "Chương trình lần này có sự đồng hành của diễn viên Ninh Dương Lan Ngọc. Thông qua Epic Sale, diễn viên mong muốn lan tỏa tinh thần du lịch thông minh, tiện lợi và tối ưu chi phí. Ông Iko Putera, Giám đốc Vận chuyển Traveloka, cho biết việc hợp tác cùng Lan Ngọc đánh dấu cột mốc quan trọng trên hành trình mang đến trải nghiệm du lịch tiện nghi tối ưu cho khách hàng. Tầm ảnh hưởng và đam mê du lịch của cô phù hợp với sứ mệnh nền tảng theo đuổi. Đôi bên đều muốn truyền cảm hứng khám phá thế giới qua những chuyến đi. Với Epic Sale lần này, Traveloka áp dụng ưu đãi đến 50% cho các sản phẩm du lịch, dịch vụ trên toàn thế giới. 'Đây là lời tri ân chúng tôi muốn gửi đến khách hàng đã luôn ủng hộ, gắn bó trên hành trình kiến tạo những chuyến đi đáng nhớ cùng Traveloka', ông Iko Putera cho biết. Từ khi trở thành đại sứ thương hiệu tại Việt Nam, diễn viên Ninh Dương Lan Ngọc đã có nhiều trải nghiệm du lịch chất lượng với nền tảng. Với loạt khuyến mại, ưu đãi, quà tặng trong Epic Sale 2024, cô nói sẽ tranh thủ săn vé, đặt phòng, chuẩn bị cho những chuyến đi sắp tới. Theo Lan Ngọc, chương trình mang lại cho du khách cơ hội du lịch tiện nghi với chi phí tiết kiệm, giúp khơi dậy mong muốn đi đây đi đó, khám phá thế giới. Cô đánh giá cao sự tiện lợi và các dịch vụ toàn diện của nền tảng, giúp việc lên kế hoạch cho các chuyến đi thêm dễ dàng, thú vị. Traveloka đã hợp tác cùng hàng nghìn đối tác để mang đến những deal giá ưu đãi sâu. Người dùng có thể truy cập nền tảng, theo dõi các ưu đãi hàng ngày trong các mục Vé máy bay, Khách sạn, Xperience và nhiều sản phẩm du lịch khác. 'Siêu ưu đãi Epic' (Super Epic Deal) sẽ được áp dụng cho các sản phẩm nhất định trong khung giờ giới hạn. Cụ thể, giờ vàng Epic Hour Deal ưu đãi vé máy bay mỗi thứ Bảy từ 14h-17h; đặt khách sạn giờ vàng EPIC Hotel Hour Deal diễn ra hàng ngày từ 18h-19h. Du khách có thể săn vé máy bay quốc nội và quốc tế với giá ưu đãi. Trong đó, vé nội địa Vietravel giá chỉ từ 781.925 đồng; vé China Southern Airlines đi Thâm Quyến từ 2,819 đồng; vé T'way Air đến Hàn Quốc và Nhật Bản lần lượt chỉ từ 2,667 triệu đồng và 2,682 triệu đồng. Khách hàng còn có cơ hội nghỉ dưỡng tại khách sạn 5 sao trong nước với giá từ 794.000 đồng. Hàng loạt khách sạn Hàn Quốc giá từ 1,858 triệu đồng, Nhật Bản từ 1,146 triệu đồng. Với dịch vụ giải trí, nền tảng áp dụng ưu đãi 'mua 1 tặng 1' vé tham quan Sun World, công viên nước The Amazing Bay, thủy cung Sea Life Bangkok Ocean World (Thái Lan). Để du khách có trải nghiệm du lịch trọn vẹn, Traveloka giới thiệu thêm nhiều tính năng khác như: hoàn tiền 100%, thay đổi lịch trình, thanh toán linh hoạt... Xem thêm thông tin chi tiết về chương trình Epic Sale trên ứng dụng, website và các tài khoản mạng xã hội của Traveloka. Á Hiên",
+  "summary": "781.925 đồng vé Vietravel, 2.819 triệu Thâm Quyến; 2.667 và 2.682 triệu Hàn Quốc-Nhật Bản. Khách sạn từ 794.000-1.858 triệu. Áp dụng 'mua 1 tặng 1' Sun World, The Amazing Bay, Sea Life Bangkok Ocean World. Hoàn tiền 100%, thay đổi lịch trình, thanh toán linh hoạt trên Traveloka. Epic Sale của Ninh Dương Lan Ngọc mong muốn lan tỏa tinh thần du lịch thông minh và áp dụng ưu đãi đến 50% cho các sản phẩm toàn thế giới nhằm tri ân khách hàng và khích lệ khám phá thế giới qua những chuyến đi tiện nghi với chi phí tiết kiệm.",
+  "faithfulness_score": 0.8,
+  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng có thể thiếu một số chi tiết quan trọng như việc hợp tác giữa Traveloka và Ninh Dương Lan Ngọc, cũng như một số thông tin về các dịch vụ và ưu đãi cụ thể.",
+  "relevance_score": 0.7,
+  "relevance_reason": "Bản tóm tắt bao gồm một số ý chính như giá vé máy bay, khách sạn và các ưu đãi, nhưng có thể bỏ sót một số thông điệp cốt lõi như sứ mệnh của Traveloka và tầm ảnh hưởng của Ninh Dương Lan Ngọc.",
+  "coherence_conciseness_score": 0.9,
+  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, tuy nhiên có thể có một số từ ngữ lặp lại hoặc không cần thiết, nhưng tổng thể vẫn rõ ràng và súc tích."
+}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
up code chay dc
</commit_message>
<xml_diff>
--- a/Thư mục KQ/VB sau tóm tắt/test_results.xlsx
+++ b/Thư mục KQ/VB sau tóm tắt/test_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,7 +453,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Taste Studio của Regent Hotels &amp; Resorts tổ chức với chủ đề 'Dáng hình của biển', giới hạn 20 khách mời mỗi tối. Sự kiện quy tụ nhiều đầu bếp và nghệ sĩ nổi tiếng, từ Mr. Dripping (drip art) đến Francesco (Milan), Huân Trần (Regent Phú Quốc) và Andy Huỳnh (Oku). Regent Phú Quốc mong muốn tiếp tục kiến tạo trải nghiệm đưa nét bản địa đặc sắc lên bản đồ thế giới cho khách hàng hạng sang.</t>
+          <t>Regent Hotels &amp; Resorts tổ chức Taste Studio với chủ đề 'Dáng hình của biển', quy tụ nhiều đầu bếp và nghệ sĩ nổi tiếng, giới hạn 20 khách mời mỗi tối.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -462,13 +462,13 @@
   "id": 1,
   "style": "news_brief",
   "article": "Taste Studio do thương hiệu Regent Hotels &amp; Resorts tổ chức nhằm mang đến trải nghiệm đa giác quan qua ẩm thực và nghệ thuật. Sự kiện này quy tụ nhiều đầu bếp và nghệ sĩ nổi tiếng, từ nhà thiết kế thời trang đến nhạc sĩ, kết hợp cùng các thương hiệu hàng đầu như Vietnam Airlines. Sự kiện hướng đến phân khúc khách hàng sang trọng. Mùa một và hai diễn ra lần được vào tháng 4, tháng 11 năm ngoái. Taste Studio năm nay với chủ đề 'Dáng hình của biển', giới hạn 20 khách mời mỗi tối. Các khách mời được tham gia vào chuỗi khám phá gồm 7 chương đặc sắc về vẻ đẹp của biển, qua lăng kính nghệ sĩ tài hoa Mr. Dripping - nghệ sĩ vẽ tranh bằng phương pháp nhỏ giọt (drip art). Không gian nhà hàng, nơi diễn ra sự kiện với nội thất dùng tre, mây và tầm vông do kiến trúc sư Nguyễn Trung Nghĩa thiết kế. Ngoài hai nghệ sĩ này, Taste Studio còn có sự tham gia của bếp trưởng Francesco đến từ Milan, với 20 năm kinh nghiệm làm việc tại các khách sạn danh tiếng thế giới, đang bắt đầu hành trình mới tại Việt Nam. Ông đảm nhận vai trò cố vấn ẩm thực tại Regent Phú Quốc, mang đến trải nghiệm độc đáo cho thực khách. Bên cạnh đó, phó bếp trưởng điều hành Huân Trần tại chương trình mong muốn chinh phục các hương vị vùng miền khác nhau. Được nếm nhiều nguyên liệu địa phương và các loại gia vị đặc biệt, vị đầu bếp để lại điểm nhấn riêng trong cách giữ gìn, nâng tầm phong vị của quê hương tại Regent Phú Quốc. Chương trình có sự góp mặt của bếp trưởng nhà hàng Oku - Andy Huỳnh. Trước khi gia nhập Regent Phú Quốc, anh phát triển kỹ thuật nấu ăn Nhật Bản tại Nobu, San Diego và Nassau. Các món ăn của Andy luôn mang ý nghĩa hướng về cội nguồn. Bếp trưởng nhà hàng Ocean Club Daniel và bếp trưởng Duyến Nguyễn của khu nghỉ dưỡng này cũng tham gia, sáng tạo một số hương vị độc đáo từ nguyên liệu địa phương. Đại diện Regent Phú Quốc cho biết, thông qua Taste Studio, đơn vị mong muốn tiếp tục kiến tạo trải nghiệm đưa nét bản địa đặc sắc của Việt Nam lên bản đồ thế giới, từ đó chinh phục khách hàng hạng sang và giới chuyên gia. Thanh Thư",
-  "summary": "Taste Studio của Regent Hotels &amp; Resorts tổ chức với chủ đề 'Dáng hình của biển', giới hạn 20 khách mời mỗi tối. Sự kiện quy tụ nhiều đầu bếp và nghệ sĩ nổi tiếng, từ Mr. Dripping (drip art) đến Francesco (Milan), Huân Trần (Regent Phú Quốc) và Andy Huỳnh (Oku). Regent Phú Quốc mong muốn tiếp tục kiến tạo trải nghiệm đưa nét bản địa đặc sắc lên bản đồ thế giới cho khách hàng hạng sang.",
-  "faithfulness_score": 0.9,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, nhưng có bỏ sót một số chi tiết quan trọng như sự tham gia của các thương hiệu hàng đầu và kiến trúc sư Nguyễn Trung Nghĩa",
-  "relevance_score": 0.8,
-  "relevance_reason": "Bản tóm tắt bao hàm các ý chính quan trọng, nhưng bỏ sót thông điệp về việc Regent Phú Quốc muốn chinh phục khách hàng hạng sang và giới chuyên gia",
+  "summary": "Regent Hotels &amp; Resorts tổ chức Taste Studio với chủ đề 'Dáng hình của biển', quy tụ nhiều đầu bếp và nghệ sĩ nổi tiếng, giới hạn 20 khách mời mỗi tối.",
+  "faithfulness_score": 0.8,
+  "faithfulness_reason": "Tóm tắt không thêm thông tin sai lệch nhưng bỏ qua một số chi tiết quan trọng như sự tham gia của các thương hiệu hàng đầu và nghệ sĩ tài năng",
+  "relevance_score": 0.6,
+  "relevance_reason": "Tóm tắt chỉ đề cập đến chủ đề của sự kiện và giới hạn khách mời, nhưng bỏ qua các thông tin quan trọng về mục tiêu của chương trình và sự tham gia của các đầu bếp nổi tiếng",
   "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, nhưng có thể rút gọn một số chi tiết để tăng tính súc tích"
+  "coherence_conciseness_reason": "Tóm tắt ngắn gọn, dễ đọc và không có thông tin trùng lặp, tuy nhiên có thể cải thiện bằng cách thêm một số chi tiết quan trọng để làm cho tóm tắt trở nên đầy đủ hơn"
 }</t>
         </is>
       </c>
@@ -481,7 +481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Amiana Resort Nha Trang tiếp tục nhận hai giải thưởng quốc tế: 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới', nổi bật với kiến trúc tự nhiên kết hợp công nghệ, bãi biển riêng tư xanh mát, hồ bơi và vườn bảo vệ môi trường.</t>
+          <t>Amiana Resort Nha Trang tiếp tục nhận hai giải thưởng 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới', sau 4 năm liên tiếp. Phong cách hòa hợp giữa truyền thống và hiện đại tạo không gian thư giãn gần gũi thiên nhiên, biệt thự có cửa sổ lớn và ban công rộng, hồ bơi riêng tư và vườn nhiệt đới xanh mát. Resort chú trọng bảo vệ môi trường bằng giải pháp bền vững.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,13 +490,13 @@
   "id": 2,
   "style": "news_brief",
   "article": "Hai giải thưởng gồm 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới'. Đây cũng là năm thứ tư liên tiếp đơn vị đạt giải thưởng này, sau quá trình thẩm định từ hội đồng chuyên môn toàn cầu và bình chọn bởi hàng nghìn du khách, khách sạn quốc tế khác. 'Giải thưởng góp phần khẳng định Amiana Resort Nha Trang là điểm đến lý tưởng cho du khách tìm kiếm không gian riêng tư, gần gũi thiên nhiên với kiến trúc cao cấp, mang lại trải nghiệm sang trọng, độc đáo', đại diện resort chia sẻ. Amiana có kiến trúc hòa hợp thiên nhiên, kết hợp yếu tố truyền thống và hiện đại, tạo nên không gian thư giãn, sang trọng nhưng vẫn giữ được cảm giác gần gũi, yên bình. Bãi biển riêng tư với hàng dừa rợp bóng xanh mát là nơi du khách có thể thư giãn, nghỉ ngơi thoải mái. Resort còn tận dụng địa hình tự nhiên để bố trí các công trình công cộng như hồ bơi, nhà hàng, phòng hội nghị, spa... Các yếu tố đậm chất nhiệt đới như dừa xanh, sóng biển, đá và gỗ được lồng ghép khéo léo trong từng chi tiết thiết kế nội ngoại thất. Biệt thự, phòng nghỉ, nhà hàng đều có sự kết hợp giữa vật liệu tự nhiên và công nghệ hiện đại. Mỗi căn biệt thự đều mang kiến trúc mở, sử dụng nội thất chủ yếu từ gỗ, đá tự nhiên. Tất cả phòng đều có cửa sổ lớn và ban công rộng, tối ưu tầm nhìn hướng biển với cảnh quan thiên nhiên vây quanh. Biệt thự còn có hồ bơi riêng, không gian vườn với các loại cây nhiệt đới, đảm bảo yếu tố riêng tư cho khách hàng. Resort không chỉ chú trọng xây dựng công trình tiện ích, mà còn đặc biệt lưu ý việc bảo vệ môi trường, sử dụng các giải pháp bền vững. Những không gian xanh, vườn cây, hồ nước đều được bố trí hợp lý, tạo nên hệ sinh thái tự nhiên trong lòng khu nghỉ dưỡng. Theo đại diện Amiana Resort Nha Trang, những chi tiết kiến trúc thông minh cùng không gian mở, vật liệu tự nhiên, sự khéo léo trong thiết kế tại đây góp phần tạo nên khu nghỉ dưỡng lý tưởng cho những ai tìm kiếm sự an yên, lãng mạn và xa hoa. Á Hiên",
-  "summary": "Amiana Resort Nha Trang tiếp tục nhận hai giải thưởng quốc tế: 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới', nổi bật với kiến trúc tự nhiên kết hợp công nghệ, bãi biển riêng tư xanh mát, hồ bơi và vườn bảo vệ môi trường.",
+  "summary": "Amiana Resort Nha Trang tiếp tục nhận hai giải thưởng 'Khu nghỉ dưỡng có thiết kế kiến trúc tốt nhất thế giới' và 'Khu nghỉ dưỡng hướng biển lãng mạn sang trọng nhất thế giới', sau 4 năm liên tiếp. Phong cách hòa hợp giữa truyền thống và hiện đại tạo không gian thư giãn gần gũi thiên nhiên, biệt thự có cửa sổ lớn và ban công rộng, hồ bơi riêng tư và vườn nhiệt đới xanh mát. Resort chú trọng bảo vệ môi trường bằng giải pháp bền vững.",
   "faithfulness_score": 0.9,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, nhưng có thể thiếu một số chi tiết quan trọng như việc Amiana Resort Nha Trang đạt giải thưởng này lần thứ tư liên tiếp và quá trình thẩm định từ hội đồng chuyên môn toàn cầu",
+  "faithfulness_reason": "Tóm tắt không thêm thông tin sai lệch, nhưng có thể làm rõ hơn về quá trình thẩm định và bình chọn của hội đồng chuyên môn toàn cầu",
   "relevance_score": 0.8,
-  "relevance_reason": "Bản tóm tắt bao hàm các ý chính quan trọng như giải thưởng, kiến trúc và môi trường, nhưng có thể bỏ sót thông điệp cốt lõi về sự kết hợp giữa vật liệu tự nhiên và công nghệ hiện đại",
+  "relevance_reason": "Tóm tắt đã bao gồm các điểm chính về giải thưởng và thiết kế của khu nghỉ dưỡng, nhưng bỏ qua một số chi tiết quan trọng như hệ sinh thái tự nhiên và sự kết hợp giữa vật liệu tự nhiên và công nghệ hiện đại",
   "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, nhưng có thể loại bỏ một số từ ngữ không cần thiết để tăng tính súc tích"
+  "coherence_conciseness_reason": "Tóm tắt được viết một cách rõ ràng, logic và dễ đọc, tuy nhiên có thể rút gọn một số câu để tăng độ súc tích"
 }</t>
         </is>
       </c>
@@ -509,7 +509,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Gỗ lũa từ sông Tiền tạo nên khu du lịch Cồn Én, với tiểu cảnh, đài quan sát và bức tranh điêu khắc dài 24 m. Du khách đến TP HCM qua quốc lộ 30 hoặc phà Tấn Long thăm đảo này với giá vé 80.000 đồng, nơi người dân đã biến hàng nghìn thân gỗ lũa thành điểm tham quan yên bình.</t>
+          <t>Cồn Én nằm giữa sông Tiền, thuộc xã Tấn Mỹ. Nơi đây là điểm đến ngắm dòng Tiền Giang và đón gió mát dịu. Du khách còn được tham quan khu du lịch sinh thái với bộ sưu tập gỗ lũa độc đáo. Gỗ lũa lấy từ đáy sông, sau khi bị bào mòn chỉ còn phần lõi bền chắc. Khu du lịch này có tiểu cảnh và nhà nghỉ làm bằng vật liệu chính là những thân cây khủng này. Một bức tranh điêu khắc dài hơn 24m nặng 20 tấn được thực hiện trên khúc gỗ trầm thủy, tùy từng đoạn chiều cao từ 1,5 - 1,8 m. Cạnh đó còn có bộ sưu tập hàng trăm chiếc xe máy biển số độc lạ và tiểu cảnh làm từ gỗ lũa. Du khách cũng ngắm hoàng hôn trên sông tại đây. Giá vé vào cổng là 80.000 đồng.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -518,13 +518,13 @@
   "id": 3,
   "style": "news_brief",
   "article": "Cồn Én nằm giữa sông Tiền, thuộc xã Tấn Mỹ, rộng hơn 300 ha. Nơi đây ngoài là điểm đến ngắm dòng Tiền Giang, đón gió sông mát dịu, còn là địa chỉ thu hút khách với bộ sưu tập gỗ lũa nội thất độc đáo của khu du lịch trên cồn. Gỗ lũa tức những thân cây khủng, vớt từ đáy sông, bên ngoài bị dòng nước bào mòn, chỉ còn phần lõi bền chắc. Hàng nghìn thân gỗ lũa được người chủ tuyển chọn làm vật liệu chính xây Khu du lịch sinh thái Cồn Én từ tiểu cảnh, nhà đến đài quan sát. Hơn 20 năm trước, ông Nguyễn Văn Nghỉ ở huyện Chợ Mới đã sưu tập rất nhiều gỗ lũa. Ban đầu ông trục vớt chúng để khơi thông dòng chảy, hạn chế tình trạng lưới đánh cá mắc vào thân cây. Lâu dần, ông yêu mến và muốn lưu giữ những thân gỗ trầm thủy này. Ba năm trước, ông Nghỉ dùng số gỗ lũa để xây khu du lịch ven sông Tiền rộng 6 ha. Đặc sắc trong các vật liệu từ gỗ lũa là bức tranh điêu khắc về phong cảnh làng quê Việt Nam xưa dài hơn 24 m, nặng 20 tấn. Bức tranh do nghệ nhân ở Huế thực hiện trong 7 năm, trên khúc gỗ trầm thủy khủng, tùy từng đoạn có chiều cao từ 1,5 - 1,8 m. Cạnh bức tranh là bộ sưu tập hàng trăm chiếc xe máy biển số độc lạ như tứ quý, sảnh tiến tới của nhiều dòng xe nổi tiếng. Dọc các lối đi là những tiểu cảnh làm từ gỗ lũa. Một số được điêu khắc thành các con vật, chim muông. Những cây gỗ lũa kích thước lớn được tận dụng làm đài quan sát cao 26 m, hoặc móng trụ để xây nhà nghỉ, cầu vượt. Khuôn viên cũng được phủ bởi nhiều cây kiểng, dừa cùng dãy nhà sàn ven sông. Tại đây du khách được ngắm hoàng hôn trên sông, tắm sông và thưởng thức ẩm thực miền Tây. Chị Phúc Điền, du khách ở TP HCM, cho biết khá thích với khung cảnh miền Tây yên bình ở Cồn Én. Chị cũng bất ngờ với sự kỳ công của người đã sưu tập hàng nghìn thân gỗ lũa và biến chúng thành điểm tham quan độc đáo. Cồn Én, nằm cách TP HCM 170 km, du khách có thể đến đây từ hướng quốc lộ 30 của tỉnh Đồng Tháp hoặc lên phà Tấn Long vượt sông Tiền từ phía huyện Chợ Mới. Giá vé vào cổng là 80.000 đồng. Ngọc Tài",
-  "summary": "Gỗ lũa từ sông Tiền tạo nên khu du lịch Cồn Én, với tiểu cảnh, đài quan sát và bức tranh điêu khắc dài 24 m. Du khách đến TP HCM qua quốc lộ 30 hoặc phà Tấn Long thăm đảo này với giá vé 80.000 đồng, nơi người dân đã biến hàng nghìn thân gỗ lũa thành điểm tham quan yên bình.",
-  "faithfulness_score": 0.8,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin nhưng có thiếu sót một số chi tiết quan trọng như vị trí của Cồn Én, diện tích khu du lịch và một số hoạt động du lịch khác",
-  "relevance_score": 0.7,
-  "relevance_reason": "Bản tóm tắt chưa bao hàm đủ các ý chính quan trọng nhất như vị trí địa lý, các hoạt động du lịch và đặc điểm nổi bật của khu du lịch Cồn Én",
+  "summary": "Cồn Én nằm giữa sông Tiền, thuộc xã Tấn Mỹ. Nơi đây là điểm đến ngắm dòng Tiền Giang và đón gió mát dịu. Du khách còn được tham quan khu du lịch sinh thái với bộ sưu tập gỗ lũa độc đáo. Gỗ lũa lấy từ đáy sông, sau khi bị bào mòn chỉ còn phần lõi bền chắc. Khu du lịch này có tiểu cảnh và nhà nghỉ làm bằng vật liệu chính là những thân cây khủng này. Một bức tranh điêu khắc dài hơn 24m nặng 20 tấn được thực hiện trên khúc gỗ trầm thủy, tùy từng đoạn chiều cao từ 1,5 - 1,8 m. Cạnh đó còn có bộ sưu tập hàng trăm chiếc xe máy biển số độc lạ và tiểu cảnh làm từ gỗ lũa. Du khách cũng ngắm hoàng hôn trên sông tại đây. Giá vé vào cổng là 80.000 đồng.",
+  "faithfulness_score": 0.9,
+  "faithfulness_reason": "Tóm tắt không thêm thông tin sai lệch, nhưng thiếu một số chi tiết quan trọng như diện tích của khu du lịch và quá trình sưu tập gỗ lũa của ông Nguyễn Văn Nghỉ",
+  "relevance_score": 0.8,
+  "relevance_reason": "Tóm tắt bao gồm các điểm chính như vị trí, đặc điểm của gỗ lũa và hoạt động du lịch, nhưng bỏ qua một số thông tin quan trọng như vị trí của Cồn Én so với TP HCM và cách di chuyển đến đó",
   "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt có mạch lạc, logic và dễ đọc, tuy nhiên có thể cải thiện bằng cách thêm một số chi tiết quan trọng và tránh trùng lặp thông tin"
+  "coherence_conciseness_reason": "Tóm tắt được viết một cách rõ ràng, logic và dễ đọc, tuy nhiên có thể rút gọn một số câu để tăng độ súc tích"
 }</t>
         </is>
       </c>
@@ -535,27 +535,8 @@
           <t>Văn phòng mới của MayTrip tại địa chỉ 833 Lê Hồng Phong, quận 10, nhằm mở rộng dịch vụ và nâng cao trải nghiệm khách hàng khu vực phía Nam. Văn phòng mới được kỳ vọng là điểm đến thuận tiện cho khách hàng trong việc tìm hiểu và sử dụng dịch vụ của công ty. Trong ngày khai trương, MayTrip trao tặng nhiều quà tặng và ưu đãi cho khách tham dự. Các voucher gồm: 2 triệu đồng cho khách đăng ký tour Bắc Á trong ba ngày khai trương, 1 triệu đồng cho tour Đông Nam Á trong ba tháng từ ngày khai trương, 500.000 đồng cho dịch vụ tour nội địa trong một năm, 200.000 đồng dịch vụ đặt phòng khách sạn hoặc xe du lịch trong 6 tháng và 100.000 đồng với dịch vụ vé máy bay trong 6 tháng. Buổi lễ khai trương văn phòng tại Sài Gòn còn giới thiệu các chương trìnhtour Nhật Bảndịp Tết Âm lịch như cung đường vàng trải nghiệm trượt tuyết, Hokkaido - miền tuyết trắng. Những chuyến đi này được MayTrip thiết kế kỹ lưỡng, phù hợp với không khí đón xuân cho gia đình và cặp đôi Việt trong dịp Tết Nguyên đán. Năm nay, MayTrip xác định tour Hokkaido là sản phẩm 'đinh' trong dịp Tết Nguyên đán. Hokkaido nằm ở miền Bắc Nhật Bản, nổi tiếng với những đợt tuyết dày và phong cảnh mùa đông đặc trưng. Tour Hokkaido dịp Tết là hành trình lý tưởng để du khách tận hưởng kỳ nghỉ theo cách mới mẻ và ấn tượng trong tuyết trắng. Bên cạnh đó, tour Hokkaido của MayTrip cũng mang đến trải nghiệm suối nước nóng onsen giữa băng tuyết, giúp du khách thư giãn sau những hoạt động trong ngày. Bên cạnh đó, MayTrip cũng cung cấp các tour du lịch khác với lịch khởi hành linh hoạt kéo dài đến hết năm 2025, gồm hành trình ngắm hoa anh đào, hoa mơ, mận và nghỉ lễ 30/4 và 1/5. Các hành trình này dựa trên xu hướng và sở thích của du khách Việt Nam. Theo đại diện công ty, sự kiện khai trương văn phòng mới tại TP HCM đánh dấu bước phát triển mới của MayTrip. Với mục tiêu ưu tiên trải nghiệm khách hàng, đơn vị hy vọng nhận được sự ủng hộ từ khách hàng để trở thành công ty lữ hành hàng đầu, hướng mục tiêu thương hiệu toàn cầu vào năm 2030. Ngoài TP HCM, MayTrip còn có văn phòng tại Hải Phòng và TP Vinh. Các văn phòng này giúp MayTrip dễ dàng tiếp cận và đáp ứng nhu cầu đa dạng của khách hàng. Công ty cam kết đảm bảo chất lượng dịch vụ để mang lại chuyến đi an toàn, trọn vẹn cho khách hàng. Thanh Thư</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MayTrip khai trương văn phòng mới tại 833 Lê Hồng Phong, quận 10 (TP HCM), với ưu đãi và tour Hokkaido dịp Tết Nguyên đán. Công ty đặt mục tiêu trở thành công ty lữ hành hàng đầu toàn cầu vào năm 2030, cam kết chất lượng dịch vụ an toàn cho khách.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>{
-  "id": 4,
-  "style": "news_brief",
-  "article": "Văn phòng mới của MayTrip tại địa chỉ 833 Lê Hồng Phong, quận 10, nhằm mở rộng dịch vụ và nâng cao trải nghiệm khách hàng khu vực phía Nam. Văn phòng mới được kỳ vọng là điểm đến thuận tiện cho khách hàng trong việc tìm hiểu và sử dụng dịch vụ của công ty. Trong ngày khai trương, MayTrip trao tặng nhiều quà tặng và ưu đãi cho khách tham dự. Các voucher gồm: 2 triệu đồng cho khách đăng ký tour Bắc Á trong ba ngày khai trương, 1 triệu đồng cho tour Đông Nam Á trong ba tháng từ ngày khai trương, 500.000 đồng cho dịch vụ tour nội địa trong một năm, 200.000 đồng dịch vụ đặt phòng khách sạn hoặc xe du lịch trong 6 tháng và 100.000 đồng với dịch vụ vé máy bay trong 6 tháng. Buổi lễ khai trương văn phòng tại Sài Gòn còn giới thiệu các chương trìnhtour Nhật Bảndịp Tết Âm lịch như cung đường vàng trải nghiệm trượt tuyết, Hokkaido - miền tuyết trắng. Những chuyến đi này được MayTrip thiết kế kỹ lưỡng, phù hợp với không khí đón xuân cho gia đình và cặp đôi Việt trong dịp Tết Nguyên đán. Năm nay, MayTrip xác định tour Hokkaido là sản phẩm 'đinh' trong dịp Tết Nguyên đán. Hokkaido nằm ở miền Bắc Nhật Bản, nổi tiếng với những đợt tuyết dày và phong cảnh mùa đông đặc trưng. Tour Hokkaido dịp Tết là hành trình lý tưởng để du khách tận hưởng kỳ nghỉ theo cách mới mẻ và ấn tượng trong tuyết trắng. Bên cạnh đó, tour Hokkaido của MayTrip cũng mang đến trải nghiệm suối nước nóng onsen giữa băng tuyết, giúp du khách thư giãn sau những hoạt động trong ngày. Bên cạnh đó, MayTrip cũng cung cấp các tour du lịch khác với lịch khởi hành linh hoạt kéo dài đến hết năm 2025, gồm hành trình ngắm hoa anh đào, hoa mơ, mận và nghỉ lễ 30/4 và 1/5. Các hành trình này dựa trên xu hướng và sở thích của du khách Việt Nam. Theo đại diện công ty, sự kiện khai trương văn phòng mới tại TP HCM đánh dấu bước phát triển mới của MayTrip. Với mục tiêu ưu tiên trải nghiệm khách hàng, đơn vị hy vọng nhận được sự ủng hộ từ khách hàng để trở thành công ty lữ hành hàng đầu, hướng mục tiêu thương hiệu toàn cầu vào năm 2030. Ngoài TP HCM, MayTrip còn có văn phòng tại Hải Phòng và TP Vinh. Các văn phòng này giúp MayTrip dễ dàng tiếp cận và đáp ứng nhu cầu đa dạng của khách hàng. Công ty cam kết đảm bảo chất lượng dịch vụ để mang lại chuyến đi an toàn, trọn vẹn cho khách hàng. Thanh Thư",
-  "summary": "MayTrip khai trương văn phòng mới tại 833 Lê Hồng Phong, quận 10 (TP HCM), với ưu đãi và tour Hokkaido dịp Tết Nguyên đán. Công ty đặt mục tiêu trở thành công ty lữ hành hàng đầu toàn cầu vào năm 2030, cam kết chất lượng dịch vụ an toàn cho khách.",
-  "faithfulness_score": 0.9,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, nhưng có thể thêm chi tiết về các ưu đãi và tour du lịch để tăng tính trung thực",
-  "relevance_score": 0.8,
-  "relevance_reason": "Bản tóm tắt bao gồm các ý chính quan trọng, nhưng có thể bỏ sót thông điệp cốt lõi về mục tiêu của công ty và các văn phòng khác",
-  "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, nhưng có thể rút gọn một số chi tiết để tăng tính súc tích"
-}</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -564,22 +545,7 @@
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>{
-  "id": 5,
-  "style": "news_brief",
-  "article": "Ngày 29/10, tại Khu du lịch Sun World Fansipan Legend, Hiệp hội Du lịch tỉnh Lào Cai công bố chương trình kích cầu du lịch lớn nhất năm với chủ đề 'Chạm Sa Pa - Chạm những tầng mây', diễn ra từ 2/11 đến 30/12. Trong thời gian này, 130 doanh nghiệp tại Sa Pa sẽ cung cấp nhiều ưu đãi lên đến 50% và cam kết đảm bảo chất lượng dịch vụ. Theo đó, Công ty Cáp treo Fansipan Sa Pa (Khu du lịch Sun World Fansipan Legend) áp dụng đồng giá vé cáp treo hai chiều Fansipan chỉ còn 550.000 đồng cho du khách Việt Nam. Mức giá này giảm 30% so với giá gốc. Du khách có thể khám phá đỉnh Fansipan, chiêm ngưỡng kiến trúc tâm linh và tham gia các hoạt động văn hóa của 7 dân tộc thiểu số Tây Bắc tại Bản Mây. Nhiều điểm du lịch khác tại Sa Pa cũng miễn phí vé tham quan và cung cấp ưu đãi hấp dẫn. Trong đó, vườn đá Tả Phìn và vườn hồng Mộng Mơ miễn phí vé, Khu du lịch Cát Cát miễn phí trải nghiệm ẩm thực Tây Bắc cùng các hoạt động vẽ sáp ong, xe lanh, dệt vải... với bà con dân bản. Các khách sạn như Chaulong Sapa, Amazing Sapa, Vườn Sa Pa, Arista Sa Pa và Le Bordeaux Sapa áp dụng giảm giá phòng trực tiếp tới 50%. Hotel de la Coupole và Lady Hill Sapa Resort có nhiều ưu đãi về dịch vụ ăn uống, spa. Một số nhà xe như Inter Bus Lines và Eco Sa Pa cũng giảm giá vé xe khứ hồi đến 30%, cung cấp đa dạng hình thức di chuyển từ xe limousine đến xe lớn. Ông Phạm Cao Vỹ, đại diện Hiệp hội Du lịch tỉnh Lào Cai nhấn mạnh sự cần thiết của việc kích cầu du lịch để phục hồi ngành sau ảnh hưởng nặng nề của bão lũ. Ông kêu gọi tất cả doanh nghiệp du lịch trên địa bàn tham gia nhằm tạo sức bật cho du lịch Sa Pa phát triển mạnh mẽ vào giai đoạn cuối năm 2024. Ông Nguyễn Xuân Chiến, Phó chủ tịch Sun Group Vùng Miền Bắc, cho biết trước đây chương trình kích cầu 'Đến Sa Pa - Bay giữa mùa hoa' thành công ngoài mong đợi. 'Lần này, thông qua chính sách ưu đãi sâu, chúng tôi hy vọng thu hút đông đảo du khách đến Sa Pa để khám phá vẻ đẹp độc đáo của mùa mây', ông Chiến nói. Ngoài chính sách ưu đãi sâu, tỉnh Lào Cai và thị xã Sa Pa tổ chức nhiều sự kiện văn hóa đặc sắc nhằm mang đến trải nghiệm độc đáo cho du khách. Các hoạt động bao gồm lễ hội truyền thống, triển lãm nghệ thuật, thể thao và giải trí. Đặc biệt là sự kiện ánh sáng 3D Mapping và lễ hội hoa sen đá lần đầu tiên được tổ chức tại Sun World Fansipan Legend. Sa Pa đang trong mùa mây - thời điểm lý tưởng để vui chơi ngoài trời. Ban tổ chức kỳ vọng chương trình kích cầu sẽ tăng sức hút của Sa Pa và củng cố vị thế là điểm đến hàng đầu miền Bắc. Thanh Thư",
-  "summary": "",
-  "faithfulness_score": 1.0,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, không sai số liệu và không xuyên tạc ý nghĩa của văn bản gốc.",
-  "relevance_score": 1.0,
-  "relevance_reason": "Bản tóm tắt bao hàm đủ các ý chính quan trọng nhất, không bỏ sót thông điệp cốt lõi nào.",
-  "coherence_conciseness_score": 1.0,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic, dễ đọc và loại bỏ được các chi tiết rườm rà/lặp từ không."
-}</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -587,27 +553,8 @@
           <t>Brisbane nằm phía đông nam bang Queensland, là thành phố lớn thứ ba tại Australia. Do gần đường xích đạo, khí hậu nơi đây ôn hòa, quanh năm nắng ấm. Trung tâm Brisbane không chỉ có những khối bê tông, khu mua sắm, mà còn bao phủ bởi mảng xanh, với 5 công viên và vườn thực vật nổi tiếng. Dưới đây là 5 điểm đến hút du khách ở Brisbane. South Bank Parklands Nằm bên bờ sông Brisbane, South Bank Parklands được ví như 'ốc đảo xanh' giữa lòng thành phố sôi động, nổi bật với rừng mưa nhiệt đới và loạt hoạt động giải trí cho mọi lứa tuổi. Ngay cửa ngõ công viên là thảm cỏ, hàng cây rợp bóng và vườn hoa. Nhiều người dân thường picnic, dã ngoại, vui chơi tại bãi biển nhân tạo Streets Beach, River Quay Green, Rainforest Green hay Liana Lounge. Ngoài ra, Wheel of Brisbane - vòng đu quay cao tới 60 m - là biểu tượng tại South Bank Parklands, dễ dàng ngắm toàn cảnh Brisbane từ trên cao. Roma Street Parkland Nằm cạnh ga xe lửa Roma Street, công viên cùng tên cũng được người dân lẫn du khách gọi là 'ốc đảo xanh mát' giữa Brisbane, ghi dấu với những khu vườn và bãi cỏ rộng lớn. Tại đây, du khách hòa mình vào khu vườn Spectacle - nơi trồng hàng nghìn gốc violets, cẩm chướng, delphiniums và foxgloves. Khí hậu ôn hòa thu hút chim kookaburras, gà lôi, vẹt. Bạn cũng có thể tổ chức tiệc BBQ ngoài trời, cho con khám phá công viên trẻ em. Brisbane City Botanic Gardens Nằm trên trục đường Alice, Brisbane City Botanic Gardens bảo tồn hàng nghìn loài thực vật quý hiếm, nổi bật với vẻ nguyên sơ. Khu vườn này là một trong những điểm đến lý tưởng cho người chuộng nét thanh bình giữa lòng đô thị. Tại đây, du khách có thể khám phá con đường dạo bộ ven sông, chiêm ngưỡng rặng thông Bunya được trồng từ năm 1858. Điểm đến tiếp theo là Bamboo Grove - con đường tre rợp mát, được ví như 'khu rừng xa xôi giữa thành phố hiện đại'. Vườn bách thảo tổ chức sự kiện quanh năm như biểu diễn Riverstage, lễ hội đa văn hóa, trưng bày nghệ thuật cùng hoạt động cộng đồng miễn phí. Trong đó, chợ Riverside Sunday Market hút hàng nghìn du khách nhờ gian hàng thủ công, trái cây tươi và ẩm thực độc đáo. Epicurious Garden Tại Epicurious, du khách có thể khám phá ẩm thực bang Queensland đa dạng, nhất là rau, củ, quả, thảo mộc hữu cơ theo mùa. 14 chuyên viên tình nguyện chăm sóc khu vườn kỹ lưỡng, mong truyền cảm hứng cho người yêu nấu ăn và trồng trọt. 'Tới Epicurious, tôi và bạn bè được hướng dẫn cách chăm sóc rau củ, trái cây, thảo mộc và thưởng thức miễn phí', một du khách viết trên Facebook, nhận hàng trăm nghìn lượt thích. Mount Coot-tha Botanic Gardens Mở cửa đón khách từ năm 1976, Mount Coot-tha Botanic Gardens tọa lạc chân núi Coot-tha, là vườn thực vật nhiệt đới hàng đầu Brisbane, diện tích đến 56 ha. Dạo quanh khu vườn, du khách có thể chiêm ngưỡng hoa xuân, các loài cây nhiệt đới và khu thảo dược. Nơi đây là điểm đến quen thuộc của người yêu thiên nhiên, picnic, mê hoạt động thể chất, với đường chạy bộ thoáng đãng. Để khám phá thành thủ phủ bang Queensland, bạn có thể chọn đường bay thẳng từ TP HCM đến Brisbane của Vietjet, với 9 giờ trên máy bay thân rộng, thoải mái cùng loạt dịch vụ tiện ích, ưu đãi như: bảo hiểm Sky Care miễn phí, chương trình tích điểm SkyJoy, đổi quà từ hơn 250 thương hiệu lớn toàn cầu. Trước đó ngày14-15/9, Vietjet đồng hành lễ hội thả diều Vietjet Redcliffe KiteFest tại Redcliffe, Queensland. Hãng hàng không Việt còn áp dụng nhiều chương trình ưu đãi nhân dịp đón hành khách thứ 200 triệu. Đông Vệ</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Brisbane, thành phố lớn thứ ba của Australia với khí hậu ôn hòa quanh năm. Thành phố có nhiều công viên và vườn thực vật nổi tiếng như South Bank Parklands, Roma Street Parkland và Brisbane City Botanic Gardens bảo tồn hàng nghìn loài cây quý hiếm trên trục đường Alice. Hội chợ Riverside Sunday Market hút du khách với gian hàng thủ công, trái cây tươi và ẩm thực độc đáo. Epicurious Garden giới thiệu ẩm thực Queensland đa dạng. Mount Coot-tha Botanic Gardens nằm trên núi Coot-tha, là vườn thực vật lớn của Brisbane. Vietjet cung cấp đường bay thẳng TP HCM - Brisbane với nhiều dịch vụ tiện ích và chương trình ưu đãi nhân dịp đón hành khách thứ 200 triệu.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>{
-  "id": 6,
-  "style": "news_brief",
-  "article": "Brisbane nằm phía đông nam bang Queensland, là thành phố lớn thứ ba tại Australia. Do gần đường xích đạo, khí hậu nơi đây ôn hòa, quanh năm nắng ấm. Trung tâm Brisbane không chỉ có những khối bê tông, khu mua sắm, mà còn bao phủ bởi mảng xanh, với 5 công viên và vườn thực vật nổi tiếng. Dưới đây là 5 điểm đến hút du khách ở Brisbane. South Bank Parklands Nằm bên bờ sông Brisbane, South Bank Parklands được ví như 'ốc đảo xanh' giữa lòng thành phố sôi động, nổi bật với rừng mưa nhiệt đới và loạt hoạt động giải trí cho mọi lứa tuổi. Ngay cửa ngõ công viên là thảm cỏ, hàng cây rợp bóng và vườn hoa. Nhiều người dân thường picnic, dã ngoại, vui chơi tại bãi biển nhân tạo Streets Beach, River Quay Green, Rainforest Green hay Liana Lounge. Ngoài ra, Wheel of Brisbane - vòng đu quay cao tới 60 m - là biểu tượng tại South Bank Parklands, dễ dàng ngắm toàn cảnh Brisbane từ trên cao. Roma Street Parkland Nằm cạnh ga xe lửa Roma Street, công viên cùng tên cũng được người dân lẫn du khách gọi là 'ốc đảo xanh mát' giữa Brisbane, ghi dấu với những khu vườn và bãi cỏ rộng lớn. Tại đây, du khách hòa mình vào khu vườn Spectacle - nơi trồng hàng nghìn gốc violets, cẩm chướng, delphiniums và foxgloves. Khí hậu ôn hòa thu hút chim kookaburras, gà lôi, vẹt. Bạn cũng có thể tổ chức tiệc BBQ ngoài trời, cho con khám phá công viên trẻ em. Brisbane City Botanic Gardens Nằm trên trục đường Alice, Brisbane City Botanic Gardens bảo tồn hàng nghìn loài thực vật quý hiếm, nổi bật với vẻ nguyên sơ. Khu vườn này là một trong những điểm đến lý tưởng cho người chuộng nét thanh bình giữa lòng đô thị. Tại đây, du khách có thể khám phá con đường dạo bộ ven sông, chiêm ngưỡng rặng thông Bunya được trồng từ năm 1858. Điểm đến tiếp theo là Bamboo Grove - con đường tre rợp mát, được ví như 'khu rừng xa xôi giữa thành phố hiện đại'. Vườn bách thảo tổ chức sự kiện quanh năm như biểu diễn Riverstage, lễ hội đa văn hóa, trưng bày nghệ thuật cùng hoạt động cộng đồng miễn phí. Trong đó, chợ Riverside Sunday Market hút hàng nghìn du khách nhờ gian hàng thủ công, trái cây tươi và ẩm thực độc đáo. Epicurious Garden Tại Epicurious, du khách có thể khám phá ẩm thực bang Queensland đa dạng, nhất là rau, củ, quả, thảo mộc hữu cơ theo mùa. 14 chuyên viên tình nguyện chăm sóc khu vườn kỹ lưỡng, mong truyền cảm hứng cho người yêu nấu ăn và trồng trọt. 'Tới Epicurious, tôi và bạn bè được hướng dẫn cách chăm sóc rau củ, trái cây, thảo mộc và thưởng thức miễn phí', một du khách viết trên Facebook, nhận hàng trăm nghìn lượt thích. Mount Coot-tha Botanic Gardens Mở cửa đón khách từ năm 1976, Mount Coot-tha Botanic Gardens tọa lạc chân núi Coot-tha, là vườn thực vật nhiệt đới hàng đầu Brisbane, diện tích đến 56 ha. Dạo quanh khu vườn, du khách có thể chiêm ngưỡng hoa xuân, các loài cây nhiệt đới và khu thảo dược. Nơi đây là điểm đến quen thuộc của người yêu thiên nhiên, picnic, mê hoạt động thể chất, với đường chạy bộ thoáng đãng. Để khám phá thành thủ phủ bang Queensland, bạn có thể chọn đường bay thẳng từ TP HCM đến Brisbane của Vietjet, với 9 giờ trên máy bay thân rộng, thoải mái cùng loạt dịch vụ tiện ích, ưu đãi như: bảo hiểm Sky Care miễn phí, chương trình tích điểm SkyJoy, đổi quà từ hơn 250 thương hiệu lớn toàn cầu. Trước đó ngày14-15/9, Vietjet đồng hành lễ hội thả diều Vietjet Redcliffe KiteFest tại Redcliffe, Queensland. Hãng hàng không Việt còn áp dụng nhiều chương trình ưu đãi nhân dịp đón hành khách thứ 200 triệu. Đông Vệ",
-  "summary": "Brisbane, thành phố lớn thứ ba của Australia với khí hậu ôn hòa quanh năm. Thành phố có nhiều công viên và vườn thực vật nổi tiếng như South Bank Parklands, Roma Street Parkland và Brisbane City Botanic Gardens bảo tồn hàng nghìn loài cây quý hiếm trên trục đường Alice. Hội chợ Riverside Sunday Market hút du khách với gian hàng thủ công, trái cây tươi và ẩm thực độc đáo. Epicurious Garden giới thiệu ẩm thực Queensland đa dạng. Mount Coot-tha Botanic Gardens nằm trên núi Coot-tha, là vườn thực vật lớn của Brisbane. Vietjet cung cấp đường bay thẳng TP HCM - Brisbane với nhiều dịch vụ tiện ích và chương trình ưu đãi nhân dịp đón hành khách thứ 200 triệu.",
-  "faithfulness_score": 0.8,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng có bỏ sót một số chi tiết quan trọng như mô tả cụ thể về các hoạt động giải trí tại South Bank Parklands và Roma Street Parkland",
-  "relevance_score": 0.9,
-  "relevance_reason": "Bản tóm tắt bao hàm đủ các ý chính quan trọng nhất về các điểm đến hút du khách ở Brisbane, tuy nhiên có thể thêm thông tin về các sự kiện và hoạt động tại các công viên",
-  "coherence_conciseness_score": 0.7,
-  "coherence_conciseness_reason": "Bản tóm tắt có logic và dễ đọc nhưng có thể cải thiện bằng cách loại bỏ các từ ngữ lặp từ và sắp xếp lại cấu trúc câu cho rõ ràng hơn"
-}</t>
-        </is>
-      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -616,22 +563,7 @@
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>{
-  "id": 7,
-  "style": "news_brief",
-  "article": "Công ty du lịch NhatbanAZ mở bán chùm tour Nhật Bản khởi hành dịp Tết Dương lịch và Âm lịch từ đầu tháng 10. Trong đó, các tour truyền thống đến Osaka, Kyoto và Tokyo được làm mới bằng những hoạt động phù hợp với mùa đông xuân như trượt tuyết tại Fujiten Resort, ngắm tuyết làng cổ Oshino Hakkai và tham gia lễ hội ánh sáng Nabana no sato. NhatbanAZ cũng mở rộng các cung đường mới cho du khách trải nghiệm trong dịp Tết 2025. Cụ thể, tour Hokkaido gồm Asahikawa, Monbetsu và Sapporo với giá 55,9 triệu đồng mỗi khách. Du khách sẽ tham gia câu cá trên băng, đi tàu phá băng và thưởng thức bia hơi tại Sapporo, cùng dịch vụ hàng không 5 sao và lưu trú khách sạn 4 sao quốc tế. Tour thứ hai là chuyến thăm làng cổ Shirakawago, núi Phú Sĩ và Tokyo trong 6 ngày 5 đêm với giá 31,9 triệu đồng mỗi khách. Du khách sẽ được chiêm ngưỡng tuyết trắng tại Shirakawago, một Di sản Văn hóa Thế giới của UNESCO từ năm 1995. Tour cũng gồm tham quan lâu đài Matsumoto - di tích bảo vật quốc gia của Nhật Bản và trải nghiệm trượt tuyết tại Fujiten Snow Resort - top 3 khu trượt tuyết nổi tiếng. Bà Hồ Như Thảo, Giám đốc Điều hành NhatbanAZ Văn phòng TP HCM cho biết sản phẩm mới này nhận được sự quan tâm lớn từ du khách, đặc biệt là những người từng đi Nhật và muốn trở lại với hành trình mới. Khu vực Hokkaido được biết đến với tuyết rơi dày đặc hơn Tokyo hay Osaka, nên lịch khởi hành tour Hokkaido dịp Tết Âm lịch nhận được nhiều đăng ký giữ chỗ. Trong dịp Tết Nguyên đán 2025, NhatbanAZ cung cấp các hành trình từ 5 đến 6 ngày với mức giá cơ bản đến cao cấp, khoảng 31,9 - 55,9 triệu đồng mỗi khách để đáp ứng nhu cầu đa dạng. Giá tour Tết có phần chênh lệch so với ngày thường và tăng so với cùng kỳ năm trước. Do đó, NhatbanAZ chủ động gặp gỡ và làm việc với các đối tác cung cấp dịch vụ, từ đó xây dựng chương trình, đưa ra chính sách ưu đãi tốt nhất cho khách hàng. Với kinh nghiệm hơn 15 năm trong ngành du lịch chuyên thị trường Nhật Bản, NhatbanAZ thuộc danh sách công ty chỉ định nộp visa bởi Đại sứ quán Nhật Bản đề xuất. Đồng thời là đối tác chiến lược của các hãng hàng không, khách sạn và đối tác land tour uy tín tại Nhật Bản. Công ty cũng là nhà tư vấn và tổ chức những chuyến Famtrip kết nối các công ty du lịch Việt Nam tới tham quan xúc tiến đầu tư, hợp tác tại Nhật Bản. Thanh Thư",
-  "summary": "",
-  "faithfulness_score": 1.0,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, sai số liệu, hay xuyên tạc ý nghĩa của văn bản gốc",
-  "relevance_score": 1.0,
-  "relevance_reason": "Bản tóm tắt bao hàm đủ các ý chính quan trọng nhất và không bỏ sót thông điệp cốt lõi nào",
-  "coherence_conciseness_score": 1.0,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic, dễ đọc và loại bỏ được các chi tiết rườm rà/lặp từ không"
-}</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -639,27 +571,8 @@
           <t>Theo bảng xếp hạng 20 quốc gia tốt nhất thế giới năm 2024 (The Best Countries in the World) do tạp chí du lịch Mỹ Condé Nast Traveler công bố vào tháng 10, Việt Nam ở vị trí 15 với 89 điểm. Một điểm đến khác thuộc Đông Nam Á có mặt trong danh sách này là Thái Lan, xếp thứ ba với 92,29 điểm. Đứng đầu top 20 là Nhật Bản với 95,32 điểm. Xếp hạng nằm trong giải thưởng thường niênReaders' Choice Awards của tạp chí Mỹ, dựa trên đánh giá của hơn 575.000 độc giả về các trải nghiệm du lịch ở mỗi quốc gia, xét theo các tiêu chí văn hóa, cảnh quan, dịch vụ du lịch và cơ sở hạ tầng. Độc giả của Condé Nast Traveler nhận xét Việt Nam thu hút du khách nhờ vẻ đẹp mộc mạc và quyến rũ. 'Với lượng khách nước ngoài đang trên đà tăng từ 2019 đến nay, Việt Nam không còn là điểm đến đáng chú ý mà thành điểm đến đáng ghé thăm', biên tập tờ Condé Nast Traveler viết. Theo số liệu từ Tổng cục Thống kê, trong 9 tháng đầu năm, Việt Nam đón hơn 12,7 triệu lượt khách quốc tế, vượt lượng khách cả năm 2023 là 12,6 triệu lượt. Lượng khách quốc tế đến Việt Nam tăng trưởng tích cực 9 tháng đầu năm 2024, với một số thị trường phục hồi hoàn toàn, tăng mạnh so với 2019, theo Cục Du lịch Quốc gia. Cục cũng dự đoán với đà tăng trường như hiện nay, Việt Nam sẽ hoàn thành mục tiêu đón 17-18 triệu lượt khách quốc tế năm 2024. Thái Lan được tạp chí Mỹ nhận xét là quốc gia đa dạng cảnh quan, giao thông thuận tiện với nhiều tàu thuyền, xe buýt đêm và chuyến bay nội địa giá rẻ. Ẩm thực cũng là điểm sáng của xứ chùa Vàng khi có nhiều khu chợ đêm nhộn nhịp, bày bán đặc sản địa phương. 8 tháng đầu năm 2024, Thái Lan đón hơn 20 triệu lượt khách quốc tế, tăng 34% so với cùng kỳ năm trước. Quốc gia này đặt mục tiêu đón ít nhất 36-37 triệu lượt khách nước ngoài trong cả năm nay, kỳ vọng thu về khoảng 3.500 tỷ baht (95,5 tỷ USD). Condé Nast Traveler là tạp chí du lịch nổi tiếng toàn cầu, ra mắt vào năm 1987. Các bảng xếp hạng của Condé Nast Traveler như Readers' Choice Awards được chuyên gia du lịch đánh giá là uy tín vì dựa trên ý kiến từ hàng triệu độc giả quốc tế. Bích Phương(TheoCNTraveller)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>LỖI: 'NoneType' object is not iterable</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>{
-  "id": 8,
-  "style": "news_brief",
-  "article": "Theo bảng xếp hạng 20 quốc gia tốt nhất thế giới năm 2024 (The Best Countries in the World) do tạp chí du lịch Mỹ Condé Nast Traveler công bố vào tháng 10, Việt Nam ở vị trí 15 với 89 điểm. Một điểm đến khác thuộc Đông Nam Á có mặt trong danh sách này là Thái Lan, xếp thứ ba với 92,29 điểm. Đứng đầu top 20 là Nhật Bản với 95,32 điểm. Xếp hạng nằm trong giải thưởng thường niênReaders' Choice Awards của tạp chí Mỹ, dựa trên đánh giá của hơn 575.000 độc giả về các trải nghiệm du lịch ở mỗi quốc gia, xét theo các tiêu chí văn hóa, cảnh quan, dịch vụ du lịch và cơ sở hạ tầng. Độc giả của Condé Nast Traveler nhận xét Việt Nam thu hút du khách nhờ vẻ đẹp mộc mạc và quyến rũ. 'Với lượng khách nước ngoài đang trên đà tăng từ 2019 đến nay, Việt Nam không còn là điểm đến đáng chú ý mà thành điểm đến đáng ghé thăm', biên tập tờ Condé Nast Traveler viết. Theo số liệu từ Tổng cục Thống kê, trong 9 tháng đầu năm, Việt Nam đón hơn 12,7 triệu lượt khách quốc tế, vượt lượng khách cả năm 2023 là 12,6 triệu lượt. Lượng khách quốc tế đến Việt Nam tăng trưởng tích cực 9 tháng đầu năm 2024, với một số thị trường phục hồi hoàn toàn, tăng mạnh so với 2019, theo Cục Du lịch Quốc gia. Cục cũng dự đoán với đà tăng trường như hiện nay, Việt Nam sẽ hoàn thành mục tiêu đón 17-18 triệu lượt khách quốc tế năm 2024. Thái Lan được tạp chí Mỹ nhận xét là quốc gia đa dạng cảnh quan, giao thông thuận tiện với nhiều tàu thuyền, xe buýt đêm và chuyến bay nội địa giá rẻ. Ẩm thực cũng là điểm sáng của xứ chùa Vàng khi có nhiều khu chợ đêm nhộn nhịp, bày bán đặc sản địa phương. 8 tháng đầu năm 2024, Thái Lan đón hơn 20 triệu lượt khách quốc tế, tăng 34% so với cùng kỳ năm trước. Quốc gia này đặt mục tiêu đón ít nhất 36-37 triệu lượt khách nước ngoài trong cả năm nay, kỳ vọng thu về khoảng 3.500 tỷ baht (95,5 tỷ USD). Condé Nast Traveler là tạp chí du lịch nổi tiếng toàn cầu, ra mắt vào năm 1987. Các bảng xếp hạng của Condé Nast Traveler như Readers' Choice Awards được chuyên gia du lịch đánh giá là uy tín vì dựa trên ý kiến từ hàng triệu độc giả quốc tế. Bích Phương(TheoCNTraveller)",
-  "summary": "LỖI: 'NoneType' object is not iterable",
-  "faithfulness_score": 0.0,
-  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin gì về văn bản gốc, không có nội dung để đánh giá tính trung thực.",
-  "relevance_score": 0.0,
-  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không thể đánh giá tính bao quát.",
-  "coherence_conciseness_score": 0.0,
-  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá tính mạch lạc và súc tích."
-}</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -667,27 +580,8 @@
           <t>Theo KTO Việt Nam, 8 tháng năm nay, Hàn Quốc đón 389.000 lượt khách Việt, tăng 27% so với cùng kỳ năm 2023. Số lượng khách Việt Nam đến Hàn Quốc dự kiến tăng mạnh hơn bởi đất nước này đang bước vào mùa lá vàng đẹp nhất năm. Đại diện KTO khẳng định, Việt Nam là thị trường quan trọng với ngành du lịch Hàn Quốc với nhiều sự kiện tổ chức thành công. Cụ thể, trong năm nay, KTO Việt Nam xúc tiến các chương trình quảng bá, phát triển sản phẩm du lịch Hàn Quốc phù hợp với nhu cầu du khách Việt. Kết quả, nhiều sản phẩm du lịch mới được ra mắt thị trường trong nước như: tour du lịch Hàn Quốc kết hợp giải chạy Marathon tại Gyeongju và Jeju, tour trải nghiệm Esports, tour lễ hội đèn lồng truyền thống Yeondeunghoe hay tour đạp xe đạp đường dài khám phá Hàn Quốc... Chương trình Năm du lịch Hàn Quốc 2023-2024 (Visit Korea Year 2023-2024) do Tổng cục du lịch Hàn Quốc (KTO) triển khai cũng mang đến những hoạt động mới mẻ, quảng bá du lịch Hàn Quốc đến cộng đồng quốc tế. Bên cạnh đó, nhằm mang đến những trải nghiệm chân thực và đậm chất bản địa, KTO tổ chức nhiều famtour. Nổi bật là famtour trải nghiệm Esports cùng các KOL hàng đầu làng thể thao điện tử như: SofM, reviewer Duy Thẩm, Hải Triều, streamer Hà Tiều Phu, BLV Esports nổi tiếng Văn Tùng, Hoàng Luân, kết hợp Box Esports. Làn sóng văn hóa Hallyu cũng được lồng ghép vào sản phẩm du lịch, khi hàng loạt tên tuổi lớn đến Việt Nam trong khuôn khổ sự kiện Korea Travel Festa, tổ chức tháng 5 vừa qua. Mới nhất, KTO Việt Nam có mặt tại Hội chợ Du lịch Quốc tế (ITE) TP HCM, mang theo không gian đặc trưng Hàn Quốc cùng nhiều trải nghiệm mới mẻ, độc đáo. Nắm bắt nhu cầu du lịch Hàn Quốc tăng cao trong mùa cuối năm của du khách Việt, KTO Việt Nam tiếp tục đẩy mạnh các chương trình ưu đãi đặc biệt. Cùng các đối tác, công ty du lịch hàng đầu Việt Nam, KTO góp phần phát triển nhiều tuyến điểm mới trong hành trình du lịch Hàn Quốc, mang đến đa dạng lựa chọn và nhiều trải nghiệm cho khách hàng. Hồi tháng 5, KTO Việt Nam ký kết thỏa thuận hợp tác cùng Tập đoàn Vingroup, nhằm thúc đẩy hơn nữa sự giao lưu, trao đổi du lịch giữa hai nước. Theo đó, KTO triển khai chiến dịch hỗ trợ dành riêng cho khách hàng thuộc hệ sinh thái Vingroup khi mua tour du lịch Hàn Quốc từ tháng 10 đến tháng 12 Cụ thể, chủ sở hữu xe Vinfast, cư dân Vinhomes, nhân viên Vingroup) và hội viên Vinclub (gọi chung là Vintizen) sẽ nhận được mức giá ưu đãi đặc biệt từ các công ty du lịch và KTO Việt Nam. Bên cạnh mức giá ưu đãi từ các công ty du lịch, Vintizen có cơ hội áp dụng đồng thời voucher trị giá một triệu đồng mỗi khách hàng, mua tối đa 5 tour du lịch Hàn Quốc để nhận voucher lên đến 5 triệu đồng từ KTO Việt Nam, trong thời gian 1-10/10. Ngoài thời gian trên, du khách mua tour tại các đối tác du lịch sẽ nhận được nhiều phần quà Hàn Quốc từ KTO Việt Nam. Thanh Thư</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Hàn Quốc đón 389.000 lượt khách Việt Nam tăng 27% nhờ mùa lá vàng đẹp nhất năm và chương trình quảng bá du lịch mới, trong đó Vintizen hưởng ưu đãi giảm giá tour từ tháng 10 đến tháng 12 với voucher trị giá một triệu đồng mỗi khách hàng.</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>{
-  "id": 9,
-  "style": "news_brief",
-  "article": "Theo KTO Việt Nam, 8 tháng năm nay, Hàn Quốc đón 389.000 lượt khách Việt, tăng 27% so với cùng kỳ năm 2023. Số lượng khách Việt Nam đến Hàn Quốc dự kiến tăng mạnh hơn bởi đất nước này đang bước vào mùa lá vàng đẹp nhất năm. Đại diện KTO khẳng định, Việt Nam là thị trường quan trọng với ngành du lịch Hàn Quốc với nhiều sự kiện tổ chức thành công. Cụ thể, trong năm nay, KTO Việt Nam xúc tiến các chương trình quảng bá, phát triển sản phẩm du lịch Hàn Quốc phù hợp với nhu cầu du khách Việt. Kết quả, nhiều sản phẩm du lịch mới được ra mắt thị trường trong nước như: tour du lịch Hàn Quốc kết hợp giải chạy Marathon tại Gyeongju và Jeju, tour trải nghiệm Esports, tour lễ hội đèn lồng truyền thống Yeondeunghoe hay tour đạp xe đạp đường dài khám phá Hàn Quốc... Chương trình Năm du lịch Hàn Quốc 2023-2024 (Visit Korea Year 2023-2024) do Tổng cục du lịch Hàn Quốc (KTO) triển khai cũng mang đến những hoạt động mới mẻ, quảng bá du lịch Hàn Quốc đến cộng đồng quốc tế. Bên cạnh đó, nhằm mang đến những trải nghiệm chân thực và đậm chất bản địa, KTO tổ chức nhiều famtour. Nổi bật là famtour trải nghiệm Esports cùng các KOL hàng đầu làng thể thao điện tử như: SofM, reviewer Duy Thẩm, Hải Triều, streamer Hà Tiều Phu, BLV Esports nổi tiếng Văn Tùng, Hoàng Luân, kết hợp Box Esports. Làn sóng văn hóa Hallyu cũng được lồng ghép vào sản phẩm du lịch, khi hàng loạt tên tuổi lớn đến Việt Nam trong khuôn khổ sự kiện Korea Travel Festa, tổ chức tháng 5 vừa qua. Mới nhất, KTO Việt Nam có mặt tại Hội chợ Du lịch Quốc tế (ITE) TP HCM, mang theo không gian đặc trưng Hàn Quốc cùng nhiều trải nghiệm mới mẻ, độc đáo. Nắm bắt nhu cầu du lịch Hàn Quốc tăng cao trong mùa cuối năm của du khách Việt, KTO Việt Nam tiếp tục đẩy mạnh các chương trình ưu đãi đặc biệt. Cùng các đối tác, công ty du lịch hàng đầu Việt Nam, KTO góp phần phát triển nhiều tuyến điểm mới trong hành trình du lịch Hàn Quốc, mang đến đa dạng lựa chọn và nhiều trải nghiệm cho khách hàng. Hồi tháng 5, KTO Việt Nam ký kết thỏa thuận hợp tác cùng Tập đoàn Vingroup, nhằm thúc đẩy hơn nữa sự giao lưu, trao đổi du lịch giữa hai nước. Theo đó, KTO triển khai chiến dịch hỗ trợ dành riêng cho khách hàng thuộc hệ sinh thái Vingroup khi mua tour du lịch Hàn Quốc từ tháng 10 đến tháng 12 Cụ thể, chủ sở hữu xe Vinfast, cư dân Vinhomes, nhân viên Vingroup) và hội viên Vinclub (gọi chung là Vintizen) sẽ nhận được mức giá ưu đãi đặc biệt từ các công ty du lịch và KTO Việt Nam. Bên cạnh mức giá ưu đãi từ các công ty du lịch, Vintizen có cơ hội áp dụng đồng thời voucher trị giá một triệu đồng mỗi khách hàng, mua tối đa 5 tour du lịch Hàn Quốc để nhận voucher lên đến 5 triệu đồng từ KTO Việt Nam, trong thời gian 1-10/10. Ngoài thời gian trên, du khách mua tour tại các đối tác du lịch sẽ nhận được nhiều phần quà Hàn Quốc từ KTO Việt Nam. Thanh Thư",
-  "summary": "Hàn Quốc đón 389.000 lượt khách Việt Nam tăng 27% nhờ mùa lá vàng đẹp nhất năm và chương trình quảng bá du lịch mới, trong đó Vintizen hưởng ưu đãi giảm giá tour từ tháng 10 đến tháng 12 với voucher trị giá một triệu đồng mỗi khách hàng.",
-  "faithfulness_score": 0.8,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng có thể thiếu chính xác khi không đề cập đầy đủ đến các chương trình quảng bá du lịch và sự kiện cụ thể",
-  "relevance_score": 0.7,
-  "relevance_reason": "Bản tóm tắt bao gồm một số ý chính nhưng bỏ sót thông tin quan trọng về các sản phẩm du lịch mới và chương trình Năm du lịch Hàn Quốc 2023-2024",
-  "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, tuy nhiên có thể rút gọn một số chi tiết để tăng tính súc tích"
-}</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -695,27 +589,8 @@
           <t>Diễn đàn năm nay là sự kiện trọng điểm do UBND tỉnh Kiên Giang phối hợp Bộ Nông nghiệp và Phát triển nông thôn tổ chức. Công ty Cổ phần Truyền Thông Vương Hậu (TP HCM) là đơn vị phụ trách tổ chức. Với chủ đề 'Liên kết cùng phát triển - Kiên Giang 2024', diễn đàn hướng đến tăng cường hợp tác, liên kết giữa các tỉnh, thành phố trong vùng Đồng bằng sông Cửu Long với các Bộ, ngành Trung ương, các địa phương khác trên cả nước. Từ đó, các bên có thêm cơ sở đẩy mạnh, phát huy tiềm năng về sản phẩm OCOP của vùng. Đến nay, đã có trên 35 tỉnh, thành phố đăng ký tham gia diễn đàn cùng hơn 300 nhà đầu tư đến tìm hiểu cơ hội, xúc tiến hợp tác kinh doanh. Diễn đàn dự kiến thu hút khoảng 50.000-100.000 khách tham quan suốt thời gian diễn ra. Hơn 320 gian hàng từ các tỉnh ĐBSCL và cả nước sẽ cùng trưng bày, giới thiệu các sản phẩm OCOP tiêu biểu, công nghiệp nông thôn, đặc sản địa phương. Ngoài chương trình chính, sự kiện còn bao gồm chuỗi hoạt động khác như: triển lãm sản phẩm OCOP; hội thi 'Sản phẩm OCOP tiêu biểu ĐBSCL 2024'; các hội nghị, hội thảo, ký kết biên bản hợp tác... Đặc biệt, khách tham dự còn được tìm hiểu quy trình sản xuất nước mắm truyền thống Phú Quốc, một trong những đặc sản nổi tiếng của Kiên Giang. Buổi tối, diễn dàn có các chương trình ca nhạc với sự góp mặt của các ca sĩ, nghệ sĩ nổi tiếng. Diễn đàn kết nối sản phẩm OCOP là sự kiện thường niên do Bộ Nông nghiệp và Phát triển nông thôn phối hợp UBND các tỉnh, thành phố vùng Đồng bằng sông Cửu Long tổ chức quy mô cấp vùng. Đây vừa là nơi giao lưu, kết nối kinh doanh, vừa là cơ hội để các sản phẩm này vươn ra thế giới, góp phần phát triển kinh tế nông nghiệp, xây dựng nông thôn mới bền vững. Á Hiên</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Diễn đàn năm nay là sự kiện trọng điểm do UBND tỉnh Kiên Giang phối hợp với Bộ Nông nghiệp và Phát triển nông thôn tổ chức. Công ty Cổ phần Truyền Thông Vương Hậu (TP HCM) phụ trách việc tổ chức. Chủ đề của diễn đàn là 'Liên kết cùng phát triển - Kiên Giang 2024', hướng đến tăng cường hợp tác giữa các tỉnh, thành phố trong vùng Đồng bằng sông Cửu Long với Bộ ngành Trung ương và địa phương khác trên cả nước. Diễn đàn đã thu hút hơn 35 tỉnh/thành phố đăng ký tham gia cùng gần 300 nhà đầu tư tìm hiểu cơ hội xúc tiến hợp tác kinh doanh, dự kiến sẽ có khoảng 50-100 nghìn khách tham quan và trưng bày hơn 320 gian hàng từ các tỉnh ĐBSCL và cả nước. Ngoài chương trình chính như triển lãm sản phẩm OCOP, hội thi 'Sản phẩm OCOP tiêu biểu ĐBSCL 2024', diễn đàn còn có chuỗi hoạt động khác gồm: ký kết biên bản hợp tác, ca nhạc với sự góp mặt của các nghệ sĩ nổi tiếng. Đây là sự kiện thường niên do Bộ Nông nghiệp và Phát triển nông thôn phối hợp UBND các tỉnh/thành phố vùng Đồng bằng sông Cửu Long tổ chức, vừa giúp giao lưu kinh doanh vừa tạo cơ hội cho sản phẩm OCOP vươn ra thế giới.</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>{
-  "id": 10,
-  "style": "news_brief",
-  "article": "Diễn đàn năm nay là sự kiện trọng điểm do UBND tỉnh Kiên Giang phối hợp Bộ Nông nghiệp và Phát triển nông thôn tổ chức. Công ty Cổ phần Truyền Thông Vương Hậu (TP HCM) là đơn vị phụ trách tổ chức. Với chủ đề 'Liên kết cùng phát triển - Kiên Giang 2024', diễn đàn hướng đến tăng cường hợp tác, liên kết giữa các tỉnh, thành phố trong vùng Đồng bằng sông Cửu Long với các Bộ, ngành Trung ương, các địa phương khác trên cả nước. Từ đó, các bên có thêm cơ sở đẩy mạnh, phát huy tiềm năng về sản phẩm OCOP của vùng. Đến nay, đã có trên 35 tỉnh, thành phố đăng ký tham gia diễn đàn cùng hơn 300 nhà đầu tư đến tìm hiểu cơ hội, xúc tiến hợp tác kinh doanh. Diễn đàn dự kiến thu hút khoảng 50.000-100.000 khách tham quan suốt thời gian diễn ra. Hơn 320 gian hàng từ các tỉnh ĐBSCL và cả nước sẽ cùng trưng bày, giới thiệu các sản phẩm OCOP tiêu biểu, công nghiệp nông thôn, đặc sản địa phương. Ngoài chương trình chính, sự kiện còn bao gồm chuỗi hoạt động khác như: triển lãm sản phẩm OCOP; hội thi 'Sản phẩm OCOP tiêu biểu ĐBSCL 2024'; các hội nghị, hội thảo, ký kết biên bản hợp tác... Đặc biệt, khách tham dự còn được tìm hiểu quy trình sản xuất nước mắm truyền thống Phú Quốc, một trong những đặc sản nổi tiếng của Kiên Giang. Buổi tối, diễn dàn có các chương trình ca nhạc với sự góp mặt của các ca sĩ, nghệ sĩ nổi tiếng. Diễn đàn kết nối sản phẩm OCOP là sự kiện thường niên do Bộ Nông nghiệp và Phát triển nông thôn phối hợp UBND các tỉnh, thành phố vùng Đồng bằng sông Cửu Long tổ chức quy mô cấp vùng. Đây vừa là nơi giao lưu, kết nối kinh doanh, vừa là cơ hội để các sản phẩm này vươn ra thế giới, góp phần phát triển kinh tế nông nghiệp, xây dựng nông thôn mới bền vững. Á Hiên",
-  "summary": "Diễn đàn năm nay là sự kiện trọng điểm do UBND tỉnh Kiên Giang phối hợp với Bộ Nông nghiệp và Phát triển nông thôn tổ chức. Công ty Cổ phần Truyền Thông Vương Hậu (TP HCM) phụ trách việc tổ chức. Chủ đề của diễn đàn là 'Liên kết cùng phát triển - Kiên Giang 2024', hướng đến tăng cường hợp tác giữa các tỉnh, thành phố trong vùng Đồng bằng sông Cửu Long với Bộ ngành Trung ương và địa phương khác trên cả nước. Diễn đàn đã thu hút hơn 35 tỉnh/thành phố đăng ký tham gia cùng gần 300 nhà đầu tư tìm hiểu cơ hội xúc tiến hợp tác kinh doanh, dự kiến sẽ có khoảng 50-100 nghìn khách tham quan và trưng bày hơn 320 gian hàng từ các tỉnh ĐBSCL và cả nước. Ngoài chương trình chính như triển lãm sản phẩm OCOP, hội thi 'Sản phẩm OCOP tiêu biểu ĐBSCL 2024', diễn đàn còn có chuỗi hoạt động khác gồm: ký kết biên bản hợp tác, ca nhạc với sự góp mặt của các nghệ sĩ nổi tiếng. Đây là sự kiện thường niên do Bộ Nông nghiệp và Phát triển nông thôn phối hợp UBND các tỉnh/thành phố vùng Đồng bằng sông Cửu Long tổ chức, vừa giúp giao lưu kinh doanh vừa tạo cơ hội cho sản phẩm OCOP vươn ra thế giới.",
-  "faithfulness_score": 0.9,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thêm thông tin, nhưng có một số chi tiết được tóm tắt không đầy đủ như việc khách tham dự có thể tìm hiểu quy trình sản xuất nước mắm truyền thống Phú Quốc",
-  "relevance_score": 0.8,
-  "relevance_reason": "Bản tóm tắt bao hàm đủ các ý chính quan trọng, nhưng có thể thêm thông tin về mục tiêu của diễn đàn và ý nghĩa của việc tăng cường hợp tác giữa các tỉnh, thành phố",
-  "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, nhưng có thể rút gọn một số câu để tăng tính súc tích"
-}</t>
-        </is>
-      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -723,27 +598,8 @@
           <t>Bên lề đường khu vực Chiêm Mai, nơi có nhiều xưởng làm gốm, các mặt hàng bị ngâm nước vẫn còn bùn đất bám lại. Những sản phẩm còn sử dụng được người dân mang ra phơi nắng. Bên lề đường khu vực Chiêm Mai, nơi có nhiều xưởng làm gốm, các mặt hàng bị ngâm nước vẫn còn bùn đất bám lại. Những sản phẩm còn sử dụng được người dân mang ra phơi nắng. Trong chợ gốm, nhiều cửa hàng quây bạt, chưa mở cửa lại. 'Nhiều chủ hàng chưa mở lại do phải dọn dẹp nhà cửa bị ngập trước đó, chưa có thời gian dọn cửa hàng', chị Tuyết, chủ một cửa hàng, nói. Trong chợ gốm, nhiều cửa hàng quây bạt, chưa mở cửa lại. 'Nhiều chủ hàng chưa mở lại do phải dọn dẹp nhà cửa bị ngập trước đó, chưa có thời gian dọn cửa hàng', chị Tuyết, chủ một cửa hàng, nói. Chị Lan, chủ một cửa hàng trong chợ, cho biết nhà chị không bị thiệt hại nặng nên dọn hàng ra sớm để đón khách. 'Ngày thường ít khách lui tới nhưng đông vào dịp cuối tuần', chị Lan nói. Chị Lan, chủ một cửa hàng trong chợ, cho biết nhà chị không bị thiệt hại nặng nên dọn hàng ra sớm để đón khách. 'Ngày thường ít khách lui tới nhưng đông vào dịp cuối tuần', chị Lan nói. Cửa hàng nặn gốm của chị Lan đã sẵn sàng đón khách hàng đến trải nghiệm. Cửa hàng nặn gốm của chị Lan đã sẵn sàng đón khách hàng đến trải nghiệm. Các gian hàng mở lại với lác đác du khách tới tham quan, mua sắm - trái với khung cảnh tấp nập mỗi dịp lễ, Tết khi mặt hàng gốm sứ được nhiều người tìm mua. Các gian hàng mở lại với lác đác du khách tới tham quan, mua sắm - trái với khung cảnh tấp nập mỗi dịp lễ, Tết khi mặt hàng gốm sứ được nhiều người tìm mua. Bảo tàng gốm Bát Tràng nằm gần ngoài đê, trước khi vào làng gốm, cũng đã mở cửa sẵn sàng đón khách. Bảo tàng được xây dựng từ năm 2018 với kinh phí 150 tỷ đồng, là 'trung tâm tinh hoa làng nghề Việt'. Bảo tàng gốm Bát Tràng nằm gần ngoài đê, trước khi vào làng gốm, cũng đã mở cửa sẵn sàng đón khách. Bảo tàng được xây dựng từ năm 2018 với kinh phí 150 tỷ đồng, là 'trung tâm tinh hoa làng nghề Việt'. Bên trong bảo tàng có thiết kế độc đáo, nhiều tầng với các chuyên đề khác nhau về lịch sử hình thành, phát triển cũng như các loại hình gốm tại Bát Tràng. 'Đến làng gốm để có trải nghiệm thú vị, thay đổi không khí và tìm hiểu về gốm truyền thống', Phạm Hoàng Hiệu, Thanh Xuân, Hà Nội, cho biết khi đến đây sau những ngày phải ở nhà vì mưa lụt. Bên trong bảo tàng có thiết kế độc đáo, nhiều tầng với các chuyên đề khác nhau về lịch sử hình thành, phát triển cũng như các loại hình gốm tại Bát Tràng. 'Đến làng gốm để có trải nghiệm thú vị, thay đổi không khí và tìm hiểu về gốm truyền thống', Phạm Hoàng Hiệu, Thanh Xuân, Hà Nội, cho biết khi đến đây sau những ngày phải ở nhà vì mưa lụt. Đình làng Bát Tràng hơn 300 tuổi không bị ảnh hưởng sau trận lụt. Đình được coi là 'báu vật đi cùng năm tháng' ở làng, hiện lưu giữ hơn 50 đạo sắc phong. Đình Bát Tràng được Bộ Văn hóa Thể thao và Du lịch cấp bằng Di tích văn hóa kiến trúc nghệ thuật năm 2005. Đình làng Bát Tràng hơn 300 tuổi không bị ảnh hưởng sau trận lụt. Đình được coi là 'báu vật đi cùng năm tháng' ở làng, hiện lưu giữ hơn 50 đạo sắc phong. Đình Bát Tràng được Bộ Văn hóa Thể thao và Du lịch cấp bằng Di tích văn hóa kiến trúc nghệ thuật năm 2005. Hoàng Giang</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>LỖI: 'NoneType' object is not iterable</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>{
-  "id": 11,
-  "style": "news_brief",
-  "article": "Bên lề đường khu vực Chiêm Mai, nơi có nhiều xưởng làm gốm, các mặt hàng bị ngâm nước vẫn còn bùn đất bám lại. Những sản phẩm còn sử dụng được người dân mang ra phơi nắng. Bên lề đường khu vực Chiêm Mai, nơi có nhiều xưởng làm gốm, các mặt hàng bị ngâm nước vẫn còn bùn đất bám lại. Những sản phẩm còn sử dụng được người dân mang ra phơi nắng. Trong chợ gốm, nhiều cửa hàng quây bạt, chưa mở cửa lại. 'Nhiều chủ hàng chưa mở lại do phải dọn dẹp nhà cửa bị ngập trước đó, chưa có thời gian dọn cửa hàng', chị Tuyết, chủ một cửa hàng, nói. Trong chợ gốm, nhiều cửa hàng quây bạt, chưa mở cửa lại. 'Nhiều chủ hàng chưa mở lại do phải dọn dẹp nhà cửa bị ngập trước đó, chưa có thời gian dọn cửa hàng', chị Tuyết, chủ một cửa hàng, nói. Chị Lan, chủ một cửa hàng trong chợ, cho biết nhà chị không bị thiệt hại nặng nên dọn hàng ra sớm để đón khách. 'Ngày thường ít khách lui tới nhưng đông vào dịp cuối tuần', chị Lan nói. Chị Lan, chủ một cửa hàng trong chợ, cho biết nhà chị không bị thiệt hại nặng nên dọn hàng ra sớm để đón khách. 'Ngày thường ít khách lui tới nhưng đông vào dịp cuối tuần', chị Lan nói. Cửa hàng nặn gốm của chị Lan đã sẵn sàng đón khách hàng đến trải nghiệm. Cửa hàng nặn gốm của chị Lan đã sẵn sàng đón khách hàng đến trải nghiệm. Các gian hàng mở lại với lác đác du khách tới tham quan, mua sắm - trái với khung cảnh tấp nập mỗi dịp lễ, Tết khi mặt hàng gốm sứ được nhiều người tìm mua. Các gian hàng mở lại với lác đác du khách tới tham quan, mua sắm - trái với khung cảnh tấp nập mỗi dịp lễ, Tết khi mặt hàng gốm sứ được nhiều người tìm mua. Bảo tàng gốm Bát Tràng nằm gần ngoài đê, trước khi vào làng gốm, cũng đã mở cửa sẵn sàng đón khách. Bảo tàng được xây dựng từ năm 2018 với kinh phí 150 tỷ đồng, là 'trung tâm tinh hoa làng nghề Việt'. Bảo tàng gốm Bát Tràng nằm gần ngoài đê, trước khi vào làng gốm, cũng đã mở cửa sẵn sàng đón khách. Bảo tàng được xây dựng từ năm 2018 với kinh phí 150 tỷ đồng, là 'trung tâm tinh hoa làng nghề Việt'. Bên trong bảo tàng có thiết kế độc đáo, nhiều tầng với các chuyên đề khác nhau về lịch sử hình thành, phát triển cũng như các loại hình gốm tại Bát Tràng. 'Đến làng gốm để có trải nghiệm thú vị, thay đổi không khí và tìm hiểu về gốm truyền thống', Phạm Hoàng Hiệu, Thanh Xuân, Hà Nội, cho biết khi đến đây sau những ngày phải ở nhà vì mưa lụt. Bên trong bảo tàng có thiết kế độc đáo, nhiều tầng với các chuyên đề khác nhau về lịch sử hình thành, phát triển cũng như các loại hình gốm tại Bát Tràng. 'Đến làng gốm để có trải nghiệm thú vị, thay đổi không khí và tìm hiểu về gốm truyền thống', Phạm Hoàng Hiệu, Thanh Xuân, Hà Nội, cho biết khi đến đây sau những ngày phải ở nhà vì mưa lụt. Đình làng Bát Tràng hơn 300 tuổi không bị ảnh hưởng sau trận lụt. Đình được coi là 'báu vật đi cùng năm tháng' ở làng, hiện lưu giữ hơn 50 đạo sắc phong. Đình Bát Tràng được Bộ Văn hóa Thể thao và Du lịch cấp bằng Di tích văn hóa kiến trúc nghệ thuật năm 2005. Đình làng Bát Tràng hơn 300 tuổi không bị ảnh hưởng sau trận lụt. Đình được coi là 'báu vật đi cùng năm tháng' ở làng, hiện lưu giữ hơn 50 đạo sắc phong. Đình Bát Tràng được Bộ Văn hóa Thể thao và Du lịch cấp bằng Di tích văn hóa kiến trúc nghệ thuật năm 2005. Hoàng Giang",
-  "summary": "LỖI: 'NoneType' object is not iterable",
-  "faithfulness_score": 0.0,
-  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin nào về văn bản gốc, không phản ánh nội dung của văn bản.",
-  "relevance_score": 0.0,
-  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không đề cập đến các sự kiện, tình huống hoặc thông điệp chính.",
-  "coherence_conciseness_score": 0.0,
-  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá về tính mạch lạc và súc tích."
-}</t>
-        </is>
-      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -751,27 +607,8 @@
           <t>Bếp trưởng Christian Le Squer nổi tiếng với 22 năm liên tiếp đạt 3 sao Michelin, hiện đảm nhiệm vai trò bếp trưởng tại La Maison 1888. Nhà hàng là điểm đến ẩm thực Pháp cao cấp, nằm ngay trong khuôn viên resort InterContinental Danang Sun Peninsula Resort. Tháng 7 vừa qua đánh dấu cột mốc quan trọng khi La Maison 1888 gia nhập 'bản đồ' Michelin Guide với ngôi sao đầu tiên. Với sự điều hành của bếp trưởng Christian Le Squer, thực khách sẽ được trải nghiệm ẩm thực Pháp cao cấp giao hòa giữa nghệ thuật và thẩm mỹ cao cấp, mang đậm dấu ấn cá nhân của ông. Ông Seif Hamdy, Tổng giám đốc khu nghỉ dưỡng cho biết sự góp mặt của bếp trưởng Christian tại InterContinental Danang là bước tiến quan trọng. Sự sáng tạo trong ẩm thực cùng khả năng của ông là điều đã được chứng minh bằng 22 năm liên tục được trao tặng ba sao Michelin. Christian Le Squer còn từng đạt danh hiệu 'Bếp trưởng của năm' do Gault &amp; Millau trao tặng năm 2023. 'Christian Le Squer sẽ mang đến làn gió mới cùng tầm nhìn sáng tạo, góp phần nâng tầm trải nghiệm ẩm thực cho thực khách tại La Maison 1888 với phong cách 'haute couture' đặc trưng do chính ông tạo ra', ông Seif Hamdy nói. Sinh ra và lớn lên bên bờ biển Brittany (Pháp), bếp trưởng Christian có nhiều trải nghiệm tuổi thơ gắn liền với ẩm thực. Những ký ức thuở nhỏ gieo cho ông đam mê ẩm thực sâu sắc và dẫn lối ông đến kinh đô ánh sáng và thời trang Paris. Đến năm 34 tuổi, ông được trao sao Michelin đầu tiên tại nhà hàng Café de la Paix. Thành công này đã thôi thúc ông tiếp tục hành trình chinh phục những đỉnh cao ẩm thực kế tiếp. Sau đó, ông gia nhập nhà hàng Pavillon Ledoyen năm 1999, giúp nơi này giành được ba sao Michelin không lâu sau đó. Thành tích này được ông Christian lặp lại tại Le Cinq, nhà hàng Pháp biểu tượng tại khách sạn Four Seasons Hotel George V ở Paris. Bếp trưởng Christian ví von phong cách ẩm thực độc đáo của mình như những tác phẩm thời trang nghệ thuật cao cấp 'haute couture' trên bàn ăn. Ông cho biết mỗi món đều mang dấu ấn riêng biệt, sở hữu hương vị và diện mạo thanh lịch như một bộ trang phục sang trọng hay một chai nước hoa độc bản được giới thiệu tại Tuần lễ Thời trang Paris. Sau nhiều chuyến ghé thăm Việt Nam, đặc biệt là Đà Nẵng, ông hiểu hơn về nhu cầu của thực khách nơi đây. Nhiều người ông gặp cho biết họ tìm kiếm sự kết hợp hài hòa giữa truyền thống và hiện đại trong ẩm thực Pháp. Việc khám phá các hương vị, nguyên liệu, văn hóa ẩm thực đặc sắc của Việt Nam đã trở thành nguồn cảm hứng để ông phác họa nên bức tranh ẩm thực riêng cho La Maison 1888. 'Tôi rất mong chờ được cùng làm việc với đội ngũ tài năng tại La Maison 1888, đặc biệt là Bếp trưởng Florian Stein', Christian nói. Nằm trong một dinh thự theo phong cách Đông Dương thanh lịch do Bill Bensley thiết kế, La Maison 1888 là một trong những điểm đến ẩm thực quốc tế đáng cân nhắc tại Đông Nam Á. Nhà hàng sở hữu hầm rượu vang với bộ sưu tập phong phú cùng tầm nhìn đẹp hướng biển. Nơi đây chinh phục thực khách bằng ẩm thực cao cấp với chất lượng được Michelin công nhận cùng không gian sang trọng đậm chất Pháp. Sắp tới, bếp trưởng Christian hứa hẹn mang đến nhiều bất ngờ thú vị, góp phần nâng tầm trải nghiệm ẩm thực của thực khách tại đây. Á Hiên</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>LỖI: 'NoneType' object is not iterable</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>{
-  "id": 12,
-  "style": "news_brief",
-  "article": "Bếp trưởng Christian Le Squer nổi tiếng với 22 năm liên tiếp đạt 3 sao Michelin, hiện đảm nhiệm vai trò bếp trưởng tại La Maison 1888. Nhà hàng là điểm đến ẩm thực Pháp cao cấp, nằm ngay trong khuôn viên resort InterContinental Danang Sun Peninsula Resort. Tháng 7 vừa qua đánh dấu cột mốc quan trọng khi La Maison 1888 gia nhập 'bản đồ' Michelin Guide với ngôi sao đầu tiên. Với sự điều hành của bếp trưởng Christian Le Squer, thực khách sẽ được trải nghiệm ẩm thực Pháp cao cấp giao hòa giữa nghệ thuật và thẩm mỹ cao cấp, mang đậm dấu ấn cá nhân của ông. Ông Seif Hamdy, Tổng giám đốc khu nghỉ dưỡng cho biết sự góp mặt của bếp trưởng Christian tại InterContinental Danang là bước tiến quan trọng. Sự sáng tạo trong ẩm thực cùng khả năng của ông là điều đã được chứng minh bằng 22 năm liên tục được trao tặng ba sao Michelin. Christian Le Squer còn từng đạt danh hiệu 'Bếp trưởng của năm' do Gault &amp; Millau trao tặng năm 2023. 'Christian Le Squer sẽ mang đến làn gió mới cùng tầm nhìn sáng tạo, góp phần nâng tầm trải nghiệm ẩm thực cho thực khách tại La Maison 1888 với phong cách 'haute couture' đặc trưng do chính ông tạo ra', ông Seif Hamdy nói. Sinh ra và lớn lên bên bờ biển Brittany (Pháp), bếp trưởng Christian có nhiều trải nghiệm tuổi thơ gắn liền với ẩm thực. Những ký ức thuở nhỏ gieo cho ông đam mê ẩm thực sâu sắc và dẫn lối ông đến kinh đô ánh sáng và thời trang Paris. Đến năm 34 tuổi, ông được trao sao Michelin đầu tiên tại nhà hàng Café de la Paix. Thành công này đã thôi thúc ông tiếp tục hành trình chinh phục những đỉnh cao ẩm thực kế tiếp. Sau đó, ông gia nhập nhà hàng Pavillon Ledoyen năm 1999, giúp nơi này giành được ba sao Michelin không lâu sau đó. Thành tích này được ông Christian lặp lại tại Le Cinq, nhà hàng Pháp biểu tượng tại khách sạn Four Seasons Hotel George V ở Paris. Bếp trưởng Christian ví von phong cách ẩm thực độc đáo của mình như những tác phẩm thời trang nghệ thuật cao cấp 'haute couture' trên bàn ăn. Ông cho biết mỗi món đều mang dấu ấn riêng biệt, sở hữu hương vị và diện mạo thanh lịch như một bộ trang phục sang trọng hay một chai nước hoa độc bản được giới thiệu tại Tuần lễ Thời trang Paris. Sau nhiều chuyến ghé thăm Việt Nam, đặc biệt là Đà Nẵng, ông hiểu hơn về nhu cầu của thực khách nơi đây. Nhiều người ông gặp cho biết họ tìm kiếm sự kết hợp hài hòa giữa truyền thống và hiện đại trong ẩm thực Pháp. Việc khám phá các hương vị, nguyên liệu, văn hóa ẩm thực đặc sắc của Việt Nam đã trở thành nguồn cảm hứng để ông phác họa nên bức tranh ẩm thực riêng cho La Maison 1888. 'Tôi rất mong chờ được cùng làm việc với đội ngũ tài năng tại La Maison 1888, đặc biệt là Bếp trưởng Florian Stein', Christian nói. Nằm trong một dinh thự theo phong cách Đông Dương thanh lịch do Bill Bensley thiết kế, La Maison 1888 là một trong những điểm đến ẩm thực quốc tế đáng cân nhắc tại Đông Nam Á. Nhà hàng sở hữu hầm rượu vang với bộ sưu tập phong phú cùng tầm nhìn đẹp hướng biển. Nơi đây chinh phục thực khách bằng ẩm thực cao cấp với chất lượng được Michelin công nhận cùng không gian sang trọng đậm chất Pháp. Sắp tới, bếp trưởng Christian hứa hẹn mang đến nhiều bất ngờ thú vị, góp phần nâng tầm trải nghiệm ẩm thực của thực khách tại đây. Á Hiên",
-  "summary": "LỖI: 'NoneType' object is not iterable",
-  "faithfulness_score": 0.0,
-  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin nào về văn bản gốc, không có nội dung để đánh giá tính trung thực.",
-  "relevance_score": 0.0,
-  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không có nội dung để đánh giá tính bao quát.",
-  "coherence_conciseness_score": 0.0,
-  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá tính mạch lạc và súc tích."
-}</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -779,27 +616,8 @@
           <t>Đại diện Sun World Sầm Sơn cho biết chương trình ưu đãi nhằm tri ân khách hàng đã ủng hộ suốt thời gian công viên nước ra mắt. Từ ngày 3/9, giá 100.000 đồng áp dụng chung cho mọi lứa tuổi. Trước đó, giá gốc 200.000 đồng (khách ngoại tỉnh) và 150.000 đồng (người Thanh Hóa). Riêng bé dưới 1 m được miễn phí vé. Khai trương đúng dịp cao điểm hè 30/6, Sun World Sầm Sơn - công viên nước quy mô nhất miền Bắc cùng tổ hợp trò chơi đạt kỷ lục châu Á - Thái Bình Dương - là 'cú hích' cho du lịch Sầm Sơn năm nay, hút hàng nghìn lượt khách mỗi ngày. Công viên nước thuộc phường Quảng Châu, Quảng Tiến, ngay đại lộ Nam sông Mã - cửa ngõ Sầm Sơn, cách trung tâm TP Thanh Hóa13 km và bãi biển Sầm Sơn 1,5 km. Thiết kế không gian lấy cảm hứng từ truyện dân gian Việt Nam, kết hợp hài hòa kiến trúc truyền thống và hiện đại. Các trò chơi cùng cảnh quan vừa gần gũi, vừa mới mẻ. Công viên nước chia ba phân khu riêng biệt dành cho mọi lứa tuổi: gia đình, trẻ em và khu cảm giác mạnh. Trong đó, trò 'Vịnh sóng thần' có diện tích 6.100 m2, chiều dài bờ biển nhân tạo đến 179 m. Cụ thể, phân khu cảm giác mạnh tập hợp những trò tốc độ, kích thích, góp phần giúp du khách giải tỏa áp lực công việc, cuộc sống. Điển hình là tổ hợp hàm cá mập, với các đường trượt uốn lượn, độ dốc cao chủ đề 'cá mập hung tàn' hay 'cá mập siêu bạo chúa'. Nhằm đáp ứng nhu cầu vui chơi của gia đình lẫn nhóm bạn trẻ, ban tổ chức kiến tạo mê cung quy mô lớn, nhấn vào các đường trượt đan chéo và vực lốc xoáy (tổ hợp ống trượt uốn lượn, xoắn ốc như các xoáy nước dành cho phao đôi đầu tiên tại châu Á - Thái Bình Dương). Du khách có thể khám phá đa dạng đường trượt gồm: 'cá đuối vượt sóng', 'cá trê vượt thác' hay 8 làn trượt thảm bạch tuộc. Chủ dự án cũng bố trí phân khu bến tuổi thơ cho trẻ, với 3 tổ hợp nhỏ mô hình sinh vật dưới nước quen thuộc. Bao quanh khu trò chơi là sông lười, gợi nhớ dòng Đơ tại Sầm Sơn. Tại đây, du khách có thể lênh đênh theo dòng nước, thư giãn và tận hưởng cảm giác sảng khoái như trẻ thơ. Nếu muốn khám phá trọn vẹn công viên nước, du khách nên đến từ 10h hoặc 15h bởi nắng không quá gắt, thích hợp với cả người già lẫn trẻ nhỏ. Vạn Phát</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Sun World Sầm Sơn giảm giá vé 100.000 đồng từ ngày 3/9, miễn phí cho trẻ dưới 1m. Công viên nước quy mô lớn nằm gần trung tâm TP Thanh Hóa, hấp dẫn du khách nhờ nhiều trò chơi kết hợp giữa truyền thống và hiện đại.</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>{
-  "id": 13,
-  "style": "news_brief",
-  "article": "Đại diện Sun World Sầm Sơn cho biết chương trình ưu đãi nhằm tri ân khách hàng đã ủng hộ suốt thời gian công viên nước ra mắt. Từ ngày 3/9, giá 100.000 đồng áp dụng chung cho mọi lứa tuổi. Trước đó, giá gốc 200.000 đồng (khách ngoại tỉnh) và 150.000 đồng (người Thanh Hóa). Riêng bé dưới 1 m được miễn phí vé. Khai trương đúng dịp cao điểm hè 30/6, Sun World Sầm Sơn - công viên nước quy mô nhất miền Bắc cùng tổ hợp trò chơi đạt kỷ lục châu Á - Thái Bình Dương - là 'cú hích' cho du lịch Sầm Sơn năm nay, hút hàng nghìn lượt khách mỗi ngày. Công viên nước thuộc phường Quảng Châu, Quảng Tiến, ngay đại lộ Nam sông Mã - cửa ngõ Sầm Sơn, cách trung tâm TP Thanh Hóa13 km và bãi biển Sầm Sơn 1,5 km. Thiết kế không gian lấy cảm hứng từ truyện dân gian Việt Nam, kết hợp hài hòa kiến trúc truyền thống và hiện đại. Các trò chơi cùng cảnh quan vừa gần gũi, vừa mới mẻ. Công viên nước chia ba phân khu riêng biệt dành cho mọi lứa tuổi: gia đình, trẻ em và khu cảm giác mạnh. Trong đó, trò 'Vịnh sóng thần' có diện tích 6.100 m2, chiều dài bờ biển nhân tạo đến 179 m. Cụ thể, phân khu cảm giác mạnh tập hợp những trò tốc độ, kích thích, góp phần giúp du khách giải tỏa áp lực công việc, cuộc sống. Điển hình là tổ hợp hàm cá mập, với các đường trượt uốn lượn, độ dốc cao chủ đề 'cá mập hung tàn' hay 'cá mập siêu bạo chúa'. Nhằm đáp ứng nhu cầu vui chơi của gia đình lẫn nhóm bạn trẻ, ban tổ chức kiến tạo mê cung quy mô lớn, nhấn vào các đường trượt đan chéo và vực lốc xoáy (tổ hợp ống trượt uốn lượn, xoắn ốc như các xoáy nước dành cho phao đôi đầu tiên tại châu Á - Thái Bình Dương). Du khách có thể khám phá đa dạng đường trượt gồm: 'cá đuối vượt sóng', 'cá trê vượt thác' hay 8 làn trượt thảm bạch tuộc. Chủ dự án cũng bố trí phân khu bến tuổi thơ cho trẻ, với 3 tổ hợp nhỏ mô hình sinh vật dưới nước quen thuộc. Bao quanh khu trò chơi là sông lười, gợi nhớ dòng Đơ tại Sầm Sơn. Tại đây, du khách có thể lênh đênh theo dòng nước, thư giãn và tận hưởng cảm giác sảng khoái như trẻ thơ. Nếu muốn khám phá trọn vẹn công viên nước, du khách nên đến từ 10h hoặc 15h bởi nắng không quá gắt, thích hợp với cả người già lẫn trẻ nhỏ. Vạn Phát",
-  "summary": "Sun World Sầm Sơn giảm giá vé 100.000 đồng từ ngày 3/9, miễn phí cho trẻ dưới 1m. Công viên nước quy mô lớn nằm gần trung tâm TP Thanh Hóa, hấp dẫn du khách nhờ nhiều trò chơi kết hợp giữa truyền thống và hiện đại.",
-  "faithfulness_score": 0.8,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng thiếu sót một số chi tiết quan trọng như thời gian khai trương, các phân khu trong công viên nước và một số trò chơi đặc biệt",
-  "relevance_score": 0.7,
-  "relevance_reason": "Bản tóm tắt chưa bao hàm đủ các ý chính quan trọng như mục đích của chương trình ưu đãi, vị trí và thiết kế của công viên nước",
-  "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt có logic, dễ đọc và súc tích, tuy nhiên có thể cải thiện bằng cách thêm một số chi tiết quan trọng mà không làm cho bản tóm tắt trở nên rườm rà"
-}</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -807,27 +625,8 @@
           <t>Chiều 28/8, khách sạn Grand Mercure Hanoi đón hơn 200 vị khách thuộc đoàn 4.500 du khách từ Ấn Độ sang Việt Nam. Theo ông Remi Faubel, tổng quản lý khách sạn, đây là cơ hội lớn để quảng bá nét đẹp văn hóa, truyền thống tới khách quốc tế. 'Chúng tôi tự tin các yếu tố như lối kiến trúc Đông Dương, hệ thống cửa Bức Bàn, các chi tiết nội thất lấy cảm hứng từ hoa sen, trống đồng, hạt gạo, ruộng bậc thang,... sẽ góp phần để lại ấn tượng tốt đẹp trong lòng du khách', ông Faubel nói. Do nhu cầu của khách, Grand Mercure Hanoi vẫn phục vụ chủ yếu các món Ấn. Bếp trưởng - Nguyễn Minh Nguyện lý giải, du khách Ấn Độ luôn có nhu cầu thưởng thức ẩm thực đất nước họ để có cảm giác gần gũi và thoải mái khi đi du lịch. Đó cũng là cách họ gìn giữ văn hóa và chế độ ăn truyền thống. 'Khi lên kế hoạch, chúng tôi phải trao đổi với phía đại diện đoàn để nắm thông tin về chế độ ăn, suất ăn tôn giáo, yêu cầu đặc biệt, từ đó lựa chọn các loại gia vị đặc trưng của Ấn Độ để các món ăn giữ được hương vị', vị bếp trưởng nói. Tuy nhiên, khách sạn cũng chuẩn bị thêm một số món ăn đặc trưng của Việt Nam như gà, bánh cuốn, xôi, hoa quả nhiệt đới... để giới thiệu đến đoàn khách. Từ ngày 27/8 đến 3/9, Việt Nam đón 4.500 du khách thuộc tập đoàn dược phẩm lớn đến từ Ấn Độ. Dự kiến, họ sẽ chia thành các nhóm nhỏ tới Hà Nội - Ninh Bình - Hạ Long và sử dụng các dịch vụ lưu trú, ăn uống tại các khách sạn 5 sao trên địa bàn thủ đô. Ấn Độ là một trong 10 thị trường khách du lịch quốc tế lớn nhất Việt Nam. Theo số liệu từ Cục Du lịch Quốc gia, trong 6 tháng đầu năm, nước ta đã đón 231.000 lượt khách Ấn Độ, tăng 164% so với cùng kỳ năm 2023. Việt Nam có nhiều thế mạnh để thu hút và phát triển thị trường này. Các đường bay thẳng giữa hai nước được khai thác trong thời gian gần đây khiến thời gian di chuyển rút ngắn chỉ còn khoảng 4 - 5 tiếng. Theo Outlook Traveller, Việt Nam sở hữu những cảnh quan đẹp, nền văn hóa đa dạng và chiều sâu lịch sử. Giá thành dịch vụ cạnh tranh khiến nước ta trở thành điểm đến lý tưởng cho du khách Ấn Độ. Lan Anh</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Hàng nghìn du khách Ấn Độ đến Grand Mercure Hanoi, nơi lối kiến trúc Đông Dương và ẩm thực truyền thống tạo ấn tượng tốt. Việt Nam với cảnh quan đẹp đa dạng văn hóa lịch sử thu hút du khách do giá cả hợp lý.</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>{
-  "id": 14,
-  "style": "news_brief",
-  "article": "Chiều 28/8, khách sạn Grand Mercure Hanoi đón hơn 200 vị khách thuộc đoàn 4.500 du khách từ Ấn Độ sang Việt Nam. Theo ông Remi Faubel, tổng quản lý khách sạn, đây là cơ hội lớn để quảng bá nét đẹp văn hóa, truyền thống tới khách quốc tế. 'Chúng tôi tự tin các yếu tố như lối kiến trúc Đông Dương, hệ thống cửa Bức Bàn, các chi tiết nội thất lấy cảm hứng từ hoa sen, trống đồng, hạt gạo, ruộng bậc thang,... sẽ góp phần để lại ấn tượng tốt đẹp trong lòng du khách', ông Faubel nói. Do nhu cầu của khách, Grand Mercure Hanoi vẫn phục vụ chủ yếu các món Ấn. Bếp trưởng - Nguyễn Minh Nguyện lý giải, du khách Ấn Độ luôn có nhu cầu thưởng thức ẩm thực đất nước họ để có cảm giác gần gũi và thoải mái khi đi du lịch. Đó cũng là cách họ gìn giữ văn hóa và chế độ ăn truyền thống. 'Khi lên kế hoạch, chúng tôi phải trao đổi với phía đại diện đoàn để nắm thông tin về chế độ ăn, suất ăn tôn giáo, yêu cầu đặc biệt, từ đó lựa chọn các loại gia vị đặc trưng của Ấn Độ để các món ăn giữ được hương vị', vị bếp trưởng nói. Tuy nhiên, khách sạn cũng chuẩn bị thêm một số món ăn đặc trưng của Việt Nam như gà, bánh cuốn, xôi, hoa quả nhiệt đới... để giới thiệu đến đoàn khách. Từ ngày 27/8 đến 3/9, Việt Nam đón 4.500 du khách thuộc tập đoàn dược phẩm lớn đến từ Ấn Độ. Dự kiến, họ sẽ chia thành các nhóm nhỏ tới Hà Nội - Ninh Bình - Hạ Long và sử dụng các dịch vụ lưu trú, ăn uống tại các khách sạn 5 sao trên địa bàn thủ đô. Ấn Độ là một trong 10 thị trường khách du lịch quốc tế lớn nhất Việt Nam. Theo số liệu từ Cục Du lịch Quốc gia, trong 6 tháng đầu năm, nước ta đã đón 231.000 lượt khách Ấn Độ, tăng 164% so với cùng kỳ năm 2023. Việt Nam có nhiều thế mạnh để thu hút và phát triển thị trường này. Các đường bay thẳng giữa hai nước được khai thác trong thời gian gần đây khiến thời gian di chuyển rút ngắn chỉ còn khoảng 4 - 5 tiếng. Theo Outlook Traveller, Việt Nam sở hữu những cảnh quan đẹp, nền văn hóa đa dạng và chiều sâu lịch sử. Giá thành dịch vụ cạnh tranh khiến nước ta trở thành điểm đến lý tưởng cho du khách Ấn Độ. Lan Anh",
-  "summary": "Hàng nghìn du khách Ấn Độ đến Grand Mercure Hanoi, nơi lối kiến trúc Đông Dương và ẩm thực truyền thống tạo ấn tượng tốt. Việt Nam với cảnh quan đẹp đa dạng văn hóa lịch sử thu hút du khách do giá cả hợp lý.",
-  "faithfulness_score": 0.8,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng thiếu sót một số chi tiết quan trọng như số lượng du khách và các hoạt động cụ thể tại khách sạn",
-  "relevance_score": 0.7,
-  "relevance_reason": "Bản tóm tắt chưa bao hàm đủ các ý chính quan trọng như nhu cầu ẩm thực của du khách Ấn Độ và việc giới thiệu văn hóa Việt Nam",
-  "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, tuy nhiên có thể rút gọn một số từ ngữ để tăng tính súc tích"
-}</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -835,27 +634,8 @@
           <t>Theo Báo cáo Hạnh phúc Thế giới (World Happiness Report) 2024 của Liên Hợp Quốc công bố hồi tháng 3, Lithuania là quốc gia 'hạnh phúc nhất thế giới dành cho những người dưới 30 tuổi (gen Z)'. Hai nhà sáng tạo nội dung Ammar Kandil và Staffan Taylor đến từ Yes Theory, kênh truyền thông nổi tiếng của Canada, quyết định đến thủ đô Vilnius để tìm hiểu xem liệu báo cáo có nói đúng. Khi hạ cánh xuống Vilnius, Amma và Staffan bắt đầu nói chuyện với người dân địa phương. Hầu hết người trẻ đều đồng ý quốc gia họ đang sống là nơi tốt nhờ 'đồ ăn tuyệt vời, người dân thân thiện, nhiều cơ hội nghề nghiệp và nền kinh tế đang phát triển'. Nhiều người trong số đó cho rằng các khó khăn mà thế hệ trước chịu đựng đã dạy thế hệ trẻ ngày nay cách tận hưởng cuộc sống trong từng khoảnh khắc và 'tìm thấy vẻ đẹp trong những điều giản dị'. Để thu hút nhiều người trẻ đến nói chuyện hơn, Amma và Staffan đã tổ chức một buổi gặp gỡ. Tại sự kiện, những người tham dự lần lượt bày tỏ quan điểm. 'Sau một năm sống tại Mỹ, tôi đánh giá cao cuộc sống ở Lithuania vì tính kết nối với thiên nhiên', một thanh niên chia sẻ. Người này nói thêm du khách có thể dễ dàng tiếp cận một hồ nước hay khu rừng tại Lithuania và chiêm ngưỡng khung cảnh thiên nhiên tuyệt đẹp ở đó. 'Lithuania chưa bao giờ tốt như hiện nay', một phụ nữ trẻ khác thừa nhận. Khi nói về hạnh phúc, một người dân địa phương cho biết dù người trẻ sống ở đất nước này 'khá vui vẻ' nhưng không có nghĩa họ không phải đối mặt với nhiều vấn đề, áp lực cuộc sống. Sau buổi gặp gỡ, Ammar và Staffan dành phần còn lại của chuyến đi để giao lưu với người dân địa phương, ghé thăm các điểm du lịch như nhà tù cũ Lukiškės giờ là địa điểm văn hóa và tượng đài Hill of Crosses. 'Đây là một trong những trải nghiệm du lịch hạnh phúc nhất tôi từng có', Ammar, người từng đi khắp thế giới, chia sẻ với độc giả trên kênh Yes Theory khi đang tham gia một bữa tiệc tối. Steffan đồng tình khi nhận định Lithuania chắc chắn là một trong những quốc gia cởi mở, hào phóng, tử tế nhất mà anh từng đến. Video của hai du khách đến từ Canada đã thu hút gần một triệu lượt xem và bình luận chỉ sau vài ngày đăng tải. Một người từng đến Vilnius học theo diện trao đổi sinh viên chia sẻ thời gian ở Liathuania là quãng thời gian hạnh phúc nhất của mình. 'Cảm ơn Liathuania đã chào đón tôi', người này nói. 'Tình yêu, sự sáng tạo và lòng tốt có thể giúp chúng ta vượt qua quá khứ đen tối, biến tiêu cực thành ánh sáng và giúp đỡ người khác', một người dân địa phương bày tỏ sau khi xem video của Ammar và Steffan. Anh Minh(TheoYes Theory, DM)</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Lithuania được đánh giá cao về sự cởi mở, hào phóng và đồ ăn ngon. Tuy nhiên, cuộc sống vẫn có áp lực từ thế hệ trước đã dạy trẻ tận hưởng từng khoảnh khắc và tìm thấy vẻ đẹp trong giản dị.</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>{
-  "id": 15,
-  "style": "news_brief",
-  "article": "Theo Báo cáo Hạnh phúc Thế giới (World Happiness Report) 2024 của Liên Hợp Quốc công bố hồi tháng 3, Lithuania là quốc gia 'hạnh phúc nhất thế giới dành cho những người dưới 30 tuổi (gen Z)'. Hai nhà sáng tạo nội dung Ammar Kandil và Staffan Taylor đến từ Yes Theory, kênh truyền thông nổi tiếng của Canada, quyết định đến thủ đô Vilnius để tìm hiểu xem liệu báo cáo có nói đúng. Khi hạ cánh xuống Vilnius, Amma và Staffan bắt đầu nói chuyện với người dân địa phương. Hầu hết người trẻ đều đồng ý quốc gia họ đang sống là nơi tốt nhờ 'đồ ăn tuyệt vời, người dân thân thiện, nhiều cơ hội nghề nghiệp và nền kinh tế đang phát triển'. Nhiều người trong số đó cho rằng các khó khăn mà thế hệ trước chịu đựng đã dạy thế hệ trẻ ngày nay cách tận hưởng cuộc sống trong từng khoảnh khắc và 'tìm thấy vẻ đẹp trong những điều giản dị'. Để thu hút nhiều người trẻ đến nói chuyện hơn, Amma và Staffan đã tổ chức một buổi gặp gỡ. Tại sự kiện, những người tham dự lần lượt bày tỏ quan điểm. 'Sau một năm sống tại Mỹ, tôi đánh giá cao cuộc sống ở Lithuania vì tính kết nối với thiên nhiên', một thanh niên chia sẻ. Người này nói thêm du khách có thể dễ dàng tiếp cận một hồ nước hay khu rừng tại Lithuania và chiêm ngưỡng khung cảnh thiên nhiên tuyệt đẹp ở đó. 'Lithuania chưa bao giờ tốt như hiện nay', một phụ nữ trẻ khác thừa nhận. Khi nói về hạnh phúc, một người dân địa phương cho biết dù người trẻ sống ở đất nước này 'khá vui vẻ' nhưng không có nghĩa họ không phải đối mặt với nhiều vấn đề, áp lực cuộc sống. Sau buổi gặp gỡ, Ammar và Staffan dành phần còn lại của chuyến đi để giao lưu với người dân địa phương, ghé thăm các điểm du lịch như nhà tù cũ Lukiškės giờ là địa điểm văn hóa và tượng đài Hill of Crosses. 'Đây là một trong những trải nghiệm du lịch hạnh phúc nhất tôi từng có', Ammar, người từng đi khắp thế giới, chia sẻ với độc giả trên kênh Yes Theory khi đang tham gia một bữa tiệc tối. Steffan đồng tình khi nhận định Lithuania chắc chắn là một trong những quốc gia cởi mở, hào phóng, tử tế nhất mà anh từng đến. Video của hai du khách đến từ Canada đã thu hút gần một triệu lượt xem và bình luận chỉ sau vài ngày đăng tải. Một người từng đến Vilnius học theo diện trao đổi sinh viên chia sẻ thời gian ở Liathuania là quãng thời gian hạnh phúc nhất của mình. 'Cảm ơn Liathuania đã chào đón tôi', người này nói. 'Tình yêu, sự sáng tạo và lòng tốt có thể giúp chúng ta vượt qua quá khứ đen tối, biến tiêu cực thành ánh sáng và giúp đỡ người khác', một người dân địa phương bày tỏ sau khi xem video của Ammar và Steffan. Anh Minh(TheoYes Theory, DM)",
-  "summary": "Lithuania được đánh giá cao về sự cởi mở, hào phóng và đồ ăn ngon. Tuy nhiên, cuộc sống vẫn có áp lực từ thế hệ trước đã dạy trẻ tận hưởng từng khoảnh khắc và tìm thấy vẻ đẹp trong giản dị.",
-  "faithfulness_score": 0.8,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng thiếu sót một số chi tiết quan trọng như việc Lithuania được đánh giá là quốc gia hạnh phúc nhất thế giới dành cho người dưới 30 tuổi và các hoạt động của Ammar và Staffan khi đến Vilnius",
-  "relevance_score": 0.7,
-  "relevance_reason": "Bản tóm tắt không bao hàm đủ các ý chính quan trọng như việc người dân Lithuania đánh giá cao cuộc sống ở đây vì đồ ăn tuyệt vời, người dân thân thiện, nhiều cơ hội nghề nghiệp và nền kinh tế đang phát triển",
-  "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, tuy nhiên có thể rút gọn một số chi tiết để tăng tính súc tích"
-}</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -863,27 +643,8 @@
           <t>Đi dạo trong khuôn viên lâu đài của mình ở Pháp vào một buổi tối mùa hè 2023, Philippa Girling cảm thấy nhẹ nhõm khi nghe thấy tiếng cười của những du khách nữ đang lưu trú tại đây. Tiếng cười là mục tiêu mà CEO Camp Château, nơi tổ chức trại hè dành riêng cho phụ nữ, mong muốn khi mở dịch vụ này. Tuy mới thành lập được hai năm, danh sách khách đăng ký đến nghỉ dưỡng tại lâu đài cổ nằm trên đỉnh đồi ở vùng Quercy, tây nam nước Pháp, năm nay đã kín chỗ. Lượng khách chờ cho mùa hè 2025 đã lên đến 11.000 người. Philippa rất vui khi được mọi người yêu thích dịch vụ cũng nhưng cảm thấy rất tiếc cho những người trong danh sách chờ khi nhiều du khách sẽ phải đợi 20 năm mới đến lượt. Cô đang xem xét để mở rộng trại hè, giúp nhiều du khách nữ có thể sử dụng dịch vụ hơn. Philippa nói mục đích tồn tại của Camp Château rất đơn giản: mang đến cho phụ nữ trải nghiệm vui vẻ. Philippa từng làm 30 năm trong ngành ngân hàng nên thấu hiểu áp lực mà phụ nữ ngày nay phải đối mặt. Do đó, cô cùng các đồng sáng lập tạo ra Camp Château để giúp các khách hàng nữ của mình thư giãn, mang lại cho họ sự chăm sóc sức khỏe tinh thần và thể chất, không gian yên tĩnh và thời gian để hồi phục trước khi quay về cuộc sống thường ngày. Kỳ nghỉ trong trại hè kéo dài sáu ngày năm đêm với nhiều hoạt động để hội viên tham gia như làm nến, nếm thử phô mai, cưỡi ngựa, yoga. Một số phụ nữ hào hứng tham gia mọi hoạt động, số khác thích dành phần lớn thời gian nằm bên hồ bơi. Mỗi đợt đón khách khoảng 50 người. Girling, người lớn lên ở miền nam nước Anh, thường đi nghỉ ở Quercy và hiện sống ở California, Mỹ, nhận thấy 'phụ nữ khi ở bên nhau thật tuyệt vời'. Những người phụ nữ đều rất hòa đồng. Họ nằm giường tầng trong các căn phòng tại lâu đài hoặc trong lều dành cho hai người. Tất cả cùng dùng chung bữa tối tại sảnh lớn và có khung giờ phục vụ đồ uống riêng. Trọng tâm của chương trình trại hè này là trao cho phụ nữ quyền tự quyết, làm mọi thứ họ muốn và chỉ cần đối xử tử tế với nhau. Toàn bộ thiết kế của Camp Château đều hướng tới mục đích giúp mọi người có thể gặp gỡ, trò chuyện nhiều hơn một cách tự nhiên nhất. Điều duy nhất khách cần quyết định tại Camp Château là muốn nghỉ ngơi hay vui chơi. Tất cả phụ nữ đều được chào đón tại trại hè. Từ tháng 7 trở về trước, phần lớn khách đến đây là người Mỹ. Nhưng từ đầu tháng 8, số lượng quốc tịch đa dạng hơn khi có thêm các khách đến từ Andorra, Canada, Ai Cập, Anh và Nigeria. Độ tuổi từ 19 đến ngoài 70 tuổi. Nhiều người đến một mình và không ít người gọi trại hè này là 'môi trường an toàn phục vụ niềm đam mê du lịch' của họ. Ngoài ra, trại hè cũng đón các nhóm khách nhỏ gồm mẹ và con gái. Giá một kỳ nghỉ là 2.178 euro, gồm mọi chi phí ăn ở, vui chơi và không tính đưa đón sân bay, dịch vụ massage. Philippa nói số tiền này không nhỏ nhưng cô và các cộng sự đã phải tính toán để đưa ra mức giá phải chăng nhất có thể. Càng ngày, lượng khách đăng ký càng đông. Nhưng Philippa nói sẽ không tăng giá vì muốn nhiều người có thể tiếp cận trải nghiệm này thay vì hướng tới tệp khách nhà giàu. Anh Minh(TheoEuro News)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Du khách nữ đến Camp Château, lâu đài cổ ở Quercy, Tây Nam Pháp với các hoạt động như làm nến, yoga hoặc thư giãn bên hồ bơi. Mục tiêu trại hè là mang lại trải nghiệm vui vẻ và chăm sóc sức khỏe tinh thần thể chất cho phụ nữ tự quyết định mọi thứ trong sự tôn trọng lẫn nhau. Camp Château đón khách đa dạng từ Mỹ đến Andorra với 11.000 người đăng ký mùa hè năm nay, nhưng nhiều du khách phải đợi hai thập kỷ mới được phục vụ. Philippa Girling tăng giá không vì muốn tiếp cận rộng rãi hơn mà nhằm tập trung vào tệp khách giàu có; tuy nhiên, cô cũng nhận ra rằng cần mở rộng dịch vụ để giúp phụ nữ sử dụng nó dễ dàng hơn. Camp Château tạo điều kiện cho các phụ nữ thư giãn và hồi phục sau khi quay về cuộc sống thường ngày, nhấn mạnh quyền tự quyết định của họ trong sự tôn trọng lẫn nhau.</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>{
-  "id": 16,
-  "style": "news_brief",
-  "article": "Đi dạo trong khuôn viên lâu đài của mình ở Pháp vào một buổi tối mùa hè 2023, Philippa Girling cảm thấy nhẹ nhõm khi nghe thấy tiếng cười của những du khách nữ đang lưu trú tại đây. Tiếng cười là mục tiêu mà CEO Camp Château, nơi tổ chức trại hè dành riêng cho phụ nữ, mong muốn khi mở dịch vụ này. Tuy mới thành lập được hai năm, danh sách khách đăng ký đến nghỉ dưỡng tại lâu đài cổ nằm trên đỉnh đồi ở vùng Quercy, tây nam nước Pháp, năm nay đã kín chỗ. Lượng khách chờ cho mùa hè 2025 đã lên đến 11.000 người. Philippa rất vui khi được mọi người yêu thích dịch vụ cũng nhưng cảm thấy rất tiếc cho những người trong danh sách chờ khi nhiều du khách sẽ phải đợi 20 năm mới đến lượt. Cô đang xem xét để mở rộng trại hè, giúp nhiều du khách nữ có thể sử dụng dịch vụ hơn. Philippa nói mục đích tồn tại của Camp Château rất đơn giản: mang đến cho phụ nữ trải nghiệm vui vẻ. Philippa từng làm 30 năm trong ngành ngân hàng nên thấu hiểu áp lực mà phụ nữ ngày nay phải đối mặt. Do đó, cô cùng các đồng sáng lập tạo ra Camp Château để giúp các khách hàng nữ của mình thư giãn, mang lại cho họ sự chăm sóc sức khỏe tinh thần và thể chất, không gian yên tĩnh và thời gian để hồi phục trước khi quay về cuộc sống thường ngày. Kỳ nghỉ trong trại hè kéo dài sáu ngày năm đêm với nhiều hoạt động để hội viên tham gia như làm nến, nếm thử phô mai, cưỡi ngựa, yoga. Một số phụ nữ hào hứng tham gia mọi hoạt động, số khác thích dành phần lớn thời gian nằm bên hồ bơi. Mỗi đợt đón khách khoảng 50 người. Girling, người lớn lên ở miền nam nước Anh, thường đi nghỉ ở Quercy và hiện sống ở California, Mỹ, nhận thấy 'phụ nữ khi ở bên nhau thật tuyệt vời'. Những người phụ nữ đều rất hòa đồng. Họ nằm giường tầng trong các căn phòng tại lâu đài hoặc trong lều dành cho hai người. Tất cả cùng dùng chung bữa tối tại sảnh lớn và có khung giờ phục vụ đồ uống riêng. Trọng tâm của chương trình trại hè này là trao cho phụ nữ quyền tự quyết, làm mọi thứ họ muốn và chỉ cần đối xử tử tế với nhau. Toàn bộ thiết kế của Camp Château đều hướng tới mục đích giúp mọi người có thể gặp gỡ, trò chuyện nhiều hơn một cách tự nhiên nhất. Điều duy nhất khách cần quyết định tại Camp Château là muốn nghỉ ngơi hay vui chơi. Tất cả phụ nữ đều được chào đón tại trại hè. Từ tháng 7 trở về trước, phần lớn khách đến đây là người Mỹ. Nhưng từ đầu tháng 8, số lượng quốc tịch đa dạng hơn khi có thêm các khách đến từ Andorra, Canada, Ai Cập, Anh và Nigeria. Độ tuổi từ 19 đến ngoài 70 tuổi. Nhiều người đến một mình và không ít người gọi trại hè này là 'môi trường an toàn phục vụ niềm đam mê du lịch' của họ. Ngoài ra, trại hè cũng đón các nhóm khách nhỏ gồm mẹ và con gái. Giá một kỳ nghỉ là 2.178 euro, gồm mọi chi phí ăn ở, vui chơi và không tính đưa đón sân bay, dịch vụ massage. Philippa nói số tiền này không nhỏ nhưng cô và các cộng sự đã phải tính toán để đưa ra mức giá phải chăng nhất có thể. Càng ngày, lượng khách đăng ký càng đông. Nhưng Philippa nói sẽ không tăng giá vì muốn nhiều người có thể tiếp cận trải nghiệm này thay vì hướng tới tệp khách nhà giàu. Anh Minh(TheoEuro News)",
-  "summary": "Du khách nữ đến Camp Château, lâu đài cổ ở Quercy, Tây Nam Pháp với các hoạt động như làm nến, yoga hoặc thư giãn bên hồ bơi. Mục tiêu trại hè là mang lại trải nghiệm vui vẻ và chăm sóc sức khỏe tinh thần thể chất cho phụ nữ tự quyết định mọi thứ trong sự tôn trọng lẫn nhau. Camp Château đón khách đa dạng từ Mỹ đến Andorra với 11.000 người đăng ký mùa hè năm nay, nhưng nhiều du khách phải đợi hai thập kỷ mới được phục vụ. Philippa Girling tăng giá không vì muốn tiếp cận rộng rãi hơn mà nhằm tập trung vào tệp khách giàu có; tuy nhiên, cô cũng nhận ra rằng cần mở rộng dịch vụ để giúp phụ nữ sử dụng nó dễ dàng hơn. Camp Château tạo điều kiện cho các phụ nữ thư giãn và hồi phục sau khi quay về cuộc sống thường ngày, nhấn mạnh quyền tự quyết định của họ trong sự tôn trọng lẫn nhau.",
-  "faithfulness_score": 0.8,
-  "faithfulness_reason": "Bản tóm tắt có một số điểm không chính xác như việc Philippa Girling tăng giá không phải để tập trung vào tệp khách giàu có mà là không tăng giá để giúp nhiều người có thể tiếp cận trải nghiệm này",
-  "relevance_score": 0.9,
-  "relevance_reason": "Bản tóm tắt bao gồm hầu hết các ý chính quan trọng như mục tiêu của Camp Château, các hoạt động và đối tượng khách hàng, tuy nhiên có thể thêm một số chi tiết về lý do thành lập và không gian của lâu đài",
-  "coherence_conciseness_score": 0.8,
-  "coherence_conciseness_reason": "Bản tóm tắt có logic và dễ đọc, tuy nhiên có một số câu dài và phức tạp, cần được tinh gọn hơn để tăng tính súc tích"
-}</t>
-        </is>
-      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -891,27 +652,8 @@
           <t>Thời gian này tại Malaysia cũng có nhiều sự kiện để du khách trải nghiệm như: lễ hội trò chơi dân gian tại Kuala Lumpur (13-16/9), lễ hội văn hóa Putrajaya (27-29/9), lễ hội bãi biển Tanjung Aru 2024 tại Kota Kinabalu (1 và 22/9)... Điểm đến phổ biến nhất tại Malaysia là thủ đô Kuala Lumpur - đô thị sầm uất với những di sản kiến trúc cùng các cao ốc hiện đại. Công trình nổi tiếng nhất là tháp đôi Petronas cao 88 tầng. Tại đây có đài quan sát toàn cảnh thành phố, cầu treo trên không, trung tâm khám phá khoa học Petrosains, thủy cung Aquaria KLCC và trung tâm mua sắm Suria KLCC. Quận trung tâm thành phố Kuala Lumpur là Bukit Bintang, khu vực nhộn nhịp bậc nhất với các khu mua sắm, khách sạn và nhà hàng cao cấp cùng nhiều tụ điểm vui chơi, giải trí. Đảo Penang lại mang đến không khí bình yên, nhẹ nhàng. Đặc biệt, George Town - thủ phủ của bang Penang là di sản thế giới, phản ánh rõ nét dấu vết lịch sử qua từng công trình kiến trúc lẫn đời sống văn hóa của cư dân, từ những ngõ nhỏ với căn nhà hai tầng của người Hoa đến tòa hội đồng thành phố, tháp đồng hồ từ thời thuộc địa Anh. Du khách đừng quên ghé đồi Penang Hill hay đền Kek Lok Si. Langkawi là quần đảo với 99 đảo nhỏ ngoài khơi biển Andaman. Vùng đất này có nhiều bãi biển hoang sơ với khu nghỉ dưỡng cao cấp, phù hợp cho kỳ nghỉ thư giãn sau những ngày bận rộn. Ngoài ra, hòn đảo này còn là điểm đến lý tưởng cho các môn thể thao dưới nước như lặn biển, dù kéo, mô tô nước hoặc khám phá công viên địa chất hàng triệu năm tuổi. Cao nguyên Cameron là địa danh nằm ở bang Pahang, được bao phủ một màu xanh dài bất tận bởi những đồi chè và loại cây ôn đới. Khí hậu của cao nguyên này mang đến cho du khách sự mát mẻ, dễ chịu như đang ở châu Âu. Khi đến đây, du khách đừng quên ghé thăm nông trại chế biến trà, vườn hoa oải hương, thung lũng hoa hồng hay thử trekking leo núi Batu Brinchang. Malaysia có nhiều món ăn hấp dẫn du khách, nổi bật là món cơm 'quốc dân' Nasi Lemak. Món cơm này gồm cơm, nấu từ gạo với nước cốt dừa, trứng luộc, gà chiên, lạc, dưa chuột thái lát, cá khô... ăn kèm xốt sambal. Món ăn tuy đơn giản song đủ dinh dưỡng và được nhiều người ưa thích. Char Kway Teow, món hủ tiếu xào nổi tiếng của cộng đồng người Hoa tại Malaysia được chế biến từ hủ tiếu bản to xào cùng tôm, chả cá, lạp xưởng, trứng, giá đỗ và hẹ. Ngoài ra, Roti Canai là món ăn của cộng đồng người Ấn. Đây là loại bánh dẹt, thơm, giòn và xốp, thường dùng kèm các loại cà ri. Thanh Thư</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>LỖI: 'NoneType' object is not iterable</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>{
-  "id": 17,
-  "style": "news_brief",
-  "article": "Thời gian này tại Malaysia cũng có nhiều sự kiện để du khách trải nghiệm như: lễ hội trò chơi dân gian tại Kuala Lumpur (13-16/9), lễ hội văn hóa Putrajaya (27-29/9), lễ hội bãi biển Tanjung Aru 2024 tại Kota Kinabalu (1 và 22/9)... Điểm đến phổ biến nhất tại Malaysia là thủ đô Kuala Lumpur - đô thị sầm uất với những di sản kiến trúc cùng các cao ốc hiện đại. Công trình nổi tiếng nhất là tháp đôi Petronas cao 88 tầng. Tại đây có đài quan sát toàn cảnh thành phố, cầu treo trên không, trung tâm khám phá khoa học Petrosains, thủy cung Aquaria KLCC và trung tâm mua sắm Suria KLCC. Quận trung tâm thành phố Kuala Lumpur là Bukit Bintang, khu vực nhộn nhịp bậc nhất với các khu mua sắm, khách sạn và nhà hàng cao cấp cùng nhiều tụ điểm vui chơi, giải trí. Đảo Penang lại mang đến không khí bình yên, nhẹ nhàng. Đặc biệt, George Town - thủ phủ của bang Penang là di sản thế giới, phản ánh rõ nét dấu vết lịch sử qua từng công trình kiến trúc lẫn đời sống văn hóa của cư dân, từ những ngõ nhỏ với căn nhà hai tầng của người Hoa đến tòa hội đồng thành phố, tháp đồng hồ từ thời thuộc địa Anh. Du khách đừng quên ghé đồi Penang Hill hay đền Kek Lok Si. Langkawi là quần đảo với 99 đảo nhỏ ngoài khơi biển Andaman. Vùng đất này có nhiều bãi biển hoang sơ với khu nghỉ dưỡng cao cấp, phù hợp cho kỳ nghỉ thư giãn sau những ngày bận rộn. Ngoài ra, hòn đảo này còn là điểm đến lý tưởng cho các môn thể thao dưới nước như lặn biển, dù kéo, mô tô nước hoặc khám phá công viên địa chất hàng triệu năm tuổi. Cao nguyên Cameron là địa danh nằm ở bang Pahang, được bao phủ một màu xanh dài bất tận bởi những đồi chè và loại cây ôn đới. Khí hậu của cao nguyên này mang đến cho du khách sự mát mẻ, dễ chịu như đang ở châu Âu. Khi đến đây, du khách đừng quên ghé thăm nông trại chế biến trà, vườn hoa oải hương, thung lũng hoa hồng hay thử trekking leo núi Batu Brinchang. Malaysia có nhiều món ăn hấp dẫn du khách, nổi bật là món cơm 'quốc dân' Nasi Lemak. Món cơm này gồm cơm, nấu từ gạo với nước cốt dừa, trứng luộc, gà chiên, lạc, dưa chuột thái lát, cá khô... ăn kèm xốt sambal. Món ăn tuy đơn giản song đủ dinh dưỡng và được nhiều người ưa thích. Char Kway Teow, món hủ tiếu xào nổi tiếng của cộng đồng người Hoa tại Malaysia được chế biến từ hủ tiếu bản to xào cùng tôm, chả cá, lạp xưởng, trứng, giá đỗ và hẹ. Ngoài ra, Roti Canai là món ăn của cộng đồng người Ấn. Đây là loại bánh dẹt, thơm, giòn và xốp, thường dùng kèm các loại cà ri. Thanh Thư",
-  "summary": "LỖI: 'NoneType' object is not iterable",
-  "faithfulness_score": 0.0,
-  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin gì về văn bản gốc, không có nội dung để đánh giá tính trung thực.",
-  "relevance_score": 0.0,
-  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không phản ánh được nội dung chính.",
-  "coherence_conciseness_score": 0.0,
-  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá tính mạch lạc và súc tích."
-}</t>
-        </is>
-      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -919,27 +661,8 @@
           <t>Lodo, 62 tuổi, hôm 6/8 đã có buổi sáng trải nghiệm đan võng cùng với nghệ nhân ở Cù Lao Chàm. Ông bất ngờ về độ bền chắc và sự khéo léo, kỳ công của nghệ nhân làm ra nó. Lodo đã mua một chiếc võng về làm kỷ niệm trong chuyến du lịch Việt Nam lần này. 'Tôi nghĩ đây là một vật liệu xanh giúp bảo vệ môi trường', du khách đến từ Pháp nói. Theo ông Lê Vĩnh Thuận, Phó giám đốc Ban quản lý khu bảo tồn biển Cù Lao Chàm, trong dịp Festival 'Cù Lao Chàm - mùa ngô đồng đỏ' năm 2024 diễn ra từ ngày 5 đến 11/8, lượng du khách đổ về Cù Lao Chàm tham gia lễ hội 'rất đông'. Đến đây, du khách được tìm hiểu về nguồn gốc và tham gia cùng với nghệ nhân đan loại võng truyền thống của đảo. Theo giới thiệu của Trung tâm Quản lý bảo tồn di sản Hội An, sợi võng được làm từ các mảng vỏ cây ngô đồng. Sau khi được tách ra từ thân cây, vỏ sẽ được gom lại thành từng bó rồi ngâm nước ở các khe, suối trên đảo như khe Ruộng Chùa, khe Ông Thơ, khe Xóm Mới. Sau một tháng, người thợ đem vỏ về tách chọn lớp bên trong có màu trắng đục, tước từng sợi nhỏ, phơi khô cho đến khi có màu trắng tinh mới có thể bắt tay vào đan võng. Công đoạn tước đòi hỏi sự tập trung cao của người thợ vì 'sợi càng mỏng đan võng càng chặt', nghệ nhân đan võng Ngô Thị Lê, 70 tuổi, cho biết. Vào khoảng tháng 7, người dân trên đảo đi chọn vỏ những cây ngô đồng làm nguyên liệu đan võng, khi cây ra hoa, rụng hết lá, vỏ đủ khô để thu hoạch. Cây ngô đồng dùng làm võng phải có dáng thẳng mới cho ra sợi suôn, mềm, dai và chịu lực tốt. Bà Lê cho biết khi đã chọn được cây, người dân khai thác bằng cách chỉ chặt ngang thân để cây còn nảy chồi, phát triển sinh sống trở lại. Bà Huỳnh Thị Út, 56 tuổi, cùng với bà Lê là hai trong số ít nghệ nhân ở Cù Lao Chàm duy trì nghề đan võng ngô đồng cho biết loại võng này được người xã đảo sáng tạo ra trong quá trình lao động sản xuất. 'Để làm ra chiếc võng đẹp, ngoài tước sợi mỏng còn yêu cầu thắt nút các mối mắt võng đều', bà Út nói. Lodo nói những nghệ nhân đan võng đã giúp ông phân biệt võng tư có bốn dây đan nối nhau và võng sáu có sáu dây dày hơn đan thành hình tứ giác. Võng ngô đồng dài 2,6 m, đan thủ công hơn một tháng, độ bền của võng có thể kéo dài từ 5 đến 10 năm, có giá từ 5 đến 10 triệu đồng. 'Mức giá này xứng đáng với công sức những người thợ bỏ ra', Lodo cho hay. Chị Hà Nhi, 45 tuổi, sống tại Hà Nội, cũng ấn tượng với loại võng không làm từ sợi công nghiệp mà hoàn toàn từ vỏ cây. 'Những sản phẩm thủ công truyền thống thẩm mỹ cao như thế này là điểm nhấn cho du khách khi du lịch trên đảo', chị Nhi nói. Ngô đồng gắn liền với đời sống hàng ngày của người dân Cù Lao Chàm từ hơn 300 năm trước, theo Ban quản lý khu bảo tồn biển Cù Lao Chàm. Trải qua nhiều đời gìn giữ và nỗ lực bảo tồn, phát huy giá trị văn hóa, nghề đan võng ngô đồng ở địa phương được Bộ Văn hóa Thể thao và Du lịch công nhận là Di sản văn hóa phi vật thể quốc gia hôm 6/8. Tuấn Anh</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>LỖI: 'NoneType' object is not iterable</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>{
-  "id": 18,
-  "style": "news_brief",
-  "article": "Lodo, 62 tuổi, hôm 6/8 đã có buổi sáng trải nghiệm đan võng cùng với nghệ nhân ở Cù Lao Chàm. Ông bất ngờ về độ bền chắc và sự khéo léo, kỳ công của nghệ nhân làm ra nó. Lodo đã mua một chiếc võng về làm kỷ niệm trong chuyến du lịch Việt Nam lần này. 'Tôi nghĩ đây là một vật liệu xanh giúp bảo vệ môi trường', du khách đến từ Pháp nói. Theo ông Lê Vĩnh Thuận, Phó giám đốc Ban quản lý khu bảo tồn biển Cù Lao Chàm, trong dịp Festival 'Cù Lao Chàm - mùa ngô đồng đỏ' năm 2024 diễn ra từ ngày 5 đến 11/8, lượng du khách đổ về Cù Lao Chàm tham gia lễ hội 'rất đông'. Đến đây, du khách được tìm hiểu về nguồn gốc và tham gia cùng với nghệ nhân đan loại võng truyền thống của đảo. Theo giới thiệu của Trung tâm Quản lý bảo tồn di sản Hội An, sợi võng được làm từ các mảng vỏ cây ngô đồng. Sau khi được tách ra từ thân cây, vỏ sẽ được gom lại thành từng bó rồi ngâm nước ở các khe, suối trên đảo như khe Ruộng Chùa, khe Ông Thơ, khe Xóm Mới. Sau một tháng, người thợ đem vỏ về tách chọn lớp bên trong có màu trắng đục, tước từng sợi nhỏ, phơi khô cho đến khi có màu trắng tinh mới có thể bắt tay vào đan võng. Công đoạn tước đòi hỏi sự tập trung cao của người thợ vì 'sợi càng mỏng đan võng càng chặt', nghệ nhân đan võng Ngô Thị Lê, 70 tuổi, cho biết. Vào khoảng tháng 7, người dân trên đảo đi chọn vỏ những cây ngô đồng làm nguyên liệu đan võng, khi cây ra hoa, rụng hết lá, vỏ đủ khô để thu hoạch. Cây ngô đồng dùng làm võng phải có dáng thẳng mới cho ra sợi suôn, mềm, dai và chịu lực tốt. Bà Lê cho biết khi đã chọn được cây, người dân khai thác bằng cách chỉ chặt ngang thân để cây còn nảy chồi, phát triển sinh sống trở lại. Bà Huỳnh Thị Út, 56 tuổi, cùng với bà Lê là hai trong số ít nghệ nhân ở Cù Lao Chàm duy trì nghề đan võng ngô đồng cho biết loại võng này được người xã đảo sáng tạo ra trong quá trình lao động sản xuất. 'Để làm ra chiếc võng đẹp, ngoài tước sợi mỏng còn yêu cầu thắt nút các mối mắt võng đều', bà Út nói. Lodo nói những nghệ nhân đan võng đã giúp ông phân biệt võng tư có bốn dây đan nối nhau và võng sáu có sáu dây dày hơn đan thành hình tứ giác. Võng ngô đồng dài 2,6 m, đan thủ công hơn một tháng, độ bền của võng có thể kéo dài từ 5 đến 10 năm, có giá từ 5 đến 10 triệu đồng. 'Mức giá này xứng đáng với công sức những người thợ bỏ ra', Lodo cho hay. Chị Hà Nhi, 45 tuổi, sống tại Hà Nội, cũng ấn tượng với loại võng không làm từ sợi công nghiệp mà hoàn toàn từ vỏ cây. 'Những sản phẩm thủ công truyền thống thẩm mỹ cao như thế này là điểm nhấn cho du khách khi du lịch trên đảo', chị Nhi nói. Ngô đồng gắn liền với đời sống hàng ngày của người dân Cù Lao Chàm từ hơn 300 năm trước, theo Ban quản lý khu bảo tồn biển Cù Lao Chàm. Trải qua nhiều đời gìn giữ và nỗ lực bảo tồn, phát huy giá trị văn hóa, nghề đan võng ngô đồng ở địa phương được Bộ Văn hóa Thể thao và Du lịch công nhận là Di sản văn hóa phi vật thể quốc gia hôm 6/8. Tuấn Anh",
-  "summary": "LỖI: 'NoneType' object is not iterable",
-  "faithfulness_score": 0.0,
-  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin nào về văn bản gốc, không phản ánh nội dung của bài viết.",
-  "relevance_score": 0.0,
-  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ ý chính quan trọng nào từ văn bản gốc, không đề cập đến chủ đề về nghề đan võng ngô đồng tại Cù Lao Chàm.",
-  "coherence_conciseness_score": 0.0,
-  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá về tính mạch lạc và súc tích."
-}</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -947,27 +670,8 @@
           <t>Với mục tiêu quảng bá du lịch mua sắm tại Singapore, Vietrantour cùng Tổng Cục du lịch Singapore giới thiệu những điểm đến mua sắm và check in hấp dẫn. Nếu du khách đang tìm kiếm những món đồ phiên bản giới hạn của các hãng thời trang cao cấp như Prada, Louis Vuitton, Hermes, ION Orchard và Scotts Square, nên tới trục đường Orchard Road. Đặc biệt, một số thời điểm, các cửa hàng thời trang tại khu vực này khuyến mại tới 70%. Ngoài ra, một số địa điểm mua sắm người dân địa phương hay tới là Tampines 1, Jem và Westgate với nhiều cửa hàng bán lẻ, thời trang phục vụ nhu cầu đời sống. Nếu đang trong chuyến đi cùng gia đình, du khách hãy ghé qua trung tâm thương mại Tanglin Mall hoặc House of Anli với hàng nghìn mặt hàng gia dụng, sản phẩm dành cho mẹ và bé. Trong khi đó, trung tâm mua sắm Mustafa - tụ điểm mua sắm đêm khuya quen thuộc của người dân địa phương cũng là nơi nổi tiếng với những món đồ công nghệ hàng đầu, đến các sản phẩm tiêu dùng với giá cả phải chăng. Khi mua sắm tại Singapore, khách hàng còn được hoàn thuế tới 7%. Là quốc gia phát triển mạnh về dịch vụ du lịch, Singapore chú trọng nhiều đến trải nghiệm khách hàng. Đất nước này cũng được đánh giá là trạm trung gian lý tưởng để bảo hành các sản phẩm đồ hiệu, 'thiên đường' mua hàng miễn thuế với nhiều thương hiệu quốc tế và các nhãn hàng địa phương như mỹ phẩm, nước hoa, bia rượu, đồng hồ, thực phẩm... Tại Singapore, một trong những trải nghiệm thú vị là du khách có thể tự tay hoàn thiện các sản phẩm thủ công truyền thống. Các cửa hàng sẽ có thợ thủ công lành nghề hướng dẫn du khách chưng cất rượu gin tại Brass Lion Distillery, làm đồ da tại Atelier Lodge hoặc học kỹ thuật thêu tranh hạt cườm truyền thống tại Rumah Bebe. Bạn cũng có thể dạo qua khu phố di sản Kampong Gelam, nơi sở hữu những cửa hàng bày bán đồ truyền thống như đồ gốm, đồ da thủ công,.. Trải nghiệm này sẽ giúp du khách hiểu rõ hơn về nét đẹp văn hóa Singapore, đồng thời thể hiện phong cách cá nhân trong từng sản phẩm. Du khách nêndạo các nhà sách như Books Actually và Huggs-Epigram Coffee Bookshop để khám phá văn học kinh điển từ một số nhà thơ, tiểu thuyết gia của Singapore. Thanh Thư</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>LỖI: 'NoneType' object is not iterable</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>{
-  "id": 19,
-  "style": "news_brief",
-  "article": "Với mục tiêu quảng bá du lịch mua sắm tại Singapore, Vietrantour cùng Tổng Cục du lịch Singapore giới thiệu những điểm đến mua sắm và check in hấp dẫn. Nếu du khách đang tìm kiếm những món đồ phiên bản giới hạn của các hãng thời trang cao cấp như Prada, Louis Vuitton, Hermes, ION Orchard và Scotts Square, nên tới trục đường Orchard Road. Đặc biệt, một số thời điểm, các cửa hàng thời trang tại khu vực này khuyến mại tới 70%. Ngoài ra, một số địa điểm mua sắm người dân địa phương hay tới là Tampines 1, Jem và Westgate với nhiều cửa hàng bán lẻ, thời trang phục vụ nhu cầu đời sống. Nếu đang trong chuyến đi cùng gia đình, du khách hãy ghé qua trung tâm thương mại Tanglin Mall hoặc House of Anli với hàng nghìn mặt hàng gia dụng, sản phẩm dành cho mẹ và bé. Trong khi đó, trung tâm mua sắm Mustafa - tụ điểm mua sắm đêm khuya quen thuộc của người dân địa phương cũng là nơi nổi tiếng với những món đồ công nghệ hàng đầu, đến các sản phẩm tiêu dùng với giá cả phải chăng. Khi mua sắm tại Singapore, khách hàng còn được hoàn thuế tới 7%. Là quốc gia phát triển mạnh về dịch vụ du lịch, Singapore chú trọng nhiều đến trải nghiệm khách hàng. Đất nước này cũng được đánh giá là trạm trung gian lý tưởng để bảo hành các sản phẩm đồ hiệu, 'thiên đường' mua hàng miễn thuế với nhiều thương hiệu quốc tế và các nhãn hàng địa phương như mỹ phẩm, nước hoa, bia rượu, đồng hồ, thực phẩm... Tại Singapore, một trong những trải nghiệm thú vị là du khách có thể tự tay hoàn thiện các sản phẩm thủ công truyền thống. Các cửa hàng sẽ có thợ thủ công lành nghề hướng dẫn du khách chưng cất rượu gin tại Brass Lion Distillery, làm đồ da tại Atelier Lodge hoặc học kỹ thuật thêu tranh hạt cườm truyền thống tại Rumah Bebe. Bạn cũng có thể dạo qua khu phố di sản Kampong Gelam, nơi sở hữu những cửa hàng bày bán đồ truyền thống như đồ gốm, đồ da thủ công,.. Trải nghiệm này sẽ giúp du khách hiểu rõ hơn về nét đẹp văn hóa Singapore, đồng thời thể hiện phong cách cá nhân trong từng sản phẩm. Du khách nêndạo các nhà sách như Books Actually và Huggs-Epigram Coffee Bookshop để khám phá văn học kinh điển từ một số nhà thơ, tiểu thuyết gia của Singapore. Thanh Thư",
-  "summary": "LỖI: 'NoneType' object is not iterable",
-  "faithfulness_score": 0.0,
-  "faithfulness_reason": "Bản tóm tắt không cung cấp thông tin nào về văn bản gốc, không có nội dung để đánh giá tính trung thực.",
-  "relevance_score": 0.0,
-  "relevance_reason": "Bản tóm tắt không bao gồm bất kỳ thông tin quan trọng nào từ văn bản gốc, không thể đánh giá tính bao quát.",
-  "coherence_conciseness_score": 0.0,
-  "coherence_conciseness_reason": "Bản tóm tắt không có nội dung, không thể đánh giá tính mạch lạc và súc tích."
-}</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -975,27 +679,8 @@
           <t>Chương trình lần này có sự đồng hành của diễn viên Ninh Dương Lan Ngọc. Thông qua Epic Sale, diễn viên mong muốn lan tỏa tinh thần du lịch thông minh, tiện lợi và tối ưu chi phí. Ông Iko Putera, Giám đốc Vận chuyển Traveloka, cho biết việc hợp tác cùng Lan Ngọc đánh dấu cột mốc quan trọng trên hành trình mang đến trải nghiệm du lịch tiện nghi tối ưu cho khách hàng. Tầm ảnh hưởng và đam mê du lịch của cô phù hợp với sứ mệnh nền tảng theo đuổi. Đôi bên đều muốn truyền cảm hứng khám phá thế giới qua những chuyến đi. Với Epic Sale lần này, Traveloka áp dụng ưu đãi đến 50% cho các sản phẩm du lịch, dịch vụ trên toàn thế giới. 'Đây là lời tri ân chúng tôi muốn gửi đến khách hàng đã luôn ủng hộ, gắn bó trên hành trình kiến tạo những chuyến đi đáng nhớ cùng Traveloka', ông Iko Putera cho biết. Từ khi trở thành đại sứ thương hiệu tại Việt Nam, diễn viên Ninh Dương Lan Ngọc đã có nhiều trải nghiệm du lịch chất lượng với nền tảng. Với loạt khuyến mại, ưu đãi, quà tặng trong Epic Sale 2024, cô nói sẽ tranh thủ săn vé, đặt phòng, chuẩn bị cho những chuyến đi sắp tới. Theo Lan Ngọc, chương trình mang lại cho du khách cơ hội du lịch tiện nghi với chi phí tiết kiệm, giúp khơi dậy mong muốn đi đây đi đó, khám phá thế giới. Cô đánh giá cao sự tiện lợi và các dịch vụ toàn diện của nền tảng, giúp việc lên kế hoạch cho các chuyến đi thêm dễ dàng, thú vị. Traveloka đã hợp tác cùng hàng nghìn đối tác để mang đến những deal giá ưu đãi sâu. Người dùng có thể truy cập nền tảng, theo dõi các ưu đãi hàng ngày trong các mục Vé máy bay, Khách sạn, Xperience và nhiều sản phẩm du lịch khác. 'Siêu ưu đãi Epic' (Super Epic Deal) sẽ được áp dụng cho các sản phẩm nhất định trong khung giờ giới hạn. Cụ thể, giờ vàng Epic Hour Deal ưu đãi vé máy bay mỗi thứ Bảy từ 14h-17h; đặt khách sạn giờ vàng EPIC Hotel Hour Deal diễn ra hàng ngày từ 18h-19h. Du khách có thể săn vé máy bay quốc nội và quốc tế với giá ưu đãi. Trong đó, vé nội địa Vietravel giá chỉ từ 781.925 đồng; vé China Southern Airlines đi Thâm Quyến từ 2,819 đồng; vé T'way Air đến Hàn Quốc và Nhật Bản lần lượt chỉ từ 2,667 triệu đồng và 2,682 triệu đồng. Khách hàng còn có cơ hội nghỉ dưỡng tại khách sạn 5 sao trong nước với giá từ 794.000 đồng. Hàng loạt khách sạn Hàn Quốc giá từ 1,858 triệu đồng, Nhật Bản từ 1,146 triệu đồng. Với dịch vụ giải trí, nền tảng áp dụng ưu đãi 'mua 1 tặng 1' vé tham quan Sun World, công viên nước The Amazing Bay, thủy cung Sea Life Bangkok Ocean World (Thái Lan). Để du khách có trải nghiệm du lịch trọn vẹn, Traveloka giới thiệu thêm nhiều tính năng khác như: hoàn tiền 100%, thay đổi lịch trình, thanh toán linh hoạt... Xem thêm thông tin chi tiết về chương trình Epic Sale trên ứng dụng, website và các tài khoản mạng xã hội của Traveloka. Á Hiên</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>781.925 đồng vé Vietravel, 2.819 triệu Thâm Quyến; 2.667 và 2.682 triệu Hàn Quốc-Nhật Bản. Khách sạn từ 794.000-1.858 triệu. Áp dụng 'mua 1 tặng 1' Sun World, The Amazing Bay, Sea Life Bangkok Ocean World. Hoàn tiền 100%, thay đổi lịch trình, thanh toán linh hoạt trên Traveloka. Epic Sale của Ninh Dương Lan Ngọc mong muốn lan tỏa tinh thần du lịch thông minh và áp dụng ưu đãi đến 50% cho các sản phẩm toàn thế giới nhằm tri ân khách hàng và khích lệ khám phá thế giới qua những chuyến đi tiện nghi với chi phí tiết kiệm.</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>{
-  "id": 20,
-  "style": "news_brief",
-  "article": "Chương trình lần này có sự đồng hành của diễn viên Ninh Dương Lan Ngọc. Thông qua Epic Sale, diễn viên mong muốn lan tỏa tinh thần du lịch thông minh, tiện lợi và tối ưu chi phí. Ông Iko Putera, Giám đốc Vận chuyển Traveloka, cho biết việc hợp tác cùng Lan Ngọc đánh dấu cột mốc quan trọng trên hành trình mang đến trải nghiệm du lịch tiện nghi tối ưu cho khách hàng. Tầm ảnh hưởng và đam mê du lịch của cô phù hợp với sứ mệnh nền tảng theo đuổi. Đôi bên đều muốn truyền cảm hứng khám phá thế giới qua những chuyến đi. Với Epic Sale lần này, Traveloka áp dụng ưu đãi đến 50% cho các sản phẩm du lịch, dịch vụ trên toàn thế giới. 'Đây là lời tri ân chúng tôi muốn gửi đến khách hàng đã luôn ủng hộ, gắn bó trên hành trình kiến tạo những chuyến đi đáng nhớ cùng Traveloka', ông Iko Putera cho biết. Từ khi trở thành đại sứ thương hiệu tại Việt Nam, diễn viên Ninh Dương Lan Ngọc đã có nhiều trải nghiệm du lịch chất lượng với nền tảng. Với loạt khuyến mại, ưu đãi, quà tặng trong Epic Sale 2024, cô nói sẽ tranh thủ săn vé, đặt phòng, chuẩn bị cho những chuyến đi sắp tới. Theo Lan Ngọc, chương trình mang lại cho du khách cơ hội du lịch tiện nghi với chi phí tiết kiệm, giúp khơi dậy mong muốn đi đây đi đó, khám phá thế giới. Cô đánh giá cao sự tiện lợi và các dịch vụ toàn diện của nền tảng, giúp việc lên kế hoạch cho các chuyến đi thêm dễ dàng, thú vị. Traveloka đã hợp tác cùng hàng nghìn đối tác để mang đến những deal giá ưu đãi sâu. Người dùng có thể truy cập nền tảng, theo dõi các ưu đãi hàng ngày trong các mục Vé máy bay, Khách sạn, Xperience và nhiều sản phẩm du lịch khác. 'Siêu ưu đãi Epic' (Super Epic Deal) sẽ được áp dụng cho các sản phẩm nhất định trong khung giờ giới hạn. Cụ thể, giờ vàng Epic Hour Deal ưu đãi vé máy bay mỗi thứ Bảy từ 14h-17h; đặt khách sạn giờ vàng EPIC Hotel Hour Deal diễn ra hàng ngày từ 18h-19h. Du khách có thể săn vé máy bay quốc nội và quốc tế với giá ưu đãi. Trong đó, vé nội địa Vietravel giá chỉ từ 781.925 đồng; vé China Southern Airlines đi Thâm Quyến từ 2,819 đồng; vé T'way Air đến Hàn Quốc và Nhật Bản lần lượt chỉ từ 2,667 triệu đồng và 2,682 triệu đồng. Khách hàng còn có cơ hội nghỉ dưỡng tại khách sạn 5 sao trong nước với giá từ 794.000 đồng. Hàng loạt khách sạn Hàn Quốc giá từ 1,858 triệu đồng, Nhật Bản từ 1,146 triệu đồng. Với dịch vụ giải trí, nền tảng áp dụng ưu đãi 'mua 1 tặng 1' vé tham quan Sun World, công viên nước The Amazing Bay, thủy cung Sea Life Bangkok Ocean World (Thái Lan). Để du khách có trải nghiệm du lịch trọn vẹn, Traveloka giới thiệu thêm nhiều tính năng khác như: hoàn tiền 100%, thay đổi lịch trình, thanh toán linh hoạt... Xem thêm thông tin chi tiết về chương trình Epic Sale trên ứng dụng, website và các tài khoản mạng xã hội của Traveloka. Á Hiên",
-  "summary": "781.925 đồng vé Vietravel, 2.819 triệu Thâm Quyến; 2.667 và 2.682 triệu Hàn Quốc-Nhật Bản. Khách sạn từ 794.000-1.858 triệu. Áp dụng 'mua 1 tặng 1' Sun World, The Amazing Bay, Sea Life Bangkok Ocean World. Hoàn tiền 100%, thay đổi lịch trình, thanh toán linh hoạt trên Traveloka. Epic Sale của Ninh Dương Lan Ngọc mong muốn lan tỏa tinh thần du lịch thông minh và áp dụng ưu đãi đến 50% cho các sản phẩm toàn thế giới nhằm tri ân khách hàng và khích lệ khám phá thế giới qua những chuyến đi tiện nghi với chi phí tiết kiệm.",
-  "faithfulness_score": 0.8,
-  "faithfulness_reason": "Bản tóm tắt không bịa đặt thông tin nhưng có thể thiếu một số chi tiết quan trọng như việc hợp tác giữa Traveloka và Ninh Dương Lan Ngọc, cũng như một số thông tin về các dịch vụ và ưu đãi cụ thể.",
-  "relevance_score": 0.7,
-  "relevance_reason": "Bản tóm tắt bao gồm một số ý chính như giá vé máy bay, khách sạn và các ưu đãi, nhưng có thể bỏ sót một số thông điệp cốt lõi như sứ mệnh của Traveloka và tầm ảnh hưởng của Ninh Dương Lan Ngọc.",
-  "coherence_conciseness_score": 0.9,
-  "coherence_conciseness_reason": "Bản tóm tắt trôi chảy, logic và dễ đọc, tuy nhiên có thể có một số từ ngữ lặp lại hoặc không cần thiết, nhưng tổng thể vẫn rõ ràng và súc tích."
-}</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>